<commit_message>
Deploying to gh-pages from @ open-resource-discovery/specification@5f06cf18bbcabaca3c0ab5eb8b97570fafd01799 🚀
</commit_message>
<xml_diff>
--- a/spec-v1/interfaces/Document.xlsx
+++ b/spec-v1/interfaces/Document.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1432" uniqueCount="206">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1441" uniqueCount="209">
   <si>
     <t>Entity Name</t>
   </si>
@@ -482,6 +482,15 @@
   </si>
   <si>
     <t>Capability Integration Aspect</t>
+  </si>
+  <si>
+    <t>array&lt;CapabilityIntegrationAspectSubset&gt;</t>
+  </si>
+  <si>
+    <t>Capability Integration Aspect Subset</t>
+  </si>
+  <si>
+    <t>skillName</t>
   </si>
   <si>
     <t>Vendor</t>
@@ -1005,7 +1014,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D477"/>
+  <dimension ref="A1:D480"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -5353,13 +5362,13 @@
         <v>127</v>
       </c>
       <c r="B311" t="s">
-        <v>94</v>
+        <v>121</v>
       </c>
       <c r="C311" t="b">
         <v>0</v>
       </c>
       <c r="D311" t="s">
-        <v>130</v>
+        <v>9</v>
       </c>
     </row>
     <row r="312" spans="1:4" x14ac:dyDescent="0.25">
@@ -5367,13 +5376,13 @@
         <v>127</v>
       </c>
       <c r="B312" t="s">
-        <v>19</v>
+        <v>94</v>
       </c>
       <c r="C312" t="b">
         <v>0</v>
       </c>
       <c r="D312" t="s">
-        <v>20</v>
+        <v>130</v>
       </c>
     </row>
     <row r="313" spans="1:4" x14ac:dyDescent="0.25">
@@ -5381,13 +5390,13 @@
         <v>127</v>
       </c>
       <c r="B313" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="C313" t="b">
         <v>0</v>
       </c>
       <c r="D313" t="s">
-        <v>9</v>
+        <v>20</v>
       </c>
     </row>
     <row r="314" spans="1:4" x14ac:dyDescent="0.25">
@@ -5395,13 +5404,13 @@
         <v>127</v>
       </c>
       <c r="B314" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C314" t="b">
         <v>0</v>
       </c>
       <c r="D314" t="s">
-        <v>33</v>
+        <v>9</v>
       </c>
     </row>
     <row r="315" spans="1:4" x14ac:dyDescent="0.25">
@@ -5409,13 +5418,13 @@
         <v>127</v>
       </c>
       <c r="B315" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C315" t="b">
         <v>0</v>
       </c>
       <c r="D315" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="316" spans="1:4" x14ac:dyDescent="0.25">
@@ -5423,27 +5432,27 @@
         <v>127</v>
       </c>
       <c r="B316" t="s">
-        <v>85</v>
+        <v>34</v>
       </c>
       <c r="C316" t="b">
         <v>0</v>
       </c>
       <c r="D316" t="s">
-        <v>51</v>
+        <v>35</v>
       </c>
     </row>
     <row r="317" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A317" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="B317" t="s">
-        <v>97</v>
+        <v>85</v>
       </c>
       <c r="C317" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D317" t="s">
-        <v>6</v>
+        <v>51</v>
       </c>
     </row>
     <row r="318" spans="1:4" x14ac:dyDescent="0.25">
@@ -5451,10 +5460,10 @@
         <v>131</v>
       </c>
       <c r="B318" t="s">
-        <v>115</v>
+        <v>97</v>
       </c>
       <c r="C318" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D318" t="s">
         <v>6</v>
@@ -5465,10 +5474,10 @@
         <v>131</v>
       </c>
       <c r="B319" t="s">
-        <v>98</v>
+        <v>115</v>
       </c>
       <c r="C319" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D319" t="s">
         <v>6</v>
@@ -5479,7 +5488,7 @@
         <v>131</v>
       </c>
       <c r="B320" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C320" t="b">
         <v>1</v>
@@ -5493,13 +5502,13 @@
         <v>131</v>
       </c>
       <c r="B321" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C321" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D321" t="s">
-        <v>101</v>
+        <v>6</v>
       </c>
     </row>
     <row r="322" spans="1:4" x14ac:dyDescent="0.25">
@@ -5507,13 +5516,13 @@
         <v>131</v>
       </c>
       <c r="B322" t="s">
-        <v>38</v>
+        <v>100</v>
       </c>
       <c r="C322" t="b">
         <v>0</v>
       </c>
       <c r="D322" t="s">
-        <v>6</v>
+        <v>101</v>
       </c>
     </row>
     <row r="323" spans="1:4" x14ac:dyDescent="0.25">
@@ -5521,7 +5530,7 @@
         <v>131</v>
       </c>
       <c r="B323" t="s">
-        <v>116</v>
+        <v>38</v>
       </c>
       <c r="C323" t="b">
         <v>0</v>
@@ -5532,13 +5541,13 @@
     </row>
     <row r="324" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A324" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B324" t="s">
-        <v>5</v>
+        <v>116</v>
       </c>
       <c r="C324" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D324" t="s">
         <v>6</v>
@@ -5549,10 +5558,10 @@
         <v>132</v>
       </c>
       <c r="B325" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C325" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D325" t="s">
         <v>6</v>
@@ -5563,13 +5572,13 @@
         <v>132</v>
       </c>
       <c r="B326" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C326" t="b">
         <v>0</v>
       </c>
       <c r="D326" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="327" spans="1:4" x14ac:dyDescent="0.25">
@@ -5577,13 +5586,13 @@
         <v>132</v>
       </c>
       <c r="B327" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C327" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D327" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="328" spans="1:4" x14ac:dyDescent="0.25">
@@ -5591,10 +5600,10 @@
         <v>132</v>
       </c>
       <c r="B328" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C328" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D328" t="s">
         <v>6</v>
@@ -5605,7 +5614,7 @@
         <v>132</v>
       </c>
       <c r="B329" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C329" t="b">
         <v>0</v>
@@ -5619,10 +5628,10 @@
         <v>132</v>
       </c>
       <c r="B330" t="s">
-        <v>45</v>
+        <v>12</v>
       </c>
       <c r="C330" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D330" t="s">
         <v>6</v>
@@ -5633,13 +5642,13 @@
         <v>132</v>
       </c>
       <c r="B331" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C331" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D331" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="332" spans="1:4" x14ac:dyDescent="0.25">
@@ -5647,13 +5656,13 @@
         <v>132</v>
       </c>
       <c r="B332" t="s">
-        <v>13</v>
+        <v>46</v>
       </c>
       <c r="C332" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D332" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="333" spans="1:4" x14ac:dyDescent="0.25">
@@ -5661,10 +5670,10 @@
         <v>132</v>
       </c>
       <c r="B333" t="s">
-        <v>37</v>
+        <v>13</v>
       </c>
       <c r="C333" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D333" t="s">
         <v>6</v>
@@ -5675,10 +5684,10 @@
         <v>132</v>
       </c>
       <c r="B334" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C334" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D334" t="s">
         <v>6</v>
@@ -5689,7 +5698,7 @@
         <v>132</v>
       </c>
       <c r="B335" t="s">
-        <v>52</v>
+        <v>38</v>
       </c>
       <c r="C335" t="b">
         <v>1</v>
@@ -5703,10 +5712,10 @@
         <v>132</v>
       </c>
       <c r="B336" t="s">
-        <v>60</v>
+        <v>52</v>
       </c>
       <c r="C336" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D336" t="s">
         <v>6</v>
@@ -5717,13 +5726,13 @@
         <v>132</v>
       </c>
       <c r="B337" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C337" t="b">
         <v>0</v>
       </c>
       <c r="D337" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="338" spans="1:4" x14ac:dyDescent="0.25">
@@ -5731,13 +5740,13 @@
         <v>132</v>
       </c>
       <c r="B338" t="s">
-        <v>133</v>
+        <v>61</v>
       </c>
       <c r="C338" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D338" t="s">
-        <v>51</v>
+        <v>9</v>
       </c>
     </row>
     <row r="339" spans="1:4" x14ac:dyDescent="0.25">
@@ -5745,13 +5754,13 @@
         <v>132</v>
       </c>
       <c r="B339" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C339" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D339" t="s">
-        <v>135</v>
+        <v>51</v>
       </c>
     </row>
     <row r="340" spans="1:4" x14ac:dyDescent="0.25">
@@ -5759,13 +5768,13 @@
         <v>132</v>
       </c>
       <c r="B340" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="C340" t="b">
         <v>0</v>
       </c>
       <c r="D340" t="s">
-        <v>9</v>
+        <v>135</v>
       </c>
     </row>
     <row r="341" spans="1:4" x14ac:dyDescent="0.25">
@@ -5773,13 +5782,13 @@
         <v>132</v>
       </c>
       <c r="B341" t="s">
-        <v>19</v>
+        <v>136</v>
       </c>
       <c r="C341" t="b">
         <v>0</v>
       </c>
       <c r="D341" t="s">
-        <v>20</v>
+        <v>9</v>
       </c>
     </row>
     <row r="342" spans="1:4" x14ac:dyDescent="0.25">
@@ -5787,13 +5796,13 @@
         <v>132</v>
       </c>
       <c r="B342" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="C342" t="b">
         <v>0</v>
       </c>
       <c r="D342" t="s">
-        <v>9</v>
+        <v>20</v>
       </c>
     </row>
     <row r="343" spans="1:4" x14ac:dyDescent="0.25">
@@ -5801,13 +5810,13 @@
         <v>132</v>
       </c>
       <c r="B343" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C343" t="b">
         <v>0</v>
       </c>
       <c r="D343" t="s">
-        <v>33</v>
+        <v>9</v>
       </c>
     </row>
     <row r="344" spans="1:4" x14ac:dyDescent="0.25">
@@ -5815,27 +5824,27 @@
         <v>132</v>
       </c>
       <c r="B344" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C344" t="b">
         <v>0</v>
       </c>
       <c r="D344" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="345" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A345" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="B345" t="s">
-        <v>10</v>
+        <v>34</v>
       </c>
       <c r="C345" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D345" t="s">
-        <v>6</v>
+        <v>35</v>
       </c>
     </row>
     <row r="346" spans="1:4" x14ac:dyDescent="0.25">
@@ -5843,10 +5852,10 @@
         <v>137</v>
       </c>
       <c r="B346" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C346" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D346" t="s">
         <v>6</v>
@@ -5857,13 +5866,13 @@
         <v>137</v>
       </c>
       <c r="B347" t="s">
-        <v>133</v>
+        <v>12</v>
       </c>
       <c r="C347" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D347" t="s">
-        <v>51</v>
+        <v>6</v>
       </c>
     </row>
     <row r="348" spans="1:4" x14ac:dyDescent="0.25">
@@ -5871,10 +5880,10 @@
         <v>137</v>
       </c>
       <c r="B348" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="C348" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D348" t="s">
         <v>51</v>
@@ -5885,13 +5894,13 @@
         <v>137</v>
       </c>
       <c r="B349" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C349" t="b">
         <v>0</v>
       </c>
       <c r="D349" t="s">
-        <v>140</v>
+        <v>51</v>
       </c>
     </row>
     <row r="350" spans="1:4" x14ac:dyDescent="0.25">
@@ -5899,13 +5908,13 @@
         <v>137</v>
       </c>
       <c r="B350" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="C350" t="b">
         <v>0</v>
       </c>
       <c r="D350" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
     </row>
     <row r="351" spans="1:4" x14ac:dyDescent="0.25">
@@ -5913,13 +5922,13 @@
         <v>137</v>
       </c>
       <c r="B351" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="C351" t="b">
         <v>0</v>
       </c>
       <c r="D351" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
     </row>
     <row r="352" spans="1:4" x14ac:dyDescent="0.25">
@@ -5927,27 +5936,27 @@
         <v>137</v>
       </c>
       <c r="B352" t="s">
-        <v>32</v>
+        <v>143</v>
       </c>
       <c r="C352" t="b">
         <v>0</v>
       </c>
       <c r="D352" t="s">
-        <v>33</v>
+        <v>144</v>
       </c>
     </row>
     <row r="353" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A353" t="s">
-        <v>145</v>
+        <v>137</v>
       </c>
       <c r="B353" t="s">
-        <v>5</v>
+        <v>32</v>
       </c>
       <c r="C353" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D353" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
     </row>
     <row r="354" spans="1:4" x14ac:dyDescent="0.25">
@@ -5955,10 +5964,10 @@
         <v>145</v>
       </c>
       <c r="B354" t="s">
-        <v>146</v>
+        <v>5</v>
       </c>
       <c r="C354" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D354" t="s">
         <v>6</v>
@@ -5969,13 +5978,13 @@
         <v>145</v>
       </c>
       <c r="B355" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C355" t="b">
         <v>0</v>
       </c>
       <c r="D355" t="s">
-        <v>148</v>
+        <v>6</v>
       </c>
     </row>
     <row r="356" spans="1:4" x14ac:dyDescent="0.25">
@@ -5983,27 +5992,27 @@
         <v>145</v>
       </c>
       <c r="B356" t="s">
-        <v>32</v>
+        <v>147</v>
       </c>
       <c r="C356" t="b">
         <v>0</v>
       </c>
       <c r="D356" t="s">
-        <v>33</v>
+        <v>148</v>
       </c>
     </row>
     <row r="357" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A357" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="B357" t="s">
-        <v>5</v>
+        <v>32</v>
       </c>
       <c r="C357" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D357" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
     </row>
     <row r="358" spans="1:4" x14ac:dyDescent="0.25">
@@ -6011,10 +6020,10 @@
         <v>149</v>
       </c>
       <c r="B358" t="s">
-        <v>146</v>
+        <v>5</v>
       </c>
       <c r="C358" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D358" t="s">
         <v>6</v>
@@ -6025,13 +6034,13 @@
         <v>149</v>
       </c>
       <c r="B359" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C359" t="b">
         <v>0</v>
       </c>
       <c r="D359" t="s">
-        <v>150</v>
+        <v>6</v>
       </c>
     </row>
     <row r="360" spans="1:4" x14ac:dyDescent="0.25">
@@ -6039,13 +6048,13 @@
         <v>149</v>
       </c>
       <c r="B360" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="C360" t="b">
         <v>0</v>
       </c>
       <c r="D360" t="s">
-        <v>9</v>
+        <v>150</v>
       </c>
     </row>
     <row r="361" spans="1:4" x14ac:dyDescent="0.25">
@@ -6053,35 +6062,35 @@
         <v>149</v>
       </c>
       <c r="B361" t="s">
-        <v>32</v>
+        <v>151</v>
       </c>
       <c r="C361" t="b">
         <v>0</v>
       </c>
       <c r="D361" t="s">
-        <v>33</v>
+        <v>9</v>
       </c>
     </row>
     <row r="362" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A362" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="B362" t="s">
-        <v>153</v>
+        <v>32</v>
       </c>
       <c r="C362" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D362" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
     </row>
     <row r="363" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A363" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="B363" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="C363" t="b">
         <v>1</v>
@@ -6092,10 +6101,10 @@
     </row>
     <row r="364" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A364" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="B364" t="s">
-        <v>5</v>
+        <v>155</v>
       </c>
       <c r="C364" t="b">
         <v>1</v>
@@ -6109,10 +6118,10 @@
         <v>156</v>
       </c>
       <c r="B365" t="s">
-        <v>146</v>
+        <v>5</v>
       </c>
       <c r="C365" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D365" t="s">
         <v>6</v>
@@ -6123,150 +6132,150 @@
         <v>156</v>
       </c>
       <c r="B366" t="s">
-        <v>32</v>
+        <v>146</v>
       </c>
       <c r="C366" t="b">
         <v>0</v>
       </c>
       <c r="D366" t="s">
-        <v>33</v>
+        <v>6</v>
       </c>
     </row>
     <row r="367" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A367" t="s">
+        <v>156</v>
+      </c>
+      <c r="B367" t="s">
+        <v>147</v>
+      </c>
+      <c r="C367" t="b">
+        <v>0</v>
+      </c>
+      <c r="D367" t="s">
         <v>157</v>
-      </c>
-      <c r="B367" t="s">
-        <v>5</v>
-      </c>
-      <c r="C367" t="b">
-        <v>1</v>
-      </c>
-      <c r="D367" t="s">
-        <v>6</v>
       </c>
     </row>
     <row r="368" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A368" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B368" t="s">
-        <v>10</v>
+        <v>32</v>
       </c>
       <c r="C368" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D368" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
     </row>
     <row r="369" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A369" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B369" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="C369" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D369" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="370" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A370" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="B370" t="s">
-        <v>31</v>
+        <v>5</v>
       </c>
       <c r="C370" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D370" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="371" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A371" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="B371" t="s">
-        <v>32</v>
+        <v>10</v>
       </c>
       <c r="C371" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D371" t="s">
-        <v>33</v>
+        <v>6</v>
       </c>
     </row>
     <row r="372" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A372" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="B372" t="s">
-        <v>34</v>
+        <v>161</v>
       </c>
       <c r="C372" t="b">
         <v>0</v>
       </c>
       <c r="D372" t="s">
-        <v>35</v>
+        <v>9</v>
       </c>
     </row>
     <row r="373" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A373" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="B373" t="s">
-        <v>13</v>
+        <v>31</v>
       </c>
       <c r="C373" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D373" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="374" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A374" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="B374" t="s">
-        <v>52</v>
+        <v>32</v>
       </c>
       <c r="C374" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D374" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
     </row>
     <row r="375" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A375" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="B375" t="s">
-        <v>160</v>
+        <v>34</v>
       </c>
       <c r="C375" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D375" t="s">
-        <v>6</v>
+        <v>35</v>
       </c>
     </row>
     <row r="376" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A376" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="B376" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C376" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D376" t="s">
         <v>6</v>
@@ -6274,13 +6283,13 @@
     </row>
     <row r="377" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A377" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="B377" t="s">
-        <v>99</v>
+        <v>52</v>
       </c>
       <c r="C377" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D377" t="s">
         <v>6</v>
@@ -6288,10 +6297,10 @@
     </row>
     <row r="378" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A378" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B378" t="s">
-        <v>10</v>
+        <v>163</v>
       </c>
       <c r="C378" t="b">
         <v>1</v>
@@ -6302,13 +6311,13 @@
     </row>
     <row r="379" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A379" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B379" t="s">
-        <v>99</v>
+        <v>12</v>
       </c>
       <c r="C379" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D379" t="s">
         <v>6</v>
@@ -6316,10 +6325,10 @@
     </row>
     <row r="380" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A380" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B380" t="s">
-        <v>12</v>
+        <v>99</v>
       </c>
       <c r="C380" t="b">
         <v>0</v>
@@ -6330,7 +6339,7 @@
     </row>
     <row r="381" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A381" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B381" t="s">
         <v>10</v>
@@ -6344,7 +6353,7 @@
     </row>
     <row r="382" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A382" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B382" t="s">
         <v>99</v>
@@ -6358,7 +6367,7 @@
     </row>
     <row r="383" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A383" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B383" t="s">
         <v>12</v>
@@ -6372,10 +6381,10 @@
     </row>
     <row r="384" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A384" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="B384" t="s">
-        <v>98</v>
+        <v>10</v>
       </c>
       <c r="C384" t="b">
         <v>1</v>
@@ -6386,10 +6395,10 @@
     </row>
     <row r="385" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A385" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="B385" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="C385" t="b">
         <v>1</v>
@@ -6400,10 +6409,10 @@
     </row>
     <row r="386" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A386" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="B386" t="s">
-        <v>115</v>
+        <v>12</v>
       </c>
       <c r="C386" t="b">
         <v>0</v>
@@ -6414,10 +6423,10 @@
     </row>
     <row r="387" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A387" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="B387" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C387" t="b">
         <v>1</v>
@@ -6428,7 +6437,7 @@
     </row>
     <row r="388" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A388" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B388" t="s">
         <v>97</v>
@@ -6442,7 +6451,7 @@
     </row>
     <row r="389" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A389" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B389" t="s">
         <v>115</v>
@@ -6456,7 +6465,7 @@
     </row>
     <row r="390" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A390" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B390" t="s">
         <v>99</v>
@@ -6470,7 +6479,7 @@
     </row>
     <row r="391" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A391" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="B391" t="s">
         <v>97</v>
@@ -6484,7 +6493,7 @@
     </row>
     <row r="392" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A392" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="B392" t="s">
         <v>115</v>
@@ -6498,7 +6507,7 @@
     </row>
     <row r="393" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A393" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="B393" t="s">
         <v>99</v>
@@ -6512,13 +6521,13 @@
     </row>
     <row r="394" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A394" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B394" t="s">
-        <v>167</v>
+        <v>97</v>
       </c>
       <c r="C394" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D394" t="s">
         <v>6</v>
@@ -6526,10 +6535,10 @@
     </row>
     <row r="395" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A395" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B395" t="s">
-        <v>7</v>
+        <v>115</v>
       </c>
       <c r="C395" t="b">
         <v>0</v>
@@ -6540,52 +6549,52 @@
     </row>
     <row r="396" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A396" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B396" t="s">
-        <v>8</v>
+        <v>99</v>
       </c>
       <c r="C396" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D396" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="397" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A397" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="B397" t="s">
-        <v>32</v>
+        <v>170</v>
       </c>
       <c r="C397" t="b">
         <v>0</v>
       </c>
       <c r="D397" t="s">
-        <v>33</v>
+        <v>6</v>
       </c>
     </row>
     <row r="398" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A398" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="B398" t="s">
-        <v>34</v>
+        <v>7</v>
       </c>
       <c r="C398" t="b">
         <v>0</v>
       </c>
       <c r="D398" t="s">
-        <v>35</v>
+        <v>6</v>
       </c>
     </row>
     <row r="399" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A399" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="B399" t="s">
-        <v>31</v>
+        <v>8</v>
       </c>
       <c r="C399" t="b">
         <v>0</v>
@@ -6596,66 +6605,66 @@
     </row>
     <row r="400" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A400" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B400" t="s">
-        <v>169</v>
+        <v>32</v>
       </c>
       <c r="C400" t="b">
         <v>0</v>
       </c>
       <c r="D400" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
     </row>
     <row r="401" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A401" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B401" t="s">
-        <v>8</v>
+        <v>34</v>
       </c>
       <c r="C401" t="b">
         <v>0</v>
       </c>
       <c r="D401" t="s">
-        <v>9</v>
+        <v>35</v>
       </c>
     </row>
     <row r="402" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A402" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B402" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C402" t="b">
         <v>0</v>
       </c>
       <c r="D402" t="s">
-        <v>33</v>
+        <v>9</v>
       </c>
     </row>
     <row r="403" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A403" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="B403" t="s">
-        <v>34</v>
+        <v>172</v>
       </c>
       <c r="C403" t="b">
         <v>0</v>
       </c>
       <c r="D403" t="s">
-        <v>35</v>
+        <v>6</v>
       </c>
     </row>
     <row r="404" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A404" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="B404" t="s">
-        <v>31</v>
+        <v>8</v>
       </c>
       <c r="C404" t="b">
         <v>0</v>
@@ -6666,38 +6675,38 @@
     </row>
     <row r="405" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A405" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="B405" t="s">
-        <v>13</v>
+        <v>32</v>
       </c>
       <c r="C405" t="b">
         <v>0</v>
       </c>
       <c r="D405" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
     </row>
     <row r="406" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A406" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="B406" t="s">
-        <v>10</v>
+        <v>34</v>
       </c>
       <c r="C406" t="b">
         <v>0</v>
       </c>
       <c r="D406" t="s">
-        <v>6</v>
+        <v>35</v>
       </c>
     </row>
     <row r="407" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A407" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="B407" t="s">
-        <v>8</v>
+        <v>31</v>
       </c>
       <c r="C407" t="b">
         <v>0</v>
@@ -6708,38 +6717,38 @@
     </row>
     <row r="408" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A408" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="B408" t="s">
-        <v>32</v>
+        <v>13</v>
       </c>
       <c r="C408" t="b">
         <v>0</v>
       </c>
       <c r="D408" t="s">
-        <v>33</v>
+        <v>6</v>
       </c>
     </row>
     <row r="409" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A409" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="B409" t="s">
-        <v>34</v>
+        <v>10</v>
       </c>
       <c r="C409" t="b">
         <v>0</v>
       </c>
       <c r="D409" t="s">
-        <v>35</v>
+        <v>6</v>
       </c>
     </row>
     <row r="410" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A410" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="B410" t="s">
-        <v>31</v>
+        <v>8</v>
       </c>
       <c r="C410" t="b">
         <v>0</v>
@@ -6750,49 +6759,49 @@
     </row>
     <row r="411" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A411" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="B411" t="s">
-        <v>97</v>
+        <v>32</v>
       </c>
       <c r="C411" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D411" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
     </row>
     <row r="412" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A412" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="B412" t="s">
-        <v>115</v>
+        <v>34</v>
       </c>
       <c r="C412" t="b">
         <v>0</v>
       </c>
       <c r="D412" t="s">
-        <v>6</v>
+        <v>35</v>
       </c>
     </row>
     <row r="413" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A413" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="B413" t="s">
-        <v>172</v>
+        <v>31</v>
       </c>
       <c r="C413" t="b">
         <v>0</v>
       </c>
       <c r="D413" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="414" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A414" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="B414" t="s">
         <v>97</v>
@@ -6806,7 +6815,7 @@
     </row>
     <row r="415" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A415" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="B415" t="s">
         <v>115</v>
@@ -6820,10 +6829,10 @@
     </row>
     <row r="416" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A416" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="B416" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="C416" t="b">
         <v>0</v>
@@ -6834,13 +6843,13 @@
     </row>
     <row r="417" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A417" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="B417" t="s">
-        <v>174</v>
+        <v>97</v>
       </c>
       <c r="C417" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D417" t="s">
         <v>6</v>
@@ -6848,13 +6857,13 @@
     </row>
     <row r="418" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A418" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B418" t="s">
-        <v>176</v>
+        <v>115</v>
       </c>
       <c r="C418" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D418" t="s">
         <v>6</v>
@@ -6862,13 +6871,13 @@
     </row>
     <row r="419" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A419" t="s">
+        <v>176</v>
+      </c>
+      <c r="B419" t="s">
         <v>175</v>
       </c>
-      <c r="B419" t="s">
-        <v>10</v>
-      </c>
       <c r="C419" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D419" t="s">
         <v>6</v>
@@ -6876,10 +6885,10 @@
     </row>
     <row r="420" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A420" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B420" t="s">
-        <v>12</v>
+        <v>177</v>
       </c>
       <c r="C420" t="b">
         <v>0</v>
@@ -6890,58 +6899,58 @@
     </row>
     <row r="421" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A421" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="B421" t="s">
-        <v>32</v>
+        <v>179</v>
       </c>
       <c r="C421" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D421" t="s">
-        <v>33</v>
+        <v>6</v>
       </c>
     </row>
     <row r="422" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A422" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="B422" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C422" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D422" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="423" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A423" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="B423" t="s">
-        <v>177</v>
+        <v>12</v>
       </c>
       <c r="C423" t="b">
         <v>0</v>
       </c>
       <c r="D423" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="424" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A424" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="B424" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="C424" t="b">
         <v>0</v>
       </c>
       <c r="D424" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
     </row>
     <row r="425" spans="1:4" x14ac:dyDescent="0.25">
@@ -6949,13 +6958,13 @@
         <v>178</v>
       </c>
       <c r="B425" t="s">
-        <v>179</v>
+        <v>8</v>
       </c>
       <c r="C425" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D425" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="426" spans="1:4" x14ac:dyDescent="0.25">
@@ -6963,13 +6972,13 @@
         <v>178</v>
       </c>
       <c r="B426" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="C426" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D426" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="427" spans="1:4" x14ac:dyDescent="0.25">
@@ -6977,10 +6986,10 @@
         <v>178</v>
       </c>
       <c r="B427" t="s">
-        <v>10</v>
+        <v>38</v>
       </c>
       <c r="C427" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D427" t="s">
         <v>6</v>
@@ -6988,13 +6997,13 @@
     </row>
     <row r="428" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A428" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="B428" t="s">
-        <v>12</v>
+        <v>182</v>
       </c>
       <c r="C428" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D428" t="s">
         <v>6</v>
@@ -7002,86 +7011,86 @@
     </row>
     <row r="429" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A429" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="B429" t="s">
-        <v>32</v>
+        <v>179</v>
       </c>
       <c r="C429" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D429" t="s">
-        <v>33</v>
+        <v>6</v>
       </c>
     </row>
     <row r="430" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A430" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="B430" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C430" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D430" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="431" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A431" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="B431" t="s">
-        <v>46</v>
+        <v>12</v>
       </c>
       <c r="C431" t="b">
         <v>0</v>
       </c>
       <c r="D431" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="432" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A432" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="B432" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="C432" t="b">
         <v>0</v>
       </c>
       <c r="D432" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
     </row>
     <row r="433" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A433" t="s">
-        <v>84</v>
+        <v>181</v>
       </c>
       <c r="B433" t="s">
-        <v>180</v>
+        <v>8</v>
       </c>
       <c r="C433" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D433" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="434" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A434" t="s">
-        <v>84</v>
+        <v>181</v>
       </c>
       <c r="B434" t="s">
-        <v>12</v>
+        <v>46</v>
       </c>
       <c r="C434" t="b">
         <v>0</v>
       </c>
       <c r="D434" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="435" spans="1:4" x14ac:dyDescent="0.25">
@@ -7089,38 +7098,38 @@
         <v>181</v>
       </c>
       <c r="B435" t="s">
-        <v>182</v>
+        <v>38</v>
       </c>
       <c r="C435" t="b">
         <v>0</v>
       </c>
       <c r="D435" t="s">
-        <v>183</v>
+        <v>6</v>
       </c>
     </row>
     <row r="436" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A436" t="s">
-        <v>181</v>
+        <v>84</v>
       </c>
       <c r="B436" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C436" t="b">
         <v>1</v>
       </c>
       <c r="D436" t="s">
-        <v>185</v>
+        <v>6</v>
       </c>
     </row>
     <row r="437" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A437" t="s">
-        <v>186</v>
+        <v>84</v>
       </c>
       <c r="B437" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="C437" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D437" t="s">
         <v>6</v>
@@ -7128,38 +7137,38 @@
     </row>
     <row r="438" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A438" t="s">
+        <v>184</v>
+      </c>
+      <c r="B438" t="s">
+        <v>185</v>
+      </c>
+      <c r="C438" t="b">
+        <v>0</v>
+      </c>
+      <c r="D438" t="s">
         <v>186</v>
-      </c>
-      <c r="B438" t="s">
-        <v>187</v>
-      </c>
-      <c r="C438" t="b">
-        <v>1</v>
-      </c>
-      <c r="D438" t="s">
-        <v>6</v>
       </c>
     </row>
     <row r="439" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A439" t="s">
+        <v>184</v>
+      </c>
+      <c r="B439" t="s">
+        <v>187</v>
+      </c>
+      <c r="C439" t="b">
+        <v>1</v>
+      </c>
+      <c r="D439" t="s">
         <v>188</v>
-      </c>
-      <c r="B439" t="s">
-        <v>5</v>
-      </c>
-      <c r="C439" t="b">
-        <v>1</v>
-      </c>
-      <c r="D439" t="s">
-        <v>6</v>
       </c>
     </row>
     <row r="440" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A440" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="B440" t="s">
-        <v>187</v>
+        <v>5</v>
       </c>
       <c r="C440" t="b">
         <v>1</v>
@@ -7173,7 +7182,7 @@
         <v>189</v>
       </c>
       <c r="B441" t="s">
-        <v>97</v>
+        <v>190</v>
       </c>
       <c r="C441" t="b">
         <v>1</v>
@@ -7184,10 +7193,10 @@
     </row>
     <row r="442" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A442" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="B442" t="s">
-        <v>190</v>
+        <v>5</v>
       </c>
       <c r="C442" t="b">
         <v>1</v>
@@ -7201,7 +7210,7 @@
         <v>191</v>
       </c>
       <c r="B443" t="s">
-        <v>97</v>
+        <v>190</v>
       </c>
       <c r="C443" t="b">
         <v>1</v>
@@ -7212,10 +7221,10 @@
     </row>
     <row r="444" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A444" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="B444" t="s">
-        <v>192</v>
+        <v>97</v>
       </c>
       <c r="C444" t="b">
         <v>1</v>
@@ -7226,10 +7235,10 @@
     </row>
     <row r="445" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A445" t="s">
+        <v>192</v>
+      </c>
+      <c r="B445" t="s">
         <v>193</v>
-      </c>
-      <c r="B445" t="s">
-        <v>5</v>
       </c>
       <c r="C445" t="b">
         <v>1</v>
@@ -7243,7 +7252,7 @@
         <v>194</v>
       </c>
       <c r="B446" t="s">
-        <v>5</v>
+        <v>97</v>
       </c>
       <c r="C446" t="b">
         <v>1</v>
@@ -7254,10 +7263,10 @@
     </row>
     <row r="447" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A447" t="s">
+        <v>194</v>
+      </c>
+      <c r="B447" t="s">
         <v>195</v>
-      </c>
-      <c r="B447" t="s">
-        <v>196</v>
       </c>
       <c r="C447" t="b">
         <v>1</v>
@@ -7268,7 +7277,7 @@
     </row>
     <row r="448" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A448" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B448" t="s">
         <v>5</v>
@@ -7285,10 +7294,10 @@
         <v>197</v>
       </c>
       <c r="B449" t="s">
-        <v>198</v>
+        <v>5</v>
       </c>
       <c r="C449" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D449" t="s">
         <v>6</v>
@@ -7296,10 +7305,10 @@
     </row>
     <row r="450" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A450" t="s">
+        <v>198</v>
+      </c>
+      <c r="B450" t="s">
         <v>199</v>
-      </c>
-      <c r="B450" t="s">
-        <v>5</v>
       </c>
       <c r="C450" t="b">
         <v>1</v>
@@ -7310,13 +7319,13 @@
     </row>
     <row r="451" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A451" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="B451" t="s">
-        <v>198</v>
+        <v>5</v>
       </c>
       <c r="C451" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D451" t="s">
         <v>6</v>
@@ -7327,10 +7336,10 @@
         <v>200</v>
       </c>
       <c r="B452" t="s">
-        <v>5</v>
+        <v>201</v>
       </c>
       <c r="C452" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D452" t="s">
         <v>6</v>
@@ -7338,13 +7347,13 @@
     </row>
     <row r="453" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A453" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="B453" t="s">
-        <v>198</v>
+        <v>5</v>
       </c>
       <c r="C453" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D453" t="s">
         <v>6</v>
@@ -7352,13 +7361,13 @@
     </row>
     <row r="454" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A454" t="s">
+        <v>202</v>
+      </c>
+      <c r="B454" t="s">
         <v>201</v>
       </c>
-      <c r="B454" t="s">
-        <v>5</v>
-      </c>
       <c r="C454" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D454" t="s">
         <v>6</v>
@@ -7366,13 +7375,13 @@
     </row>
     <row r="455" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A455" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="B455" t="s">
-        <v>198</v>
+        <v>5</v>
       </c>
       <c r="C455" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D455" t="s">
         <v>6</v>
@@ -7380,13 +7389,13 @@
     </row>
     <row r="456" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A456" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="B456" t="s">
-        <v>5</v>
+        <v>201</v>
       </c>
       <c r="C456" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D456" t="s">
         <v>6</v>
@@ -7394,13 +7403,13 @@
     </row>
     <row r="457" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A457" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="B457" t="s">
         <v>5</v>
       </c>
       <c r="C457" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D457" t="s">
         <v>6</v>
@@ -7408,10 +7417,10 @@
     </row>
     <row r="458" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A458" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="B458" t="s">
-        <v>179</v>
+        <v>201</v>
       </c>
       <c r="C458" t="b">
         <v>0</v>
@@ -7422,13 +7431,13 @@
     </row>
     <row r="459" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A459" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="B459" t="s">
-        <v>176</v>
+        <v>5</v>
       </c>
       <c r="C459" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D459" t="s">
         <v>6</v>
@@ -7436,13 +7445,13 @@
     </row>
     <row r="460" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A460" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="B460" t="s">
-        <v>204</v>
+        <v>5</v>
       </c>
       <c r="C460" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D460" t="s">
         <v>6</v>
@@ -7450,10 +7459,10 @@
     </row>
     <row r="461" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A461" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="B461" t="s">
-        <v>12</v>
+        <v>182</v>
       </c>
       <c r="C461" t="b">
         <v>0</v>
@@ -7464,13 +7473,13 @@
     </row>
     <row r="462" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A462" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B462" t="s">
-        <v>5</v>
+        <v>179</v>
       </c>
       <c r="C462" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D462" t="s">
         <v>6</v>
@@ -7478,13 +7487,13 @@
     </row>
     <row r="463" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A463" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B463" t="s">
-        <v>7</v>
+        <v>207</v>
       </c>
       <c r="C463" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D463" t="s">
         <v>6</v>
@@ -7492,24 +7501,24 @@
     </row>
     <row r="464" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A464" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B464" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="C464" t="b">
         <v>0</v>
       </c>
       <c r="D464" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="465" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A465" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="B465" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="C465" t="b">
         <v>1</v>
@@ -7520,10 +7529,10 @@
     </row>
     <row r="466" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A466" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="B466" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="C466" t="b">
         <v>0</v>
@@ -7534,24 +7543,24 @@
     </row>
     <row r="467" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A467" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="B467" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="C467" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D467" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="468" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A468" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="B468" t="s">
-        <v>45</v>
+        <v>10</v>
       </c>
       <c r="C468" t="b">
         <v>1</v>
@@ -7562,24 +7571,24 @@
     </row>
     <row r="469" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A469" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="B469" t="s">
-        <v>46</v>
+        <v>11</v>
       </c>
       <c r="C469" t="b">
         <v>0</v>
       </c>
       <c r="D469" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="470" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A470" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="B470" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C470" t="b">
         <v>1</v>
@@ -7590,13 +7599,13 @@
     </row>
     <row r="471" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A471" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="B471" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="C471" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D471" t="s">
         <v>6</v>
@@ -7604,24 +7613,24 @@
     </row>
     <row r="472" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A472" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="B472" t="s">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="C472" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D472" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="473" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A473" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="B473" t="s">
-        <v>52</v>
+        <v>13</v>
       </c>
       <c r="C473" t="b">
         <v>1</v>
@@ -7632,57 +7641,99 @@
     </row>
     <row r="474" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A474" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="B474" t="s">
-        <v>19</v>
+        <v>37</v>
       </c>
       <c r="C474" t="b">
         <v>0</v>
       </c>
       <c r="D474" t="s">
-        <v>20</v>
+        <v>6</v>
       </c>
     </row>
     <row r="475" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A475" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="B475" t="s">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="C475" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D475" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="476" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A476" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="B476" t="s">
-        <v>32</v>
+        <v>52</v>
       </c>
       <c r="C476" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D476" t="s">
-        <v>33</v>
+        <v>6</v>
       </c>
     </row>
     <row r="477" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A477" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="B477" t="s">
+        <v>19</v>
+      </c>
+      <c r="C477" t="b">
+        <v>0</v>
+      </c>
+      <c r="D477" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="478" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A478" t="s">
+        <v>208</v>
+      </c>
+      <c r="B478" t="s">
+        <v>31</v>
+      </c>
+      <c r="C478" t="b">
+        <v>0</v>
+      </c>
+      <c r="D478" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="479" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A479" t="s">
+        <v>208</v>
+      </c>
+      <c r="B479" t="s">
+        <v>32</v>
+      </c>
+      <c r="C479" t="b">
+        <v>0</v>
+      </c>
+      <c r="D479" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="480" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A480" t="s">
+        <v>208</v>
+      </c>
+      <c r="B480" t="s">
         <v>34</v>
       </c>
-      <c r="C477" t="b">
-        <v>0</v>
-      </c>
-      <c r="D477" t="s">
+      <c r="C480" t="b">
+        <v>0</v>
+      </c>
+      <c r="D480" t="s">
         <v>35</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Deploying to gh-pages from @ open-resource-discovery/specification@76ac4d200a9b71447a88120094f05c4dc80d4ff7 🚀
</commit_message>
<xml_diff>
--- a/spec-v1/interfaces/Document.xlsx
+++ b/spec-v1/interfaces/Document.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1441" uniqueCount="209">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1471" uniqueCount="209">
   <si>
     <t>Entity Name</t>
   </si>
@@ -1014,7 +1014,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D480"/>
+  <dimension ref="A1:D490"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -5222,13 +5222,13 @@
         <v>127</v>
       </c>
       <c r="B301" t="s">
-        <v>13</v>
+        <v>26</v>
       </c>
       <c r="C301" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D301" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="302" spans="1:4" x14ac:dyDescent="0.25">
@@ -5236,10 +5236,10 @@
         <v>127</v>
       </c>
       <c r="B302" t="s">
-        <v>37</v>
+        <v>13</v>
       </c>
       <c r="C302" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D302" t="s">
         <v>6</v>
@@ -5250,10 +5250,10 @@
         <v>127</v>
       </c>
       <c r="B303" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C303" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D303" t="s">
         <v>6</v>
@@ -5264,7 +5264,7 @@
         <v>127</v>
       </c>
       <c r="B304" t="s">
-        <v>52</v>
+        <v>38</v>
       </c>
       <c r="C304" t="b">
         <v>1</v>
@@ -5278,13 +5278,13 @@
         <v>127</v>
       </c>
       <c r="B305" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C305" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D305" t="s">
-        <v>51</v>
+        <v>6</v>
       </c>
     </row>
     <row r="306" spans="1:4" x14ac:dyDescent="0.25">
@@ -5292,13 +5292,13 @@
         <v>127</v>
       </c>
       <c r="B306" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C306" t="b">
         <v>0</v>
       </c>
       <c r="D306" t="s">
-        <v>6</v>
+        <v>51</v>
       </c>
     </row>
     <row r="307" spans="1:4" x14ac:dyDescent="0.25">
@@ -5306,13 +5306,13 @@
         <v>127</v>
       </c>
       <c r="B307" t="s">
-        <v>92</v>
+        <v>54</v>
       </c>
       <c r="C307" t="b">
         <v>0</v>
       </c>
       <c r="D307" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="308" spans="1:4" x14ac:dyDescent="0.25">
@@ -5320,13 +5320,13 @@
         <v>127</v>
       </c>
       <c r="B308" t="s">
-        <v>55</v>
+        <v>74</v>
       </c>
       <c r="C308" t="b">
         <v>0</v>
       </c>
       <c r="D308" t="s">
-        <v>56</v>
+        <v>6</v>
       </c>
     </row>
     <row r="309" spans="1:4" x14ac:dyDescent="0.25">
@@ -5334,13 +5334,13 @@
         <v>127</v>
       </c>
       <c r="B309" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C309" t="b">
         <v>0</v>
       </c>
       <c r="D309" t="s">
-        <v>58</v>
+        <v>6</v>
       </c>
     </row>
     <row r="310" spans="1:4" x14ac:dyDescent="0.25">
@@ -5348,13 +5348,13 @@
         <v>127</v>
       </c>
       <c r="B310" t="s">
-        <v>128</v>
+        <v>60</v>
       </c>
       <c r="C310" t="b">
         <v>0</v>
       </c>
       <c r="D310" t="s">
-        <v>129</v>
+        <v>6</v>
       </c>
     </row>
     <row r="311" spans="1:4" x14ac:dyDescent="0.25">
@@ -5362,7 +5362,7 @@
         <v>127</v>
       </c>
       <c r="B311" t="s">
-        <v>121</v>
+        <v>61</v>
       </c>
       <c r="C311" t="b">
         <v>0</v>
@@ -5376,13 +5376,13 @@
         <v>127</v>
       </c>
       <c r="B312" t="s">
-        <v>94</v>
+        <v>62</v>
       </c>
       <c r="C312" t="b">
         <v>0</v>
       </c>
       <c r="D312" t="s">
-        <v>130</v>
+        <v>63</v>
       </c>
     </row>
     <row r="313" spans="1:4" x14ac:dyDescent="0.25">
@@ -5390,13 +5390,13 @@
         <v>127</v>
       </c>
       <c r="B313" t="s">
-        <v>19</v>
+        <v>92</v>
       </c>
       <c r="C313" t="b">
         <v>0</v>
       </c>
       <c r="D313" t="s">
-        <v>20</v>
+        <v>9</v>
       </c>
     </row>
     <row r="314" spans="1:4" x14ac:dyDescent="0.25">
@@ -5404,13 +5404,13 @@
         <v>127</v>
       </c>
       <c r="B314" t="s">
-        <v>31</v>
+        <v>55</v>
       </c>
       <c r="C314" t="b">
         <v>0</v>
       </c>
       <c r="D314" t="s">
-        <v>9</v>
+        <v>56</v>
       </c>
     </row>
     <row r="315" spans="1:4" x14ac:dyDescent="0.25">
@@ -5418,13 +5418,13 @@
         <v>127</v>
       </c>
       <c r="B315" t="s">
-        <v>32</v>
+        <v>57</v>
       </c>
       <c r="C315" t="b">
         <v>0</v>
       </c>
       <c r="D315" t="s">
-        <v>33</v>
+        <v>58</v>
       </c>
     </row>
     <row r="316" spans="1:4" x14ac:dyDescent="0.25">
@@ -5432,13 +5432,13 @@
         <v>127</v>
       </c>
       <c r="B316" t="s">
-        <v>34</v>
+        <v>128</v>
       </c>
       <c r="C316" t="b">
         <v>0</v>
       </c>
       <c r="D316" t="s">
-        <v>35</v>
+        <v>129</v>
       </c>
     </row>
     <row r="317" spans="1:4" x14ac:dyDescent="0.25">
@@ -5446,161 +5446,161 @@
         <v>127</v>
       </c>
       <c r="B317" t="s">
-        <v>85</v>
+        <v>121</v>
       </c>
       <c r="C317" t="b">
         <v>0</v>
       </c>
       <c r="D317" t="s">
-        <v>51</v>
+        <v>9</v>
       </c>
     </row>
     <row r="318" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A318" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="B318" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="C318" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D318" t="s">
-        <v>6</v>
+        <v>130</v>
       </c>
     </row>
     <row r="319" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A319" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="B319" t="s">
-        <v>115</v>
+        <v>19</v>
       </c>
       <c r="C319" t="b">
         <v>0</v>
       </c>
       <c r="D319" t="s">
-        <v>6</v>
+        <v>20</v>
       </c>
     </row>
     <row r="320" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A320" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="B320" t="s">
-        <v>98</v>
+        <v>27</v>
       </c>
       <c r="C320" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D320" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="321" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A321" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="B321" t="s">
-        <v>99</v>
+        <v>28</v>
       </c>
       <c r="C321" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D321" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="322" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A322" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="B322" t="s">
-        <v>100</v>
+        <v>29</v>
       </c>
       <c r="C322" t="b">
         <v>0</v>
       </c>
       <c r="D322" t="s">
-        <v>101</v>
+        <v>9</v>
       </c>
     </row>
     <row r="323" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A323" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="B323" t="s">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="C323" t="b">
         <v>0</v>
       </c>
       <c r="D323" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="324" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A324" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="B324" t="s">
-        <v>116</v>
+        <v>32</v>
       </c>
       <c r="C324" t="b">
         <v>0</v>
       </c>
       <c r="D324" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
     </row>
     <row r="325" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A325" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="B325" t="s">
-        <v>5</v>
+        <v>34</v>
       </c>
       <c r="C325" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D325" t="s">
-        <v>6</v>
+        <v>35</v>
       </c>
     </row>
     <row r="326" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A326" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="B326" t="s">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="C326" t="b">
         <v>0</v>
       </c>
       <c r="D326" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="327" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A327" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="B327" t="s">
-        <v>8</v>
+        <v>85</v>
       </c>
       <c r="C327" t="b">
         <v>0</v>
       </c>
       <c r="D327" t="s">
-        <v>9</v>
+        <v>51</v>
       </c>
     </row>
     <row r="328" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A328" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B328" t="s">
-        <v>10</v>
+        <v>97</v>
       </c>
       <c r="C328" t="b">
         <v>1</v>
@@ -5611,10 +5611,10 @@
     </row>
     <row r="329" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A329" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B329" t="s">
-        <v>11</v>
+        <v>115</v>
       </c>
       <c r="C329" t="b">
         <v>0</v>
@@ -5625,13 +5625,13 @@
     </row>
     <row r="330" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A330" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B330" t="s">
-        <v>12</v>
+        <v>98</v>
       </c>
       <c r="C330" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D330" t="s">
         <v>6</v>
@@ -5639,10 +5639,10 @@
     </row>
     <row r="331" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A331" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B331" t="s">
-        <v>45</v>
+        <v>99</v>
       </c>
       <c r="C331" t="b">
         <v>1</v>
@@ -5653,27 +5653,27 @@
     </row>
     <row r="332" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A332" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B332" t="s">
-        <v>46</v>
+        <v>100</v>
       </c>
       <c r="C332" t="b">
         <v>0</v>
       </c>
       <c r="D332" t="s">
-        <v>9</v>
+        <v>101</v>
       </c>
     </row>
     <row r="333" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A333" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B333" t="s">
-        <v>13</v>
+        <v>38</v>
       </c>
       <c r="C333" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D333" t="s">
         <v>6</v>
@@ -5681,10 +5681,10 @@
     </row>
     <row r="334" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A334" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B334" t="s">
-        <v>37</v>
+        <v>116</v>
       </c>
       <c r="C334" t="b">
         <v>0</v>
@@ -5698,7 +5698,7 @@
         <v>132</v>
       </c>
       <c r="B335" t="s">
-        <v>38</v>
+        <v>5</v>
       </c>
       <c r="C335" t="b">
         <v>1</v>
@@ -5712,10 +5712,10 @@
         <v>132</v>
       </c>
       <c r="B336" t="s">
-        <v>52</v>
+        <v>7</v>
       </c>
       <c r="C336" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D336" t="s">
         <v>6</v>
@@ -5726,13 +5726,13 @@
         <v>132</v>
       </c>
       <c r="B337" t="s">
-        <v>60</v>
+        <v>8</v>
       </c>
       <c r="C337" t="b">
         <v>0</v>
       </c>
       <c r="D337" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="338" spans="1:4" x14ac:dyDescent="0.25">
@@ -5740,13 +5740,13 @@
         <v>132</v>
       </c>
       <c r="B338" t="s">
-        <v>61</v>
+        <v>10</v>
       </c>
       <c r="C338" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D338" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="339" spans="1:4" x14ac:dyDescent="0.25">
@@ -5754,13 +5754,13 @@
         <v>132</v>
       </c>
       <c r="B339" t="s">
-        <v>133</v>
+        <v>11</v>
       </c>
       <c r="C339" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D339" t="s">
-        <v>51</v>
+        <v>6</v>
       </c>
     </row>
     <row r="340" spans="1:4" x14ac:dyDescent="0.25">
@@ -5768,13 +5768,13 @@
         <v>132</v>
       </c>
       <c r="B340" t="s">
-        <v>134</v>
+        <v>12</v>
       </c>
       <c r="C340" t="b">
         <v>0</v>
       </c>
       <c r="D340" t="s">
-        <v>135</v>
+        <v>6</v>
       </c>
     </row>
     <row r="341" spans="1:4" x14ac:dyDescent="0.25">
@@ -5782,13 +5782,13 @@
         <v>132</v>
       </c>
       <c r="B341" t="s">
-        <v>136</v>
+        <v>45</v>
       </c>
       <c r="C341" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D341" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="342" spans="1:4" x14ac:dyDescent="0.25">
@@ -5796,13 +5796,13 @@
         <v>132</v>
       </c>
       <c r="B342" t="s">
-        <v>19</v>
+        <v>46</v>
       </c>
       <c r="C342" t="b">
         <v>0</v>
       </c>
       <c r="D342" t="s">
-        <v>20</v>
+        <v>9</v>
       </c>
     </row>
     <row r="343" spans="1:4" x14ac:dyDescent="0.25">
@@ -5810,13 +5810,13 @@
         <v>132</v>
       </c>
       <c r="B343" t="s">
-        <v>31</v>
+        <v>13</v>
       </c>
       <c r="C343" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D343" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="344" spans="1:4" x14ac:dyDescent="0.25">
@@ -5824,13 +5824,13 @@
         <v>132</v>
       </c>
       <c r="B344" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="C344" t="b">
         <v>0</v>
       </c>
       <c r="D344" t="s">
-        <v>33</v>
+        <v>6</v>
       </c>
     </row>
     <row r="345" spans="1:4" x14ac:dyDescent="0.25">
@@ -5838,21 +5838,21 @@
         <v>132</v>
       </c>
       <c r="B345" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="C345" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D345" t="s">
-        <v>35</v>
+        <v>6</v>
       </c>
     </row>
     <row r="346" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A346" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="B346" t="s">
-        <v>10</v>
+        <v>52</v>
       </c>
       <c r="C346" t="b">
         <v>1</v>
@@ -5863,10 +5863,10 @@
     </row>
     <row r="347" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A347" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="B347" t="s">
-        <v>12</v>
+        <v>60</v>
       </c>
       <c r="C347" t="b">
         <v>0</v>
@@ -5877,27 +5877,27 @@
     </row>
     <row r="348" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A348" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="B348" t="s">
-        <v>133</v>
+        <v>61</v>
       </c>
       <c r="C348" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D348" t="s">
-        <v>51</v>
+        <v>9</v>
       </c>
     </row>
     <row r="349" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A349" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="B349" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="C349" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D349" t="s">
         <v>51</v>
@@ -5905,206 +5905,206 @@
     </row>
     <row r="350" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A350" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="B350" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
       <c r="C350" t="b">
         <v>0</v>
       </c>
       <c r="D350" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
     </row>
     <row r="351" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A351" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="B351" t="s">
-        <v>141</v>
+        <v>136</v>
       </c>
       <c r="C351" t="b">
         <v>0</v>
       </c>
       <c r="D351" t="s">
-        <v>142</v>
+        <v>9</v>
       </c>
     </row>
     <row r="352" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A352" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="B352" t="s">
-        <v>143</v>
+        <v>19</v>
       </c>
       <c r="C352" t="b">
         <v>0</v>
       </c>
       <c r="D352" t="s">
-        <v>144</v>
+        <v>20</v>
       </c>
     </row>
     <row r="353" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A353" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="B353" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C353" t="b">
         <v>0</v>
       </c>
       <c r="D353" t="s">
-        <v>33</v>
+        <v>9</v>
       </c>
     </row>
     <row r="354" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A354" t="s">
-        <v>145</v>
+        <v>132</v>
       </c>
       <c r="B354" t="s">
-        <v>5</v>
+        <v>32</v>
       </c>
       <c r="C354" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D354" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
     </row>
     <row r="355" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A355" t="s">
-        <v>145</v>
+        <v>132</v>
       </c>
       <c r="B355" t="s">
-        <v>146</v>
+        <v>34</v>
       </c>
       <c r="C355" t="b">
         <v>0</v>
       </c>
       <c r="D355" t="s">
-        <v>6</v>
+        <v>35</v>
       </c>
     </row>
     <row r="356" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A356" t="s">
-        <v>145</v>
+        <v>137</v>
       </c>
       <c r="B356" t="s">
-        <v>147</v>
+        <v>10</v>
       </c>
       <c r="C356" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D356" t="s">
-        <v>148</v>
+        <v>6</v>
       </c>
     </row>
     <row r="357" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A357" t="s">
-        <v>145</v>
+        <v>137</v>
       </c>
       <c r="B357" t="s">
-        <v>32</v>
+        <v>12</v>
       </c>
       <c r="C357" t="b">
         <v>0</v>
       </c>
       <c r="D357" t="s">
-        <v>33</v>
+        <v>6</v>
       </c>
     </row>
     <row r="358" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A358" t="s">
-        <v>149</v>
+        <v>137</v>
       </c>
       <c r="B358" t="s">
-        <v>5</v>
+        <v>133</v>
       </c>
       <c r="C358" t="b">
         <v>1</v>
       </c>
       <c r="D358" t="s">
-        <v>6</v>
+        <v>51</v>
       </c>
     </row>
     <row r="359" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A359" t="s">
-        <v>149</v>
+        <v>137</v>
       </c>
       <c r="B359" t="s">
-        <v>146</v>
+        <v>138</v>
       </c>
       <c r="C359" t="b">
         <v>0</v>
       </c>
       <c r="D359" t="s">
-        <v>6</v>
+        <v>51</v>
       </c>
     </row>
     <row r="360" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A360" t="s">
-        <v>149</v>
+        <v>137</v>
       </c>
       <c r="B360" t="s">
-        <v>147</v>
+        <v>139</v>
       </c>
       <c r="C360" t="b">
         <v>0</v>
       </c>
       <c r="D360" t="s">
-        <v>150</v>
+        <v>140</v>
       </c>
     </row>
     <row r="361" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A361" t="s">
-        <v>149</v>
+        <v>137</v>
       </c>
       <c r="B361" t="s">
-        <v>151</v>
+        <v>141</v>
       </c>
       <c r="C361" t="b">
         <v>0</v>
       </c>
       <c r="D361" t="s">
-        <v>9</v>
+        <v>142</v>
       </c>
     </row>
     <row r="362" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A362" t="s">
-        <v>149</v>
+        <v>137</v>
       </c>
       <c r="B362" t="s">
-        <v>32</v>
+        <v>143</v>
       </c>
       <c r="C362" t="b">
         <v>0</v>
       </c>
       <c r="D362" t="s">
-        <v>33</v>
+        <v>144</v>
       </c>
     </row>
     <row r="363" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A363" t="s">
-        <v>152</v>
+        <v>137</v>
       </c>
       <c r="B363" t="s">
-        <v>153</v>
+        <v>32</v>
       </c>
       <c r="C363" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D363" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
     </row>
     <row r="364" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A364" t="s">
-        <v>154</v>
+        <v>145</v>
       </c>
       <c r="B364" t="s">
-        <v>155</v>
+        <v>5</v>
       </c>
       <c r="C364" t="b">
         <v>1</v>
@@ -6115,13 +6115,13 @@
     </row>
     <row r="365" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A365" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="B365" t="s">
-        <v>5</v>
+        <v>146</v>
       </c>
       <c r="C365" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D365" t="s">
         <v>6</v>
@@ -6129,55 +6129,55 @@
     </row>
     <row r="366" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A366" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="B366" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="C366" t="b">
         <v>0</v>
       </c>
       <c r="D366" t="s">
-        <v>6</v>
+        <v>148</v>
       </c>
     </row>
     <row r="367" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A367" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="B367" t="s">
-        <v>147</v>
+        <v>32</v>
       </c>
       <c r="C367" t="b">
         <v>0</v>
       </c>
       <c r="D367" t="s">
-        <v>157</v>
+        <v>33</v>
       </c>
     </row>
     <row r="368" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A368" t="s">
-        <v>156</v>
+        <v>149</v>
       </c>
       <c r="B368" t="s">
-        <v>32</v>
+        <v>5</v>
       </c>
       <c r="C368" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D368" t="s">
-        <v>33</v>
+        <v>6</v>
       </c>
     </row>
     <row r="369" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A369" t="s">
-        <v>158</v>
+        <v>149</v>
       </c>
       <c r="B369" t="s">
-        <v>159</v>
+        <v>146</v>
       </c>
       <c r="C369" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D369" t="s">
         <v>6</v>
@@ -6185,97 +6185,97 @@
     </row>
     <row r="370" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A370" t="s">
-        <v>160</v>
+        <v>149</v>
       </c>
       <c r="B370" t="s">
-        <v>5</v>
+        <v>147</v>
       </c>
       <c r="C370" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D370" t="s">
-        <v>6</v>
+        <v>150</v>
       </c>
     </row>
     <row r="371" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A371" t="s">
-        <v>160</v>
+        <v>149</v>
       </c>
       <c r="B371" t="s">
-        <v>10</v>
+        <v>151</v>
       </c>
       <c r="C371" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D371" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="372" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A372" t="s">
-        <v>160</v>
+        <v>149</v>
       </c>
       <c r="B372" t="s">
-        <v>161</v>
+        <v>32</v>
       </c>
       <c r="C372" t="b">
         <v>0</v>
       </c>
       <c r="D372" t="s">
-        <v>9</v>
+        <v>33</v>
       </c>
     </row>
     <row r="373" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A373" t="s">
-        <v>160</v>
+        <v>152</v>
       </c>
       <c r="B373" t="s">
-        <v>31</v>
+        <v>153</v>
       </c>
       <c r="C373" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D373" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="374" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A374" t="s">
-        <v>160</v>
+        <v>154</v>
       </c>
       <c r="B374" t="s">
-        <v>32</v>
+        <v>155</v>
       </c>
       <c r="C374" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D374" t="s">
-        <v>33</v>
+        <v>6</v>
       </c>
     </row>
     <row r="375" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A375" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="B375" t="s">
-        <v>34</v>
+        <v>5</v>
       </c>
       <c r="C375" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D375" t="s">
-        <v>35</v>
+        <v>6</v>
       </c>
     </row>
     <row r="376" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A376" t="s">
-        <v>162</v>
+        <v>156</v>
       </c>
       <c r="B376" t="s">
-        <v>13</v>
+        <v>146</v>
       </c>
       <c r="C376" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D376" t="s">
         <v>6</v>
@@ -6283,41 +6283,41 @@
     </row>
     <row r="377" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A377" t="s">
-        <v>162</v>
+        <v>156</v>
       </c>
       <c r="B377" t="s">
-        <v>52</v>
+        <v>147</v>
       </c>
       <c r="C377" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D377" t="s">
-        <v>6</v>
+        <v>157</v>
       </c>
     </row>
     <row r="378" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A378" t="s">
-        <v>162</v>
+        <v>156</v>
       </c>
       <c r="B378" t="s">
-        <v>163</v>
+        <v>32</v>
       </c>
       <c r="C378" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D378" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
     </row>
     <row r="379" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A379" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="B379" t="s">
-        <v>12</v>
+        <v>159</v>
       </c>
       <c r="C379" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D379" t="s">
         <v>6</v>
@@ -6325,13 +6325,13 @@
     </row>
     <row r="380" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A380" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="B380" t="s">
-        <v>99</v>
+        <v>5</v>
       </c>
       <c r="C380" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D380" t="s">
         <v>6</v>
@@ -6339,7 +6339,7 @@
     </row>
     <row r="381" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A381" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="B381" t="s">
         <v>10</v>
@@ -6353,69 +6353,69 @@
     </row>
     <row r="382" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A382" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="B382" t="s">
-        <v>99</v>
+        <v>161</v>
       </c>
       <c r="C382" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D382" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="383" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A383" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="B383" t="s">
-        <v>12</v>
+        <v>31</v>
       </c>
       <c r="C383" t="b">
         <v>0</v>
       </c>
       <c r="D383" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="384" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A384" t="s">
-        <v>165</v>
+        <v>160</v>
       </c>
       <c r="B384" t="s">
-        <v>10</v>
+        <v>32</v>
       </c>
       <c r="C384" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D384" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
     </row>
     <row r="385" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A385" t="s">
-        <v>165</v>
+        <v>160</v>
       </c>
       <c r="B385" t="s">
-        <v>99</v>
+        <v>34</v>
       </c>
       <c r="C385" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D385" t="s">
-        <v>6</v>
+        <v>35</v>
       </c>
     </row>
     <row r="386" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A386" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="B386" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C386" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D386" t="s">
         <v>6</v>
@@ -6423,10 +6423,10 @@
     </row>
     <row r="387" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A387" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="B387" t="s">
-        <v>98</v>
+        <v>52</v>
       </c>
       <c r="C387" t="b">
         <v>1</v>
@@ -6437,10 +6437,10 @@
     </row>
     <row r="388" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A388" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="B388" t="s">
-        <v>97</v>
+        <v>163</v>
       </c>
       <c r="C388" t="b">
         <v>1</v>
@@ -6451,10 +6451,10 @@
     </row>
     <row r="389" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A389" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="B389" t="s">
-        <v>115</v>
+        <v>12</v>
       </c>
       <c r="C389" t="b">
         <v>0</v>
@@ -6465,13 +6465,13 @@
     </row>
     <row r="390" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A390" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="B390" t="s">
         <v>99</v>
       </c>
       <c r="C390" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D390" t="s">
         <v>6</v>
@@ -6479,10 +6479,10 @@
     </row>
     <row r="391" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A391" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="B391" t="s">
-        <v>97</v>
+        <v>10</v>
       </c>
       <c r="C391" t="b">
         <v>1</v>
@@ -6493,13 +6493,13 @@
     </row>
     <row r="392" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A392" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="B392" t="s">
-        <v>115</v>
+        <v>99</v>
       </c>
       <c r="C392" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D392" t="s">
         <v>6</v>
@@ -6507,13 +6507,13 @@
     </row>
     <row r="393" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A393" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="B393" t="s">
-        <v>99</v>
+        <v>12</v>
       </c>
       <c r="C393" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D393" t="s">
         <v>6</v>
@@ -6521,10 +6521,10 @@
     </row>
     <row r="394" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A394" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="B394" t="s">
-        <v>97</v>
+        <v>10</v>
       </c>
       <c r="C394" t="b">
         <v>1</v>
@@ -6535,13 +6535,13 @@
     </row>
     <row r="395" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A395" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="B395" t="s">
-        <v>115</v>
+        <v>99</v>
       </c>
       <c r="C395" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D395" t="s">
         <v>6</v>
@@ -6549,13 +6549,13 @@
     </row>
     <row r="396" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A396" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="B396" t="s">
-        <v>99</v>
+        <v>12</v>
       </c>
       <c r="C396" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D396" t="s">
         <v>6</v>
@@ -6563,13 +6563,13 @@
     </row>
     <row r="397" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A397" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="B397" t="s">
-        <v>170</v>
+        <v>98</v>
       </c>
       <c r="C397" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D397" t="s">
         <v>6</v>
@@ -6577,13 +6577,13 @@
     </row>
     <row r="398" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A398" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="B398" t="s">
-        <v>7</v>
+        <v>97</v>
       </c>
       <c r="C398" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D398" t="s">
         <v>6</v>
@@ -6591,69 +6591,69 @@
     </row>
     <row r="399" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A399" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="B399" t="s">
-        <v>8</v>
+        <v>115</v>
       </c>
       <c r="C399" t="b">
         <v>0</v>
       </c>
       <c r="D399" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="400" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A400" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="B400" t="s">
-        <v>32</v>
+        <v>99</v>
       </c>
       <c r="C400" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D400" t="s">
-        <v>33</v>
+        <v>6</v>
       </c>
     </row>
     <row r="401" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A401" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="B401" t="s">
-        <v>34</v>
+        <v>97</v>
       </c>
       <c r="C401" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D401" t="s">
-        <v>35</v>
+        <v>6</v>
       </c>
     </row>
     <row r="402" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A402" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="B402" t="s">
-        <v>31</v>
+        <v>115</v>
       </c>
       <c r="C402" t="b">
         <v>0</v>
       </c>
       <c r="D402" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="403" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A403" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="B403" t="s">
-        <v>172</v>
+        <v>99</v>
       </c>
       <c r="C403" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D403" t="s">
         <v>6</v>
@@ -6661,66 +6661,66 @@
     </row>
     <row r="404" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A404" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="B404" t="s">
-        <v>8</v>
+        <v>97</v>
       </c>
       <c r="C404" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D404" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="405" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A405" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="B405" t="s">
-        <v>32</v>
+        <v>115</v>
       </c>
       <c r="C405" t="b">
         <v>0</v>
       </c>
       <c r="D405" t="s">
-        <v>33</v>
+        <v>6</v>
       </c>
     </row>
     <row r="406" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A406" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="B406" t="s">
-        <v>34</v>
+        <v>99</v>
       </c>
       <c r="C406" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D406" t="s">
-        <v>35</v>
+        <v>6</v>
       </c>
     </row>
     <row r="407" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A407" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="B407" t="s">
-        <v>31</v>
+        <v>170</v>
       </c>
       <c r="C407" t="b">
         <v>0</v>
       </c>
       <c r="D407" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="408" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A408" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="B408" t="s">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="C408" t="b">
         <v>0</v>
@@ -6731,136 +6731,136 @@
     </row>
     <row r="409" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A409" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="B409" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C409" t="b">
         <v>0</v>
       </c>
       <c r="D409" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="410" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A410" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="B410" t="s">
-        <v>8</v>
+        <v>32</v>
       </c>
       <c r="C410" t="b">
         <v>0</v>
       </c>
       <c r="D410" t="s">
-        <v>9</v>
+        <v>33</v>
       </c>
     </row>
     <row r="411" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A411" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="B411" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C411" t="b">
         <v>0</v>
       </c>
       <c r="D411" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="412" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A412" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="B412" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C412" t="b">
         <v>0</v>
       </c>
       <c r="D412" t="s">
-        <v>35</v>
+        <v>9</v>
       </c>
     </row>
     <row r="413" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A413" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="B413" t="s">
-        <v>31</v>
+        <v>172</v>
       </c>
       <c r="C413" t="b">
         <v>0</v>
       </c>
       <c r="D413" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="414" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A414" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="B414" t="s">
-        <v>97</v>
+        <v>8</v>
       </c>
       <c r="C414" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D414" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="415" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A415" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="B415" t="s">
-        <v>115</v>
+        <v>32</v>
       </c>
       <c r="C415" t="b">
         <v>0</v>
       </c>
       <c r="D415" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
     </row>
     <row r="416" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A416" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="B416" t="s">
-        <v>175</v>
+        <v>34</v>
       </c>
       <c r="C416" t="b">
         <v>0</v>
       </c>
       <c r="D416" t="s">
-        <v>6</v>
+        <v>35</v>
       </c>
     </row>
     <row r="417" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A417" t="s">
-        <v>176</v>
+        <v>171</v>
       </c>
       <c r="B417" t="s">
-        <v>97</v>
+        <v>31</v>
       </c>
       <c r="C417" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D417" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="418" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A418" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="B418" t="s">
-        <v>115</v>
+        <v>13</v>
       </c>
       <c r="C418" t="b">
         <v>0</v>
@@ -6871,10 +6871,10 @@
     </row>
     <row r="419" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A419" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="B419" t="s">
-        <v>175</v>
+        <v>10</v>
       </c>
       <c r="C419" t="b">
         <v>0</v>
@@ -6885,111 +6885,111 @@
     </row>
     <row r="420" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A420" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="B420" t="s">
-        <v>177</v>
+        <v>8</v>
       </c>
       <c r="C420" t="b">
         <v>0</v>
       </c>
       <c r="D420" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="421" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A421" t="s">
-        <v>178</v>
+        <v>173</v>
       </c>
       <c r="B421" t="s">
-        <v>179</v>
+        <v>32</v>
       </c>
       <c r="C421" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D421" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
     </row>
     <row r="422" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A422" t="s">
-        <v>178</v>
+        <v>173</v>
       </c>
       <c r="B422" t="s">
-        <v>10</v>
+        <v>34</v>
       </c>
       <c r="C422" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D422" t="s">
-        <v>6</v>
+        <v>35</v>
       </c>
     </row>
     <row r="423" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A423" t="s">
-        <v>178</v>
+        <v>173</v>
       </c>
       <c r="B423" t="s">
-        <v>12</v>
+        <v>31</v>
       </c>
       <c r="C423" t="b">
         <v>0</v>
       </c>
       <c r="D423" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="424" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A424" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="B424" t="s">
-        <v>32</v>
+        <v>97</v>
       </c>
       <c r="C424" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D424" t="s">
-        <v>33</v>
+        <v>6</v>
       </c>
     </row>
     <row r="425" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A425" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="B425" t="s">
-        <v>8</v>
+        <v>115</v>
       </c>
       <c r="C425" t="b">
         <v>0</v>
       </c>
       <c r="D425" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="426" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A426" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="B426" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
       <c r="C426" t="b">
         <v>0</v>
       </c>
       <c r="D426" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="427" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A427" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="B427" t="s">
-        <v>38</v>
+        <v>97</v>
       </c>
       <c r="C427" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D427" t="s">
         <v>6</v>
@@ -6997,13 +6997,13 @@
     </row>
     <row r="428" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A428" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="B428" t="s">
-        <v>182</v>
+        <v>115</v>
       </c>
       <c r="C428" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D428" t="s">
         <v>6</v>
@@ -7011,13 +7011,13 @@
     </row>
     <row r="429" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A429" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="B429" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="C429" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D429" t="s">
         <v>6</v>
@@ -7025,13 +7025,13 @@
     </row>
     <row r="430" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A430" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="B430" t="s">
-        <v>10</v>
+        <v>177</v>
       </c>
       <c r="C430" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D430" t="s">
         <v>6</v>
@@ -7039,13 +7039,13 @@
     </row>
     <row r="431" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A431" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="B431" t="s">
-        <v>12</v>
+        <v>179</v>
       </c>
       <c r="C431" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D431" t="s">
         <v>6</v>
@@ -7053,80 +7053,80 @@
     </row>
     <row r="432" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A432" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="B432" t="s">
-        <v>32</v>
+        <v>10</v>
       </c>
       <c r="C432" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D432" t="s">
-        <v>33</v>
+        <v>6</v>
       </c>
     </row>
     <row r="433" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A433" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="B433" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="C433" t="b">
         <v>0</v>
       </c>
       <c r="D433" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="434" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A434" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="B434" t="s">
-        <v>46</v>
+        <v>32</v>
       </c>
       <c r="C434" t="b">
         <v>0</v>
       </c>
       <c r="D434" t="s">
-        <v>9</v>
+        <v>33</v>
       </c>
     </row>
     <row r="435" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A435" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="B435" t="s">
-        <v>38</v>
+        <v>8</v>
       </c>
       <c r="C435" t="b">
         <v>0</v>
       </c>
       <c r="D435" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="436" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A436" t="s">
-        <v>84</v>
+        <v>178</v>
       </c>
       <c r="B436" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="C436" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D436" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="437" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A437" t="s">
-        <v>84</v>
+        <v>178</v>
       </c>
       <c r="B437" t="s">
-        <v>12</v>
+        <v>38</v>
       </c>
       <c r="C437" t="b">
         <v>0</v>
@@ -7137,38 +7137,38 @@
     </row>
     <row r="438" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A438" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="B438" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="C438" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D438" t="s">
-        <v>186</v>
+        <v>6</v>
       </c>
     </row>
     <row r="439" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A439" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="B439" t="s">
-        <v>187</v>
+        <v>179</v>
       </c>
       <c r="C439" t="b">
         <v>1</v>
       </c>
       <c r="D439" t="s">
-        <v>188</v>
+        <v>6</v>
       </c>
     </row>
     <row r="440" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A440" t="s">
-        <v>189</v>
+        <v>181</v>
       </c>
       <c r="B440" t="s">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="C440" t="b">
         <v>1</v>
@@ -7179,13 +7179,13 @@
     </row>
     <row r="441" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A441" t="s">
-        <v>189</v>
+        <v>181</v>
       </c>
       <c r="B441" t="s">
-        <v>190</v>
+        <v>12</v>
       </c>
       <c r="C441" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D441" t="s">
         <v>6</v>
@@ -7193,55 +7193,55 @@
     </row>
     <row r="442" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A442" t="s">
-        <v>191</v>
+        <v>181</v>
       </c>
       <c r="B442" t="s">
-        <v>5</v>
+        <v>32</v>
       </c>
       <c r="C442" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D442" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
     </row>
     <row r="443" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A443" t="s">
-        <v>191</v>
+        <v>181</v>
       </c>
       <c r="B443" t="s">
-        <v>190</v>
+        <v>8</v>
       </c>
       <c r="C443" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D443" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="444" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A444" t="s">
-        <v>192</v>
+        <v>181</v>
       </c>
       <c r="B444" t="s">
-        <v>97</v>
+        <v>46</v>
       </c>
       <c r="C444" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D444" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="445" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A445" t="s">
-        <v>192</v>
+        <v>181</v>
       </c>
       <c r="B445" t="s">
-        <v>193</v>
+        <v>38</v>
       </c>
       <c r="C445" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D445" t="s">
         <v>6</v>
@@ -7249,10 +7249,10 @@
     </row>
     <row r="446" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A446" t="s">
-        <v>194</v>
+        <v>84</v>
       </c>
       <c r="B446" t="s">
-        <v>97</v>
+        <v>183</v>
       </c>
       <c r="C446" t="b">
         <v>1</v>
@@ -7263,13 +7263,13 @@
     </row>
     <row r="447" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A447" t="s">
-        <v>194</v>
+        <v>84</v>
       </c>
       <c r="B447" t="s">
-        <v>195</v>
+        <v>12</v>
       </c>
       <c r="C447" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D447" t="s">
         <v>6</v>
@@ -7277,38 +7277,38 @@
     </row>
     <row r="448" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A448" t="s">
-        <v>196</v>
+        <v>184</v>
       </c>
       <c r="B448" t="s">
-        <v>5</v>
+        <v>185</v>
       </c>
       <c r="C448" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D448" t="s">
-        <v>6</v>
+        <v>186</v>
       </c>
     </row>
     <row r="449" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A449" t="s">
-        <v>197</v>
+        <v>184</v>
       </c>
       <c r="B449" t="s">
-        <v>5</v>
+        <v>187</v>
       </c>
       <c r="C449" t="b">
         <v>1</v>
       </c>
       <c r="D449" t="s">
-        <v>6</v>
+        <v>188</v>
       </c>
     </row>
     <row r="450" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A450" t="s">
-        <v>198</v>
+        <v>189</v>
       </c>
       <c r="B450" t="s">
-        <v>199</v>
+        <v>5</v>
       </c>
       <c r="C450" t="b">
         <v>1</v>
@@ -7319,10 +7319,10 @@
     </row>
     <row r="451" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A451" t="s">
-        <v>200</v>
+        <v>189</v>
       </c>
       <c r="B451" t="s">
-        <v>5</v>
+        <v>190</v>
       </c>
       <c r="C451" t="b">
         <v>1</v>
@@ -7333,13 +7333,13 @@
     </row>
     <row r="452" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A452" t="s">
-        <v>200</v>
+        <v>191</v>
       </c>
       <c r="B452" t="s">
-        <v>201</v>
+        <v>5</v>
       </c>
       <c r="C452" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D452" t="s">
         <v>6</v>
@@ -7347,10 +7347,10 @@
     </row>
     <row r="453" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A453" t="s">
-        <v>202</v>
+        <v>191</v>
       </c>
       <c r="B453" t="s">
-        <v>5</v>
+        <v>190</v>
       </c>
       <c r="C453" t="b">
         <v>1</v>
@@ -7361,13 +7361,13 @@
     </row>
     <row r="454" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A454" t="s">
-        <v>202</v>
+        <v>192</v>
       </c>
       <c r="B454" t="s">
-        <v>201</v>
+        <v>97</v>
       </c>
       <c r="C454" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D454" t="s">
         <v>6</v>
@@ -7375,10 +7375,10 @@
     </row>
     <row r="455" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A455" t="s">
-        <v>203</v>
+        <v>192</v>
       </c>
       <c r="B455" t="s">
-        <v>5</v>
+        <v>193</v>
       </c>
       <c r="C455" t="b">
         <v>1</v>
@@ -7389,13 +7389,13 @@
     </row>
     <row r="456" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A456" t="s">
-        <v>203</v>
+        <v>194</v>
       </c>
       <c r="B456" t="s">
-        <v>201</v>
+        <v>97</v>
       </c>
       <c r="C456" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D456" t="s">
         <v>6</v>
@@ -7403,10 +7403,10 @@
     </row>
     <row r="457" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A457" t="s">
-        <v>204</v>
+        <v>194</v>
       </c>
       <c r="B457" t="s">
-        <v>5</v>
+        <v>195</v>
       </c>
       <c r="C457" t="b">
         <v>1</v>
@@ -7417,13 +7417,13 @@
     </row>
     <row r="458" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A458" t="s">
-        <v>204</v>
+        <v>196</v>
       </c>
       <c r="B458" t="s">
-        <v>201</v>
+        <v>5</v>
       </c>
       <c r="C458" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D458" t="s">
         <v>6</v>
@@ -7431,7 +7431,7 @@
     </row>
     <row r="459" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A459" t="s">
-        <v>205</v>
+        <v>197</v>
       </c>
       <c r="B459" t="s">
         <v>5</v>
@@ -7445,13 +7445,13 @@
     </row>
     <row r="460" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A460" t="s">
-        <v>206</v>
+        <v>198</v>
       </c>
       <c r="B460" t="s">
-        <v>5</v>
+        <v>199</v>
       </c>
       <c r="C460" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D460" t="s">
         <v>6</v>
@@ -7459,13 +7459,13 @@
     </row>
     <row r="461" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A461" t="s">
-        <v>206</v>
+        <v>200</v>
       </c>
       <c r="B461" t="s">
-        <v>182</v>
+        <v>5</v>
       </c>
       <c r="C461" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D461" t="s">
         <v>6</v>
@@ -7473,10 +7473,10 @@
     </row>
     <row r="462" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A462" t="s">
-        <v>206</v>
+        <v>200</v>
       </c>
       <c r="B462" t="s">
-        <v>179</v>
+        <v>201</v>
       </c>
       <c r="C462" t="b">
         <v>0</v>
@@ -7487,10 +7487,10 @@
     </row>
     <row r="463" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A463" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
       <c r="B463" t="s">
-        <v>207</v>
+        <v>5</v>
       </c>
       <c r="C463" t="b">
         <v>1</v>
@@ -7501,10 +7501,10 @@
     </row>
     <row r="464" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A464" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
       <c r="B464" t="s">
-        <v>12</v>
+        <v>201</v>
       </c>
       <c r="C464" t="b">
         <v>0</v>
@@ -7515,7 +7515,7 @@
     </row>
     <row r="465" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A465" t="s">
-        <v>208</v>
+        <v>203</v>
       </c>
       <c r="B465" t="s">
         <v>5</v>
@@ -7529,10 +7529,10 @@
     </row>
     <row r="466" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A466" t="s">
-        <v>208</v>
+        <v>203</v>
       </c>
       <c r="B466" t="s">
-        <v>7</v>
+        <v>201</v>
       </c>
       <c r="C466" t="b">
         <v>0</v>
@@ -7543,27 +7543,27 @@
     </row>
     <row r="467" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A467" t="s">
-        <v>208</v>
+        <v>204</v>
       </c>
       <c r="B467" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="C467" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D467" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="468" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A468" t="s">
-        <v>208</v>
+        <v>204</v>
       </c>
       <c r="B468" t="s">
-        <v>10</v>
+        <v>201</v>
       </c>
       <c r="C468" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D468" t="s">
         <v>6</v>
@@ -7571,13 +7571,13 @@
     </row>
     <row r="469" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A469" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="B469" t="s">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="C469" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D469" t="s">
         <v>6</v>
@@ -7585,13 +7585,13 @@
     </row>
     <row r="470" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A470" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="B470" t="s">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="C470" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D470" t="s">
         <v>6</v>
@@ -7599,13 +7599,13 @@
     </row>
     <row r="471" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A471" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="B471" t="s">
-        <v>45</v>
+        <v>182</v>
       </c>
       <c r="C471" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D471" t="s">
         <v>6</v>
@@ -7613,24 +7613,24 @@
     </row>
     <row r="472" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A472" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="B472" t="s">
-        <v>46</v>
+        <v>179</v>
       </c>
       <c r="C472" t="b">
         <v>0</v>
       </c>
       <c r="D472" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="473" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A473" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="B473" t="s">
-        <v>13</v>
+        <v>207</v>
       </c>
       <c r="C473" t="b">
         <v>1</v>
@@ -7641,10 +7641,10 @@
     </row>
     <row r="474" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A474" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="B474" t="s">
-        <v>37</v>
+        <v>12</v>
       </c>
       <c r="C474" t="b">
         <v>0</v>
@@ -7658,7 +7658,7 @@
         <v>208</v>
       </c>
       <c r="B475" t="s">
-        <v>38</v>
+        <v>5</v>
       </c>
       <c r="C475" t="b">
         <v>1</v>
@@ -7672,10 +7672,10 @@
         <v>208</v>
       </c>
       <c r="B476" t="s">
-        <v>52</v>
+        <v>7</v>
       </c>
       <c r="C476" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D476" t="s">
         <v>6</v>
@@ -7686,13 +7686,13 @@
         <v>208</v>
       </c>
       <c r="B477" t="s">
-        <v>19</v>
+        <v>8</v>
       </c>
       <c r="C477" t="b">
         <v>0</v>
       </c>
       <c r="D477" t="s">
-        <v>20</v>
+        <v>9</v>
       </c>
     </row>
     <row r="478" spans="1:4" x14ac:dyDescent="0.25">
@@ -7700,13 +7700,13 @@
         <v>208</v>
       </c>
       <c r="B478" t="s">
-        <v>31</v>
+        <v>10</v>
       </c>
       <c r="C478" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D478" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="479" spans="1:4" x14ac:dyDescent="0.25">
@@ -7714,13 +7714,13 @@
         <v>208</v>
       </c>
       <c r="B479" t="s">
-        <v>32</v>
+        <v>11</v>
       </c>
       <c r="C479" t="b">
         <v>0</v>
       </c>
       <c r="D479" t="s">
-        <v>33</v>
+        <v>6</v>
       </c>
     </row>
     <row r="480" spans="1:4" x14ac:dyDescent="0.25">
@@ -7728,12 +7728,152 @@
         <v>208</v>
       </c>
       <c r="B480" t="s">
+        <v>12</v>
+      </c>
+      <c r="C480" t="b">
+        <v>1</v>
+      </c>
+      <c r="D480" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="481" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A481" t="s">
+        <v>208</v>
+      </c>
+      <c r="B481" t="s">
+        <v>45</v>
+      </c>
+      <c r="C481" t="b">
+        <v>1</v>
+      </c>
+      <c r="D481" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="482" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A482" t="s">
+        <v>208</v>
+      </c>
+      <c r="B482" t="s">
+        <v>46</v>
+      </c>
+      <c r="C482" t="b">
+        <v>0</v>
+      </c>
+      <c r="D482" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="483" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A483" t="s">
+        <v>208</v>
+      </c>
+      <c r="B483" t="s">
+        <v>13</v>
+      </c>
+      <c r="C483" t="b">
+        <v>1</v>
+      </c>
+      <c r="D483" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="484" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A484" t="s">
+        <v>208</v>
+      </c>
+      <c r="B484" t="s">
+        <v>37</v>
+      </c>
+      <c r="C484" t="b">
+        <v>0</v>
+      </c>
+      <c r="D484" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="485" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A485" t="s">
+        <v>208</v>
+      </c>
+      <c r="B485" t="s">
+        <v>38</v>
+      </c>
+      <c r="C485" t="b">
+        <v>1</v>
+      </c>
+      <c r="D485" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="486" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A486" t="s">
+        <v>208</v>
+      </c>
+      <c r="B486" t="s">
+        <v>52</v>
+      </c>
+      <c r="C486" t="b">
+        <v>1</v>
+      </c>
+      <c r="D486" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="487" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A487" t="s">
+        <v>208</v>
+      </c>
+      <c r="B487" t="s">
+        <v>19</v>
+      </c>
+      <c r="C487" t="b">
+        <v>0</v>
+      </c>
+      <c r="D487" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="488" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A488" t="s">
+        <v>208</v>
+      </c>
+      <c r="B488" t="s">
+        <v>31</v>
+      </c>
+      <c r="C488" t="b">
+        <v>0</v>
+      </c>
+      <c r="D488" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="489" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A489" t="s">
+        <v>208</v>
+      </c>
+      <c r="B489" t="s">
+        <v>32</v>
+      </c>
+      <c r="C489" t="b">
+        <v>0</v>
+      </c>
+      <c r="D489" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="490" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A490" t="s">
+        <v>208</v>
+      </c>
+      <c r="B490" t="s">
         <v>34</v>
       </c>
-      <c r="C480" t="b">
-        <v>0</v>
-      </c>
-      <c r="D480" t="s">
+      <c r="C490" t="b">
+        <v>0</v>
+      </c>
+      <c r="D490" t="s">
         <v>35</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Deploying to gh-pages from @ open-resource-discovery/specification@6440f0c216cdc6c65c79fc2a89a9b9ef2b625dcd 🚀
</commit_message>
<xml_diff>
--- a/spec-v1/interfaces/Document.xlsx
+++ b/spec-v1/interfaces/Document.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1471" uniqueCount="209">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1474" uniqueCount="209">
   <si>
     <t>Entity Name</t>
   </si>
@@ -1014,7 +1014,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D490"/>
+  <dimension ref="A1:D491"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -5488,13 +5488,13 @@
         <v>127</v>
       </c>
       <c r="B320" t="s">
-        <v>27</v>
+        <v>83</v>
       </c>
       <c r="C320" t="b">
         <v>0</v>
       </c>
       <c r="D320" t="s">
-        <v>9</v>
+        <v>84</v>
       </c>
     </row>
     <row r="321" spans="1:4" x14ac:dyDescent="0.25">
@@ -5502,7 +5502,7 @@
         <v>127</v>
       </c>
       <c r="B321" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C321" t="b">
         <v>0</v>
@@ -5516,7 +5516,7 @@
         <v>127</v>
       </c>
       <c r="B322" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C322" t="b">
         <v>0</v>
@@ -5530,7 +5530,7 @@
         <v>127</v>
       </c>
       <c r="B323" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C323" t="b">
         <v>0</v>
@@ -5544,13 +5544,13 @@
         <v>127</v>
       </c>
       <c r="B324" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C324" t="b">
         <v>0</v>
       </c>
       <c r="D324" t="s">
-        <v>33</v>
+        <v>9</v>
       </c>
     </row>
     <row r="325" spans="1:4" x14ac:dyDescent="0.25">
@@ -5558,13 +5558,13 @@
         <v>127</v>
       </c>
       <c r="B325" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C325" t="b">
         <v>0</v>
       </c>
       <c r="D325" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="326" spans="1:4" x14ac:dyDescent="0.25">
@@ -5572,13 +5572,13 @@
         <v>127</v>
       </c>
       <c r="B326" t="s">
-        <v>16</v>
+        <v>34</v>
       </c>
       <c r="C326" t="b">
         <v>0</v>
       </c>
       <c r="D326" t="s">
-        <v>9</v>
+        <v>35</v>
       </c>
     </row>
     <row r="327" spans="1:4" x14ac:dyDescent="0.25">
@@ -5586,27 +5586,27 @@
         <v>127</v>
       </c>
       <c r="B327" t="s">
-        <v>85</v>
+        <v>16</v>
       </c>
       <c r="C327" t="b">
         <v>0</v>
       </c>
       <c r="D327" t="s">
-        <v>51</v>
+        <v>9</v>
       </c>
     </row>
     <row r="328" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A328" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="B328" t="s">
-        <v>97</v>
+        <v>85</v>
       </c>
       <c r="C328" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D328" t="s">
-        <v>6</v>
+        <v>51</v>
       </c>
     </row>
     <row r="329" spans="1:4" x14ac:dyDescent="0.25">
@@ -5614,10 +5614,10 @@
         <v>131</v>
       </c>
       <c r="B329" t="s">
-        <v>115</v>
+        <v>97</v>
       </c>
       <c r="C329" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D329" t="s">
         <v>6</v>
@@ -5628,10 +5628,10 @@
         <v>131</v>
       </c>
       <c r="B330" t="s">
-        <v>98</v>
+        <v>115</v>
       </c>
       <c r="C330" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D330" t="s">
         <v>6</v>
@@ -5642,7 +5642,7 @@
         <v>131</v>
       </c>
       <c r="B331" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C331" t="b">
         <v>1</v>
@@ -5656,13 +5656,13 @@
         <v>131</v>
       </c>
       <c r="B332" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C332" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D332" t="s">
-        <v>101</v>
+        <v>6</v>
       </c>
     </row>
     <row r="333" spans="1:4" x14ac:dyDescent="0.25">
@@ -5670,13 +5670,13 @@
         <v>131</v>
       </c>
       <c r="B333" t="s">
-        <v>38</v>
+        <v>100</v>
       </c>
       <c r="C333" t="b">
         <v>0</v>
       </c>
       <c r="D333" t="s">
-        <v>6</v>
+        <v>101</v>
       </c>
     </row>
     <row r="334" spans="1:4" x14ac:dyDescent="0.25">
@@ -5684,7 +5684,7 @@
         <v>131</v>
       </c>
       <c r="B334" t="s">
-        <v>116</v>
+        <v>38</v>
       </c>
       <c r="C334" t="b">
         <v>0</v>
@@ -5695,13 +5695,13 @@
     </row>
     <row r="335" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A335" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B335" t="s">
-        <v>5</v>
+        <v>116</v>
       </c>
       <c r="C335" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D335" t="s">
         <v>6</v>
@@ -5712,10 +5712,10 @@
         <v>132</v>
       </c>
       <c r="B336" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C336" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D336" t="s">
         <v>6</v>
@@ -5726,13 +5726,13 @@
         <v>132</v>
       </c>
       <c r="B337" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C337" t="b">
         <v>0</v>
       </c>
       <c r="D337" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="338" spans="1:4" x14ac:dyDescent="0.25">
@@ -5740,13 +5740,13 @@
         <v>132</v>
       </c>
       <c r="B338" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C338" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D338" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="339" spans="1:4" x14ac:dyDescent="0.25">
@@ -5754,10 +5754,10 @@
         <v>132</v>
       </c>
       <c r="B339" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C339" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D339" t="s">
         <v>6</v>
@@ -5768,7 +5768,7 @@
         <v>132</v>
       </c>
       <c r="B340" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C340" t="b">
         <v>0</v>
@@ -5782,10 +5782,10 @@
         <v>132</v>
       </c>
       <c r="B341" t="s">
-        <v>45</v>
+        <v>12</v>
       </c>
       <c r="C341" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D341" t="s">
         <v>6</v>
@@ -5796,13 +5796,13 @@
         <v>132</v>
       </c>
       <c r="B342" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C342" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D342" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="343" spans="1:4" x14ac:dyDescent="0.25">
@@ -5810,13 +5810,13 @@
         <v>132</v>
       </c>
       <c r="B343" t="s">
-        <v>13</v>
+        <v>46</v>
       </c>
       <c r="C343" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D343" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="344" spans="1:4" x14ac:dyDescent="0.25">
@@ -5824,10 +5824,10 @@
         <v>132</v>
       </c>
       <c r="B344" t="s">
-        <v>37</v>
+        <v>13</v>
       </c>
       <c r="C344" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D344" t="s">
         <v>6</v>
@@ -5838,10 +5838,10 @@
         <v>132</v>
       </c>
       <c r="B345" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C345" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D345" t="s">
         <v>6</v>
@@ -5852,7 +5852,7 @@
         <v>132</v>
       </c>
       <c r="B346" t="s">
-        <v>52</v>
+        <v>38</v>
       </c>
       <c r="C346" t="b">
         <v>1</v>
@@ -5866,10 +5866,10 @@
         <v>132</v>
       </c>
       <c r="B347" t="s">
-        <v>60</v>
+        <v>52</v>
       </c>
       <c r="C347" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D347" t="s">
         <v>6</v>
@@ -5880,13 +5880,13 @@
         <v>132</v>
       </c>
       <c r="B348" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C348" t="b">
         <v>0</v>
       </c>
       <c r="D348" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="349" spans="1:4" x14ac:dyDescent="0.25">
@@ -5894,13 +5894,13 @@
         <v>132</v>
       </c>
       <c r="B349" t="s">
-        <v>133</v>
+        <v>61</v>
       </c>
       <c r="C349" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D349" t="s">
-        <v>51</v>
+        <v>9</v>
       </c>
     </row>
     <row r="350" spans="1:4" x14ac:dyDescent="0.25">
@@ -5908,13 +5908,13 @@
         <v>132</v>
       </c>
       <c r="B350" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C350" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D350" t="s">
-        <v>135</v>
+        <v>51</v>
       </c>
     </row>
     <row r="351" spans="1:4" x14ac:dyDescent="0.25">
@@ -5922,13 +5922,13 @@
         <v>132</v>
       </c>
       <c r="B351" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="C351" t="b">
         <v>0</v>
       </c>
       <c r="D351" t="s">
-        <v>9</v>
+        <v>135</v>
       </c>
     </row>
     <row r="352" spans="1:4" x14ac:dyDescent="0.25">
@@ -5936,13 +5936,13 @@
         <v>132</v>
       </c>
       <c r="B352" t="s">
-        <v>19</v>
+        <v>136</v>
       </c>
       <c r="C352" t="b">
         <v>0</v>
       </c>
       <c r="D352" t="s">
-        <v>20</v>
+        <v>9</v>
       </c>
     </row>
     <row r="353" spans="1:4" x14ac:dyDescent="0.25">
@@ -5950,13 +5950,13 @@
         <v>132</v>
       </c>
       <c r="B353" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="C353" t="b">
         <v>0</v>
       </c>
       <c r="D353" t="s">
-        <v>9</v>
+        <v>20</v>
       </c>
     </row>
     <row r="354" spans="1:4" x14ac:dyDescent="0.25">
@@ -5964,13 +5964,13 @@
         <v>132</v>
       </c>
       <c r="B354" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C354" t="b">
         <v>0</v>
       </c>
       <c r="D354" t="s">
-        <v>33</v>
+        <v>9</v>
       </c>
     </row>
     <row r="355" spans="1:4" x14ac:dyDescent="0.25">
@@ -5978,27 +5978,27 @@
         <v>132</v>
       </c>
       <c r="B355" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C355" t="b">
         <v>0</v>
       </c>
       <c r="D355" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="356" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A356" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="B356" t="s">
-        <v>10</v>
+        <v>34</v>
       </c>
       <c r="C356" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D356" t="s">
-        <v>6</v>
+        <v>35</v>
       </c>
     </row>
     <row r="357" spans="1:4" x14ac:dyDescent="0.25">
@@ -6006,10 +6006,10 @@
         <v>137</v>
       </c>
       <c r="B357" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C357" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D357" t="s">
         <v>6</v>
@@ -6020,13 +6020,13 @@
         <v>137</v>
       </c>
       <c r="B358" t="s">
-        <v>133</v>
+        <v>12</v>
       </c>
       <c r="C358" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D358" t="s">
-        <v>51</v>
+        <v>6</v>
       </c>
     </row>
     <row r="359" spans="1:4" x14ac:dyDescent="0.25">
@@ -6034,10 +6034,10 @@
         <v>137</v>
       </c>
       <c r="B359" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="C359" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D359" t="s">
         <v>51</v>
@@ -6048,13 +6048,13 @@
         <v>137</v>
       </c>
       <c r="B360" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C360" t="b">
         <v>0</v>
       </c>
       <c r="D360" t="s">
-        <v>140</v>
+        <v>51</v>
       </c>
     </row>
     <row r="361" spans="1:4" x14ac:dyDescent="0.25">
@@ -6062,13 +6062,13 @@
         <v>137</v>
       </c>
       <c r="B361" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="C361" t="b">
         <v>0</v>
       </c>
       <c r="D361" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
     </row>
     <row r="362" spans="1:4" x14ac:dyDescent="0.25">
@@ -6076,13 +6076,13 @@
         <v>137</v>
       </c>
       <c r="B362" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="C362" t="b">
         <v>0</v>
       </c>
       <c r="D362" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
     </row>
     <row r="363" spans="1:4" x14ac:dyDescent="0.25">
@@ -6090,27 +6090,27 @@
         <v>137</v>
       </c>
       <c r="B363" t="s">
-        <v>32</v>
+        <v>143</v>
       </c>
       <c r="C363" t="b">
         <v>0</v>
       </c>
       <c r="D363" t="s">
-        <v>33</v>
+        <v>144</v>
       </c>
     </row>
     <row r="364" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A364" t="s">
-        <v>145</v>
+        <v>137</v>
       </c>
       <c r="B364" t="s">
-        <v>5</v>
+        <v>32</v>
       </c>
       <c r="C364" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D364" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
     </row>
     <row r="365" spans="1:4" x14ac:dyDescent="0.25">
@@ -6118,10 +6118,10 @@
         <v>145</v>
       </c>
       <c r="B365" t="s">
-        <v>146</v>
+        <v>5</v>
       </c>
       <c r="C365" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D365" t="s">
         <v>6</v>
@@ -6132,13 +6132,13 @@
         <v>145</v>
       </c>
       <c r="B366" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C366" t="b">
         <v>0</v>
       </c>
       <c r="D366" t="s">
-        <v>148</v>
+        <v>6</v>
       </c>
     </row>
     <row r="367" spans="1:4" x14ac:dyDescent="0.25">
@@ -6146,27 +6146,27 @@
         <v>145</v>
       </c>
       <c r="B367" t="s">
-        <v>32</v>
+        <v>147</v>
       </c>
       <c r="C367" t="b">
         <v>0</v>
       </c>
       <c r="D367" t="s">
-        <v>33</v>
+        <v>148</v>
       </c>
     </row>
     <row r="368" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A368" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="B368" t="s">
-        <v>5</v>
+        <v>32</v>
       </c>
       <c r="C368" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D368" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
     </row>
     <row r="369" spans="1:4" x14ac:dyDescent="0.25">
@@ -6174,10 +6174,10 @@
         <v>149</v>
       </c>
       <c r="B369" t="s">
-        <v>146</v>
+        <v>5</v>
       </c>
       <c r="C369" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D369" t="s">
         <v>6</v>
@@ -6188,13 +6188,13 @@
         <v>149</v>
       </c>
       <c r="B370" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C370" t="b">
         <v>0</v>
       </c>
       <c r="D370" t="s">
-        <v>150</v>
+        <v>6</v>
       </c>
     </row>
     <row r="371" spans="1:4" x14ac:dyDescent="0.25">
@@ -6202,13 +6202,13 @@
         <v>149</v>
       </c>
       <c r="B371" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="C371" t="b">
         <v>0</v>
       </c>
       <c r="D371" t="s">
-        <v>9</v>
+        <v>150</v>
       </c>
     </row>
     <row r="372" spans="1:4" x14ac:dyDescent="0.25">
@@ -6216,35 +6216,35 @@
         <v>149</v>
       </c>
       <c r="B372" t="s">
-        <v>32</v>
+        <v>151</v>
       </c>
       <c r="C372" t="b">
         <v>0</v>
       </c>
       <c r="D372" t="s">
-        <v>33</v>
+        <v>9</v>
       </c>
     </row>
     <row r="373" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A373" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="B373" t="s">
-        <v>153</v>
+        <v>32</v>
       </c>
       <c r="C373" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D373" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
     </row>
     <row r="374" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A374" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="B374" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="C374" t="b">
         <v>1</v>
@@ -6255,10 +6255,10 @@
     </row>
     <row r="375" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A375" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="B375" t="s">
-        <v>5</v>
+        <v>155</v>
       </c>
       <c r="C375" t="b">
         <v>1</v>
@@ -6272,10 +6272,10 @@
         <v>156</v>
       </c>
       <c r="B376" t="s">
-        <v>146</v>
+        <v>5</v>
       </c>
       <c r="C376" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D376" t="s">
         <v>6</v>
@@ -6286,13 +6286,13 @@
         <v>156</v>
       </c>
       <c r="B377" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C377" t="b">
         <v>0</v>
       </c>
       <c r="D377" t="s">
-        <v>157</v>
+        <v>6</v>
       </c>
     </row>
     <row r="378" spans="1:4" x14ac:dyDescent="0.25">
@@ -6300,35 +6300,35 @@
         <v>156</v>
       </c>
       <c r="B378" t="s">
-        <v>32</v>
+        <v>147</v>
       </c>
       <c r="C378" t="b">
         <v>0</v>
       </c>
       <c r="D378" t="s">
-        <v>33</v>
+        <v>157</v>
       </c>
     </row>
     <row r="379" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A379" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="B379" t="s">
-        <v>159</v>
+        <v>32</v>
       </c>
       <c r="C379" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D379" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
     </row>
     <row r="380" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A380" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="B380" t="s">
-        <v>5</v>
+        <v>159</v>
       </c>
       <c r="C380" t="b">
         <v>1</v>
@@ -6342,7 +6342,7 @@
         <v>160</v>
       </c>
       <c r="B381" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="C381" t="b">
         <v>1</v>
@@ -6356,13 +6356,13 @@
         <v>160</v>
       </c>
       <c r="B382" t="s">
-        <v>161</v>
+        <v>10</v>
       </c>
       <c r="C382" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D382" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="383" spans="1:4" x14ac:dyDescent="0.25">
@@ -6370,7 +6370,7 @@
         <v>160</v>
       </c>
       <c r="B383" t="s">
-        <v>31</v>
+        <v>161</v>
       </c>
       <c r="C383" t="b">
         <v>0</v>
@@ -6384,13 +6384,13 @@
         <v>160</v>
       </c>
       <c r="B384" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C384" t="b">
         <v>0</v>
       </c>
       <c r="D384" t="s">
-        <v>33</v>
+        <v>9</v>
       </c>
     </row>
     <row r="385" spans="1:4" x14ac:dyDescent="0.25">
@@ -6398,27 +6398,27 @@
         <v>160</v>
       </c>
       <c r="B385" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C385" t="b">
         <v>0</v>
       </c>
       <c r="D385" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="386" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A386" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="B386" t="s">
-        <v>13</v>
+        <v>34</v>
       </c>
       <c r="C386" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D386" t="s">
-        <v>6</v>
+        <v>35</v>
       </c>
     </row>
     <row r="387" spans="1:4" x14ac:dyDescent="0.25">
@@ -6426,7 +6426,7 @@
         <v>162</v>
       </c>
       <c r="B387" t="s">
-        <v>52</v>
+        <v>13</v>
       </c>
       <c r="C387" t="b">
         <v>1</v>
@@ -6440,7 +6440,7 @@
         <v>162</v>
       </c>
       <c r="B388" t="s">
-        <v>163</v>
+        <v>52</v>
       </c>
       <c r="C388" t="b">
         <v>1</v>
@@ -6454,10 +6454,10 @@
         <v>162</v>
       </c>
       <c r="B389" t="s">
-        <v>12</v>
+        <v>163</v>
       </c>
       <c r="C389" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D389" t="s">
         <v>6</v>
@@ -6468,7 +6468,7 @@
         <v>162</v>
       </c>
       <c r="B390" t="s">
-        <v>99</v>
+        <v>12</v>
       </c>
       <c r="C390" t="b">
         <v>0</v>
@@ -6479,13 +6479,13 @@
     </row>
     <row r="391" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A391" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="B391" t="s">
-        <v>10</v>
+        <v>99</v>
       </c>
       <c r="C391" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D391" t="s">
         <v>6</v>
@@ -6496,7 +6496,7 @@
         <v>164</v>
       </c>
       <c r="B392" t="s">
-        <v>99</v>
+        <v>10</v>
       </c>
       <c r="C392" t="b">
         <v>1</v>
@@ -6510,10 +6510,10 @@
         <v>164</v>
       </c>
       <c r="B393" t="s">
-        <v>12</v>
+        <v>99</v>
       </c>
       <c r="C393" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D393" t="s">
         <v>6</v>
@@ -6521,13 +6521,13 @@
     </row>
     <row r="394" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A394" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B394" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C394" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D394" t="s">
         <v>6</v>
@@ -6538,7 +6538,7 @@
         <v>165</v>
       </c>
       <c r="B395" t="s">
-        <v>99</v>
+        <v>10</v>
       </c>
       <c r="C395" t="b">
         <v>1</v>
@@ -6552,10 +6552,10 @@
         <v>165</v>
       </c>
       <c r="B396" t="s">
-        <v>12</v>
+        <v>99</v>
       </c>
       <c r="C396" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D396" t="s">
         <v>6</v>
@@ -6566,10 +6566,10 @@
         <v>165</v>
       </c>
       <c r="B397" t="s">
-        <v>98</v>
+        <v>12</v>
       </c>
       <c r="C397" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D397" t="s">
         <v>6</v>
@@ -6577,10 +6577,10 @@
     </row>
     <row r="398" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A398" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B398" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C398" t="b">
         <v>1</v>
@@ -6594,10 +6594,10 @@
         <v>166</v>
       </c>
       <c r="B399" t="s">
-        <v>115</v>
+        <v>97</v>
       </c>
       <c r="C399" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D399" t="s">
         <v>6</v>
@@ -6608,10 +6608,10 @@
         <v>166</v>
       </c>
       <c r="B400" t="s">
-        <v>99</v>
+        <v>115</v>
       </c>
       <c r="C400" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D400" t="s">
         <v>6</v>
@@ -6619,10 +6619,10 @@
     </row>
     <row r="401" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A401" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B401" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="C401" t="b">
         <v>1</v>
@@ -6636,10 +6636,10 @@
         <v>167</v>
       </c>
       <c r="B402" t="s">
-        <v>115</v>
+        <v>97</v>
       </c>
       <c r="C402" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D402" t="s">
         <v>6</v>
@@ -6650,10 +6650,10 @@
         <v>167</v>
       </c>
       <c r="B403" t="s">
-        <v>99</v>
+        <v>115</v>
       </c>
       <c r="C403" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D403" t="s">
         <v>6</v>
@@ -6661,10 +6661,10 @@
     </row>
     <row r="404" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A404" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="B404" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="C404" t="b">
         <v>1</v>
@@ -6678,10 +6678,10 @@
         <v>168</v>
       </c>
       <c r="B405" t="s">
-        <v>115</v>
+        <v>97</v>
       </c>
       <c r="C405" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D405" t="s">
         <v>6</v>
@@ -6692,10 +6692,10 @@
         <v>168</v>
       </c>
       <c r="B406" t="s">
-        <v>99</v>
+        <v>115</v>
       </c>
       <c r="C406" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D406" t="s">
         <v>6</v>
@@ -6703,13 +6703,13 @@
     </row>
     <row r="407" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A407" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B407" t="s">
-        <v>170</v>
+        <v>99</v>
       </c>
       <c r="C407" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D407" t="s">
         <v>6</v>
@@ -6720,7 +6720,7 @@
         <v>169</v>
       </c>
       <c r="B408" t="s">
-        <v>7</v>
+        <v>170</v>
       </c>
       <c r="C408" t="b">
         <v>0</v>
@@ -6734,13 +6734,13 @@
         <v>169</v>
       </c>
       <c r="B409" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C409" t="b">
         <v>0</v>
       </c>
       <c r="D409" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="410" spans="1:4" x14ac:dyDescent="0.25">
@@ -6748,13 +6748,13 @@
         <v>169</v>
       </c>
       <c r="B410" t="s">
-        <v>32</v>
+        <v>8</v>
       </c>
       <c r="C410" t="b">
         <v>0</v>
       </c>
       <c r="D410" t="s">
-        <v>33</v>
+        <v>9</v>
       </c>
     </row>
     <row r="411" spans="1:4" x14ac:dyDescent="0.25">
@@ -6762,13 +6762,13 @@
         <v>169</v>
       </c>
       <c r="B411" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C411" t="b">
         <v>0</v>
       </c>
       <c r="D411" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="412" spans="1:4" x14ac:dyDescent="0.25">
@@ -6776,27 +6776,27 @@
         <v>169</v>
       </c>
       <c r="B412" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="C412" t="b">
         <v>0</v>
       </c>
       <c r="D412" t="s">
-        <v>9</v>
+        <v>35</v>
       </c>
     </row>
     <row r="413" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A413" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="B413" t="s">
-        <v>172</v>
+        <v>31</v>
       </c>
       <c r="C413" t="b">
         <v>0</v>
       </c>
       <c r="D413" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="414" spans="1:4" x14ac:dyDescent="0.25">
@@ -6804,13 +6804,13 @@
         <v>171</v>
       </c>
       <c r="B414" t="s">
-        <v>8</v>
+        <v>172</v>
       </c>
       <c r="C414" t="b">
         <v>0</v>
       </c>
       <c r="D414" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="415" spans="1:4" x14ac:dyDescent="0.25">
@@ -6818,13 +6818,13 @@
         <v>171</v>
       </c>
       <c r="B415" t="s">
-        <v>32</v>
+        <v>8</v>
       </c>
       <c r="C415" t="b">
         <v>0</v>
       </c>
       <c r="D415" t="s">
-        <v>33</v>
+        <v>9</v>
       </c>
     </row>
     <row r="416" spans="1:4" x14ac:dyDescent="0.25">
@@ -6832,13 +6832,13 @@
         <v>171</v>
       </c>
       <c r="B416" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C416" t="b">
         <v>0</v>
       </c>
       <c r="D416" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="417" spans="1:4" x14ac:dyDescent="0.25">
@@ -6846,27 +6846,27 @@
         <v>171</v>
       </c>
       <c r="B417" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="C417" t="b">
         <v>0</v>
       </c>
       <c r="D417" t="s">
-        <v>9</v>
+        <v>35</v>
       </c>
     </row>
     <row r="418" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A418" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="B418" t="s">
-        <v>13</v>
+        <v>31</v>
       </c>
       <c r="C418" t="b">
         <v>0</v>
       </c>
       <c r="D418" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="419" spans="1:4" x14ac:dyDescent="0.25">
@@ -6874,7 +6874,7 @@
         <v>173</v>
       </c>
       <c r="B419" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="C419" t="b">
         <v>0</v>
@@ -6888,13 +6888,13 @@
         <v>173</v>
       </c>
       <c r="B420" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C420" t="b">
         <v>0</v>
       </c>
       <c r="D420" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="421" spans="1:4" x14ac:dyDescent="0.25">
@@ -6902,13 +6902,13 @@
         <v>173</v>
       </c>
       <c r="B421" t="s">
-        <v>32</v>
+        <v>8</v>
       </c>
       <c r="C421" t="b">
         <v>0</v>
       </c>
       <c r="D421" t="s">
-        <v>33</v>
+        <v>9</v>
       </c>
     </row>
     <row r="422" spans="1:4" x14ac:dyDescent="0.25">
@@ -6916,13 +6916,13 @@
         <v>173</v>
       </c>
       <c r="B422" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C422" t="b">
         <v>0</v>
       </c>
       <c r="D422" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="423" spans="1:4" x14ac:dyDescent="0.25">
@@ -6930,27 +6930,27 @@
         <v>173</v>
       </c>
       <c r="B423" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="C423" t="b">
         <v>0</v>
       </c>
       <c r="D423" t="s">
-        <v>9</v>
+        <v>35</v>
       </c>
     </row>
     <row r="424" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A424" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="B424" t="s">
-        <v>97</v>
+        <v>31</v>
       </c>
       <c r="C424" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D424" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="425" spans="1:4" x14ac:dyDescent="0.25">
@@ -6958,10 +6958,10 @@
         <v>174</v>
       </c>
       <c r="B425" t="s">
-        <v>115</v>
+        <v>97</v>
       </c>
       <c r="C425" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D425" t="s">
         <v>6</v>
@@ -6972,7 +6972,7 @@
         <v>174</v>
       </c>
       <c r="B426" t="s">
-        <v>175</v>
+        <v>115</v>
       </c>
       <c r="C426" t="b">
         <v>0</v>
@@ -6983,13 +6983,13 @@
     </row>
     <row r="427" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A427" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="B427" t="s">
-        <v>97</v>
+        <v>175</v>
       </c>
       <c r="C427" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D427" t="s">
         <v>6</v>
@@ -7000,10 +7000,10 @@
         <v>176</v>
       </c>
       <c r="B428" t="s">
-        <v>115</v>
+        <v>97</v>
       </c>
       <c r="C428" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D428" t="s">
         <v>6</v>
@@ -7014,7 +7014,7 @@
         <v>176</v>
       </c>
       <c r="B429" t="s">
-        <v>175</v>
+        <v>115</v>
       </c>
       <c r="C429" t="b">
         <v>0</v>
@@ -7028,7 +7028,7 @@
         <v>176</v>
       </c>
       <c r="B430" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="C430" t="b">
         <v>0</v>
@@ -7039,13 +7039,13 @@
     </row>
     <row r="431" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A431" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="B431" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="C431" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D431" t="s">
         <v>6</v>
@@ -7056,7 +7056,7 @@
         <v>178</v>
       </c>
       <c r="B432" t="s">
-        <v>10</v>
+        <v>179</v>
       </c>
       <c r="C432" t="b">
         <v>1</v>
@@ -7070,10 +7070,10 @@
         <v>178</v>
       </c>
       <c r="B433" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C433" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D433" t="s">
         <v>6</v>
@@ -7084,13 +7084,13 @@
         <v>178</v>
       </c>
       <c r="B434" t="s">
-        <v>32</v>
+        <v>12</v>
       </c>
       <c r="C434" t="b">
         <v>0</v>
       </c>
       <c r="D434" t="s">
-        <v>33</v>
+        <v>6</v>
       </c>
     </row>
     <row r="435" spans="1:4" x14ac:dyDescent="0.25">
@@ -7098,13 +7098,13 @@
         <v>178</v>
       </c>
       <c r="B435" t="s">
-        <v>8</v>
+        <v>32</v>
       </c>
       <c r="C435" t="b">
         <v>0</v>
       </c>
       <c r="D435" t="s">
-        <v>9</v>
+        <v>33</v>
       </c>
     </row>
     <row r="436" spans="1:4" x14ac:dyDescent="0.25">
@@ -7112,7 +7112,7 @@
         <v>178</v>
       </c>
       <c r="B436" t="s">
-        <v>180</v>
+        <v>8</v>
       </c>
       <c r="C436" t="b">
         <v>0</v>
@@ -7126,24 +7126,24 @@
         <v>178</v>
       </c>
       <c r="B437" t="s">
-        <v>38</v>
+        <v>180</v>
       </c>
       <c r="C437" t="b">
         <v>0</v>
       </c>
       <c r="D437" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="438" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A438" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="B438" t="s">
-        <v>182</v>
+        <v>38</v>
       </c>
       <c r="C438" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D438" t="s">
         <v>6</v>
@@ -7154,7 +7154,7 @@
         <v>181</v>
       </c>
       <c r="B439" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="C439" t="b">
         <v>1</v>
@@ -7168,7 +7168,7 @@
         <v>181</v>
       </c>
       <c r="B440" t="s">
-        <v>10</v>
+        <v>179</v>
       </c>
       <c r="C440" t="b">
         <v>1</v>
@@ -7182,10 +7182,10 @@
         <v>181</v>
       </c>
       <c r="B441" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C441" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D441" t="s">
         <v>6</v>
@@ -7196,13 +7196,13 @@
         <v>181</v>
       </c>
       <c r="B442" t="s">
-        <v>32</v>
+        <v>12</v>
       </c>
       <c r="C442" t="b">
         <v>0</v>
       </c>
       <c r="D442" t="s">
-        <v>33</v>
+        <v>6</v>
       </c>
     </row>
     <row r="443" spans="1:4" x14ac:dyDescent="0.25">
@@ -7210,13 +7210,13 @@
         <v>181</v>
       </c>
       <c r="B443" t="s">
-        <v>8</v>
+        <v>32</v>
       </c>
       <c r="C443" t="b">
         <v>0</v>
       </c>
       <c r="D443" t="s">
-        <v>9</v>
+        <v>33</v>
       </c>
     </row>
     <row r="444" spans="1:4" x14ac:dyDescent="0.25">
@@ -7224,7 +7224,7 @@
         <v>181</v>
       </c>
       <c r="B444" t="s">
-        <v>46</v>
+        <v>8</v>
       </c>
       <c r="C444" t="b">
         <v>0</v>
@@ -7238,24 +7238,24 @@
         <v>181</v>
       </c>
       <c r="B445" t="s">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="C445" t="b">
         <v>0</v>
       </c>
       <c r="D445" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="446" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A446" t="s">
-        <v>84</v>
+        <v>181</v>
       </c>
       <c r="B446" t="s">
-        <v>183</v>
+        <v>38</v>
       </c>
       <c r="C446" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D446" t="s">
         <v>6</v>
@@ -7266,10 +7266,10 @@
         <v>84</v>
       </c>
       <c r="B447" t="s">
-        <v>12</v>
+        <v>183</v>
       </c>
       <c r="C447" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D447" t="s">
         <v>6</v>
@@ -7277,16 +7277,16 @@
     </row>
     <row r="448" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A448" t="s">
-        <v>184</v>
+        <v>84</v>
       </c>
       <c r="B448" t="s">
-        <v>185</v>
+        <v>12</v>
       </c>
       <c r="C448" t="b">
         <v>0</v>
       </c>
       <c r="D448" t="s">
-        <v>186</v>
+        <v>6</v>
       </c>
     </row>
     <row r="449" spans="1:4" x14ac:dyDescent="0.25">
@@ -7294,27 +7294,27 @@
         <v>184</v>
       </c>
       <c r="B449" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="C449" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D449" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
     </row>
     <row r="450" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A450" t="s">
-        <v>189</v>
+        <v>184</v>
       </c>
       <c r="B450" t="s">
-        <v>5</v>
+        <v>187</v>
       </c>
       <c r="C450" t="b">
         <v>1</v>
       </c>
       <c r="D450" t="s">
-        <v>6</v>
+        <v>188</v>
       </c>
     </row>
     <row r="451" spans="1:4" x14ac:dyDescent="0.25">
@@ -7322,7 +7322,7 @@
         <v>189</v>
       </c>
       <c r="B451" t="s">
-        <v>190</v>
+        <v>5</v>
       </c>
       <c r="C451" t="b">
         <v>1</v>
@@ -7333,10 +7333,10 @@
     </row>
     <row r="452" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A452" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="B452" t="s">
-        <v>5</v>
+        <v>190</v>
       </c>
       <c r="C452" t="b">
         <v>1</v>
@@ -7350,7 +7350,7 @@
         <v>191</v>
       </c>
       <c r="B453" t="s">
-        <v>190</v>
+        <v>5</v>
       </c>
       <c r="C453" t="b">
         <v>1</v>
@@ -7361,10 +7361,10 @@
     </row>
     <row r="454" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A454" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B454" t="s">
-        <v>97</v>
+        <v>190</v>
       </c>
       <c r="C454" t="b">
         <v>1</v>
@@ -7378,7 +7378,7 @@
         <v>192</v>
       </c>
       <c r="B455" t="s">
-        <v>193</v>
+        <v>97</v>
       </c>
       <c r="C455" t="b">
         <v>1</v>
@@ -7389,10 +7389,10 @@
     </row>
     <row r="456" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A456" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="B456" t="s">
-        <v>97</v>
+        <v>193</v>
       </c>
       <c r="C456" t="b">
         <v>1</v>
@@ -7406,7 +7406,7 @@
         <v>194</v>
       </c>
       <c r="B457" t="s">
-        <v>195</v>
+        <v>97</v>
       </c>
       <c r="C457" t="b">
         <v>1</v>
@@ -7417,10 +7417,10 @@
     </row>
     <row r="458" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A458" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="B458" t="s">
-        <v>5</v>
+        <v>195</v>
       </c>
       <c r="C458" t="b">
         <v>1</v>
@@ -7431,7 +7431,7 @@
     </row>
     <row r="459" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A459" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B459" t="s">
         <v>5</v>
@@ -7445,10 +7445,10 @@
     </row>
     <row r="460" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A460" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B460" t="s">
-        <v>199</v>
+        <v>5</v>
       </c>
       <c r="C460" t="b">
         <v>1</v>
@@ -7459,10 +7459,10 @@
     </row>
     <row r="461" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A461" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="B461" t="s">
-        <v>5</v>
+        <v>199</v>
       </c>
       <c r="C461" t="b">
         <v>1</v>
@@ -7476,10 +7476,10 @@
         <v>200</v>
       </c>
       <c r="B462" t="s">
-        <v>201</v>
+        <v>5</v>
       </c>
       <c r="C462" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D462" t="s">
         <v>6</v>
@@ -7487,13 +7487,13 @@
     </row>
     <row r="463" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A463" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="B463" t="s">
-        <v>5</v>
+        <v>201</v>
       </c>
       <c r="C463" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D463" t="s">
         <v>6</v>
@@ -7504,10 +7504,10 @@
         <v>202</v>
       </c>
       <c r="B464" t="s">
-        <v>201</v>
+        <v>5</v>
       </c>
       <c r="C464" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D464" t="s">
         <v>6</v>
@@ -7515,13 +7515,13 @@
     </row>
     <row r="465" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A465" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="B465" t="s">
-        <v>5</v>
+        <v>201</v>
       </c>
       <c r="C465" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D465" t="s">
         <v>6</v>
@@ -7532,10 +7532,10 @@
         <v>203</v>
       </c>
       <c r="B466" t="s">
-        <v>201</v>
+        <v>5</v>
       </c>
       <c r="C466" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D466" t="s">
         <v>6</v>
@@ -7543,13 +7543,13 @@
     </row>
     <row r="467" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A467" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B467" t="s">
-        <v>5</v>
+        <v>201</v>
       </c>
       <c r="C467" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D467" t="s">
         <v>6</v>
@@ -7560,10 +7560,10 @@
         <v>204</v>
       </c>
       <c r="B468" t="s">
-        <v>201</v>
+        <v>5</v>
       </c>
       <c r="C468" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D468" t="s">
         <v>6</v>
@@ -7571,13 +7571,13 @@
     </row>
     <row r="469" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A469" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="B469" t="s">
-        <v>5</v>
+        <v>201</v>
       </c>
       <c r="C469" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D469" t="s">
         <v>6</v>
@@ -7585,13 +7585,13 @@
     </row>
     <row r="470" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A470" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="B470" t="s">
         <v>5</v>
       </c>
       <c r="C470" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D470" t="s">
         <v>6</v>
@@ -7602,7 +7602,7 @@
         <v>206</v>
       </c>
       <c r="B471" t="s">
-        <v>182</v>
+        <v>5</v>
       </c>
       <c r="C471" t="b">
         <v>0</v>
@@ -7616,7 +7616,7 @@
         <v>206</v>
       </c>
       <c r="B472" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="C472" t="b">
         <v>0</v>
@@ -7630,10 +7630,10 @@
         <v>206</v>
       </c>
       <c r="B473" t="s">
-        <v>207</v>
+        <v>179</v>
       </c>
       <c r="C473" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D473" t="s">
         <v>6</v>
@@ -7644,10 +7644,10 @@
         <v>206</v>
       </c>
       <c r="B474" t="s">
-        <v>12</v>
+        <v>207</v>
       </c>
       <c r="C474" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D474" t="s">
         <v>6</v>
@@ -7655,13 +7655,13 @@
     </row>
     <row r="475" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A475" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="B475" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="C475" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D475" t="s">
         <v>6</v>
@@ -7672,10 +7672,10 @@
         <v>208</v>
       </c>
       <c r="B476" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C476" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D476" t="s">
         <v>6</v>
@@ -7686,13 +7686,13 @@
         <v>208</v>
       </c>
       <c r="B477" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C477" t="b">
         <v>0</v>
       </c>
       <c r="D477" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="478" spans="1:4" x14ac:dyDescent="0.25">
@@ -7700,13 +7700,13 @@
         <v>208</v>
       </c>
       <c r="B478" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C478" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D478" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="479" spans="1:4" x14ac:dyDescent="0.25">
@@ -7714,10 +7714,10 @@
         <v>208</v>
       </c>
       <c r="B479" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C479" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D479" t="s">
         <v>6</v>
@@ -7728,10 +7728,10 @@
         <v>208</v>
       </c>
       <c r="B480" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C480" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D480" t="s">
         <v>6</v>
@@ -7742,7 +7742,7 @@
         <v>208</v>
       </c>
       <c r="B481" t="s">
-        <v>45</v>
+        <v>12</v>
       </c>
       <c r="C481" t="b">
         <v>1</v>
@@ -7756,13 +7756,13 @@
         <v>208</v>
       </c>
       <c r="B482" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C482" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D482" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="483" spans="1:4" x14ac:dyDescent="0.25">
@@ -7770,13 +7770,13 @@
         <v>208</v>
       </c>
       <c r="B483" t="s">
-        <v>13</v>
+        <v>46</v>
       </c>
       <c r="C483" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D483" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="484" spans="1:4" x14ac:dyDescent="0.25">
@@ -7784,10 +7784,10 @@
         <v>208</v>
       </c>
       <c r="B484" t="s">
-        <v>37</v>
+        <v>13</v>
       </c>
       <c r="C484" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D484" t="s">
         <v>6</v>
@@ -7798,10 +7798,10 @@
         <v>208</v>
       </c>
       <c r="B485" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C485" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D485" t="s">
         <v>6</v>
@@ -7812,7 +7812,7 @@
         <v>208</v>
       </c>
       <c r="B486" t="s">
-        <v>52</v>
+        <v>38</v>
       </c>
       <c r="C486" t="b">
         <v>1</v>
@@ -7826,13 +7826,13 @@
         <v>208</v>
       </c>
       <c r="B487" t="s">
-        <v>19</v>
+        <v>52</v>
       </c>
       <c r="C487" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D487" t="s">
-        <v>20</v>
+        <v>6</v>
       </c>
     </row>
     <row r="488" spans="1:4" x14ac:dyDescent="0.25">
@@ -7840,13 +7840,13 @@
         <v>208</v>
       </c>
       <c r="B488" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="C488" t="b">
         <v>0</v>
       </c>
       <c r="D488" t="s">
-        <v>9</v>
+        <v>20</v>
       </c>
     </row>
     <row r="489" spans="1:4" x14ac:dyDescent="0.25">
@@ -7854,13 +7854,13 @@
         <v>208</v>
       </c>
       <c r="B489" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C489" t="b">
         <v>0</v>
       </c>
       <c r="D489" t="s">
-        <v>33</v>
+        <v>9</v>
       </c>
     </row>
     <row r="490" spans="1:4" x14ac:dyDescent="0.25">
@@ -7868,12 +7868,26 @@
         <v>208</v>
       </c>
       <c r="B490" t="s">
+        <v>32</v>
+      </c>
+      <c r="C490" t="b">
+        <v>0</v>
+      </c>
+      <c r="D490" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="491" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A491" t="s">
+        <v>208</v>
+      </c>
+      <c r="B491" t="s">
         <v>34</v>
       </c>
-      <c r="C490" t="b">
-        <v>0</v>
-      </c>
-      <c r="D490" t="s">
+      <c r="C491" t="b">
+        <v>0</v>
+      </c>
+      <c r="D491" t="s">
         <v>35</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Deploying to gh-pages from @ open-resource-discovery/specification@31fd1b8ef7226cea93c083cfa4a6d2f00e0c5a77 🚀
</commit_message>
<xml_diff>
--- a/spec-v1/interfaces/Document.xlsx
+++ b/spec-v1/interfaces/Document.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1474" uniqueCount="209">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1483" uniqueCount="212">
   <si>
     <t>Entity Name</t>
   </si>
@@ -448,6 +448,12 @@
     <t>array&lt;CapabilityIntegrationAspect&gt;</t>
   </si>
   <si>
+    <t>systemTypes</t>
+  </si>
+  <si>
+    <t>array&lt;SystemTypeIntegrationAspect&gt;</t>
+  </si>
+  <si>
     <t>Api Resource Integration Aspect</t>
   </si>
   <si>
@@ -487,6 +493,12 @@
     <t>array&lt;CapabilityIntegrationAspectSubset&gt;</t>
   </si>
   <si>
+    <t>System Type Integration Aspect</t>
+  </si>
+  <si>
+    <t>systemNamespace</t>
+  </si>
+  <si>
     <t>Capability Integration Aspect Subset</t>
   </si>
   <si>
@@ -527,9 +539,6 @@
   </si>
   <si>
     <t>System Type</t>
-  </si>
-  <si>
-    <t>systemNamespace</t>
   </si>
   <si>
     <t>System Version</t>
@@ -1014,7 +1023,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D491"/>
+  <dimension ref="A1:D494"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6104,38 +6113,38 @@
         <v>137</v>
       </c>
       <c r="B364" t="s">
-        <v>32</v>
+        <v>145</v>
       </c>
       <c r="C364" t="b">
         <v>0</v>
       </c>
       <c r="D364" t="s">
-        <v>33</v>
+        <v>146</v>
       </c>
     </row>
     <row r="365" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A365" t="s">
-        <v>145</v>
+        <v>137</v>
       </c>
       <c r="B365" t="s">
-        <v>5</v>
+        <v>32</v>
       </c>
       <c r="C365" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D365" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
     </row>
     <row r="366" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A366" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="B366" t="s">
-        <v>146</v>
+        <v>5</v>
       </c>
       <c r="C366" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D366" t="s">
         <v>6</v>
@@ -6143,55 +6152,55 @@
     </row>
     <row r="367" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A367" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="B367" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C367" t="b">
         <v>0</v>
       </c>
       <c r="D367" t="s">
-        <v>148</v>
+        <v>6</v>
       </c>
     </row>
     <row r="368" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A368" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="B368" t="s">
-        <v>32</v>
+        <v>149</v>
       </c>
       <c r="C368" t="b">
         <v>0</v>
       </c>
       <c r="D368" t="s">
-        <v>33</v>
+        <v>150</v>
       </c>
     </row>
     <row r="369" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A369" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="B369" t="s">
-        <v>5</v>
+        <v>32</v>
       </c>
       <c r="C369" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D369" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
     </row>
     <row r="370" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A370" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="B370" t="s">
-        <v>146</v>
+        <v>5</v>
       </c>
       <c r="C370" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D370" t="s">
         <v>6</v>
@@ -6199,58 +6208,58 @@
     </row>
     <row r="371" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A371" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="B371" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C371" t="b">
         <v>0</v>
       </c>
       <c r="D371" t="s">
-        <v>150</v>
+        <v>6</v>
       </c>
     </row>
     <row r="372" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A372" t="s">
+        <v>151</v>
+      </c>
+      <c r="B372" t="s">
         <v>149</v>
       </c>
-      <c r="B372" t="s">
-        <v>151</v>
-      </c>
       <c r="C372" t="b">
         <v>0</v>
       </c>
       <c r="D372" t="s">
-        <v>9</v>
+        <v>152</v>
       </c>
     </row>
     <row r="373" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A373" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="B373" t="s">
-        <v>32</v>
+        <v>153</v>
       </c>
       <c r="C373" t="b">
         <v>0</v>
       </c>
       <c r="D373" t="s">
-        <v>33</v>
+        <v>9</v>
       </c>
     </row>
     <row r="374" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A374" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B374" t="s">
-        <v>153</v>
+        <v>32</v>
       </c>
       <c r="C374" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D374" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
     </row>
     <row r="375" spans="1:4" x14ac:dyDescent="0.25">
@@ -6272,7 +6281,7 @@
         <v>156</v>
       </c>
       <c r="B376" t="s">
-        <v>5</v>
+        <v>157</v>
       </c>
       <c r="C376" t="b">
         <v>1</v>
@@ -6283,13 +6292,13 @@
     </row>
     <row r="377" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A377" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="B377" t="s">
-        <v>146</v>
+        <v>5</v>
       </c>
       <c r="C377" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D377" t="s">
         <v>6</v>
@@ -6297,30 +6306,30 @@
     </row>
     <row r="378" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A378" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="B378" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C378" t="b">
         <v>0</v>
       </c>
       <c r="D378" t="s">
-        <v>157</v>
+        <v>6</v>
       </c>
     </row>
     <row r="379" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A379" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="B379" t="s">
-        <v>32</v>
+        <v>149</v>
       </c>
       <c r="C379" t="b">
         <v>0</v>
       </c>
       <c r="D379" t="s">
-        <v>33</v>
+        <v>159</v>
       </c>
     </row>
     <row r="380" spans="1:4" x14ac:dyDescent="0.25">
@@ -6328,13 +6337,13 @@
         <v>158</v>
       </c>
       <c r="B380" t="s">
-        <v>159</v>
+        <v>32</v>
       </c>
       <c r="C380" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D380" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
     </row>
     <row r="381" spans="1:4" x14ac:dyDescent="0.25">
@@ -6342,7 +6351,7 @@
         <v>160</v>
       </c>
       <c r="B381" t="s">
-        <v>5</v>
+        <v>161</v>
       </c>
       <c r="C381" t="b">
         <v>1</v>
@@ -6356,10 +6365,10 @@
         <v>160</v>
       </c>
       <c r="B382" t="s">
-        <v>10</v>
+        <v>54</v>
       </c>
       <c r="C382" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D382" t="s">
         <v>6</v>
@@ -6367,111 +6376,111 @@
     </row>
     <row r="383" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A383" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="B383" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="C383" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D383" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="384" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A384" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
       <c r="B384" t="s">
-        <v>31</v>
+        <v>5</v>
       </c>
       <c r="C384" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D384" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="385" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A385" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
       <c r="B385" t="s">
-        <v>32</v>
+        <v>10</v>
       </c>
       <c r="C385" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D385" t="s">
-        <v>33</v>
+        <v>6</v>
       </c>
     </row>
     <row r="386" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A386" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
       <c r="B386" t="s">
-        <v>34</v>
+        <v>165</v>
       </c>
       <c r="C386" t="b">
         <v>0</v>
       </c>
       <c r="D386" t="s">
-        <v>35</v>
+        <v>9</v>
       </c>
     </row>
     <row r="387" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A387" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B387" t="s">
-        <v>13</v>
+        <v>31</v>
       </c>
       <c r="C387" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D387" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="388" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A388" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B388" t="s">
-        <v>52</v>
+        <v>32</v>
       </c>
       <c r="C388" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D388" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
     </row>
     <row r="389" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A389" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B389" t="s">
-        <v>163</v>
+        <v>34</v>
       </c>
       <c r="C389" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D389" t="s">
-        <v>6</v>
+        <v>35</v>
       </c>
     </row>
     <row r="390" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A390" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="B390" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C390" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D390" t="s">
         <v>6</v>
@@ -6479,13 +6488,13 @@
     </row>
     <row r="391" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A391" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="B391" t="s">
-        <v>99</v>
+        <v>52</v>
       </c>
       <c r="C391" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D391" t="s">
         <v>6</v>
@@ -6493,10 +6502,10 @@
     </row>
     <row r="392" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A392" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B392" t="s">
-        <v>10</v>
+        <v>167</v>
       </c>
       <c r="C392" t="b">
         <v>1</v>
@@ -6507,13 +6516,13 @@
     </row>
     <row r="393" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A393" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B393" t="s">
-        <v>99</v>
+        <v>12</v>
       </c>
       <c r="C393" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D393" t="s">
         <v>6</v>
@@ -6521,10 +6530,10 @@
     </row>
     <row r="394" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A394" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B394" t="s">
-        <v>12</v>
+        <v>99</v>
       </c>
       <c r="C394" t="b">
         <v>0</v>
@@ -6535,7 +6544,7 @@
     </row>
     <row r="395" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A395" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="B395" t="s">
         <v>10</v>
@@ -6549,7 +6558,7 @@
     </row>
     <row r="396" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A396" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="B396" t="s">
         <v>99</v>
@@ -6563,7 +6572,7 @@
     </row>
     <row r="397" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A397" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="B397" t="s">
         <v>12</v>
@@ -6577,10 +6586,10 @@
     </row>
     <row r="398" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A398" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="B398" t="s">
-        <v>98</v>
+        <v>10</v>
       </c>
       <c r="C398" t="b">
         <v>1</v>
@@ -6591,10 +6600,10 @@
     </row>
     <row r="399" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A399" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="B399" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="C399" t="b">
         <v>1</v>
@@ -6605,10 +6614,10 @@
     </row>
     <row r="400" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A400" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="B400" t="s">
-        <v>115</v>
+        <v>12</v>
       </c>
       <c r="C400" t="b">
         <v>0</v>
@@ -6619,10 +6628,10 @@
     </row>
     <row r="401" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A401" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="B401" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C401" t="b">
         <v>1</v>
@@ -6633,7 +6642,7 @@
     </row>
     <row r="402" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A402" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="B402" t="s">
         <v>97</v>
@@ -6647,7 +6656,7 @@
     </row>
     <row r="403" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A403" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="B403" t="s">
         <v>115</v>
@@ -6661,7 +6670,7 @@
     </row>
     <row r="404" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A404" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="B404" t="s">
         <v>99</v>
@@ -6675,7 +6684,7 @@
     </row>
     <row r="405" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A405" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="B405" t="s">
         <v>97</v>
@@ -6689,7 +6698,7 @@
     </row>
     <row r="406" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A406" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="B406" t="s">
         <v>115</v>
@@ -6703,7 +6712,7 @@
     </row>
     <row r="407" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A407" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="B407" t="s">
         <v>99</v>
@@ -6717,13 +6726,13 @@
     </row>
     <row r="408" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A408" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="B408" t="s">
-        <v>170</v>
+        <v>97</v>
       </c>
       <c r="C408" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D408" t="s">
         <v>6</v>
@@ -6731,10 +6740,10 @@
     </row>
     <row r="409" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A409" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="B409" t="s">
-        <v>7</v>
+        <v>115</v>
       </c>
       <c r="C409" t="b">
         <v>0</v>
@@ -6745,52 +6754,52 @@
     </row>
     <row r="410" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A410" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="B410" t="s">
-        <v>8</v>
+        <v>99</v>
       </c>
       <c r="C410" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D410" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="411" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A411" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="B411" t="s">
-        <v>32</v>
+        <v>174</v>
       </c>
       <c r="C411" t="b">
         <v>0</v>
       </c>
       <c r="D411" t="s">
-        <v>33</v>
+        <v>6</v>
       </c>
     </row>
     <row r="412" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A412" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="B412" t="s">
-        <v>34</v>
+        <v>7</v>
       </c>
       <c r="C412" t="b">
         <v>0</v>
       </c>
       <c r="D412" t="s">
-        <v>35</v>
+        <v>6</v>
       </c>
     </row>
     <row r="413" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A413" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="B413" t="s">
-        <v>31</v>
+        <v>8</v>
       </c>
       <c r="C413" t="b">
         <v>0</v>
@@ -6801,66 +6810,66 @@
     </row>
     <row r="414" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A414" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="B414" t="s">
-        <v>172</v>
+        <v>32</v>
       </c>
       <c r="C414" t="b">
         <v>0</v>
       </c>
       <c r="D414" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
     </row>
     <row r="415" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A415" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="B415" t="s">
-        <v>8</v>
+        <v>34</v>
       </c>
       <c r="C415" t="b">
         <v>0</v>
       </c>
       <c r="D415" t="s">
-        <v>9</v>
+        <v>35</v>
       </c>
     </row>
     <row r="416" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A416" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="B416" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C416" t="b">
         <v>0</v>
       </c>
       <c r="D416" t="s">
-        <v>33</v>
+        <v>9</v>
       </c>
     </row>
     <row r="417" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A417" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="B417" t="s">
-        <v>34</v>
+        <v>161</v>
       </c>
       <c r="C417" t="b">
         <v>0</v>
       </c>
       <c r="D417" t="s">
-        <v>35</v>
+        <v>6</v>
       </c>
     </row>
     <row r="418" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A418" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="B418" t="s">
-        <v>31</v>
+        <v>8</v>
       </c>
       <c r="C418" t="b">
         <v>0</v>
@@ -6871,38 +6880,38 @@
     </row>
     <row r="419" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A419" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="B419" t="s">
-        <v>13</v>
+        <v>32</v>
       </c>
       <c r="C419" t="b">
         <v>0</v>
       </c>
       <c r="D419" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
     </row>
     <row r="420" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A420" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="B420" t="s">
-        <v>10</v>
+        <v>34</v>
       </c>
       <c r="C420" t="b">
         <v>0</v>
       </c>
       <c r="D420" t="s">
-        <v>6</v>
+        <v>35</v>
       </c>
     </row>
     <row r="421" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A421" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="B421" t="s">
-        <v>8</v>
+        <v>31</v>
       </c>
       <c r="C421" t="b">
         <v>0</v>
@@ -6913,38 +6922,38 @@
     </row>
     <row r="422" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A422" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="B422" t="s">
-        <v>32</v>
+        <v>13</v>
       </c>
       <c r="C422" t="b">
         <v>0</v>
       </c>
       <c r="D422" t="s">
-        <v>33</v>
+        <v>6</v>
       </c>
     </row>
     <row r="423" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A423" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="B423" t="s">
-        <v>34</v>
+        <v>10</v>
       </c>
       <c r="C423" t="b">
         <v>0</v>
       </c>
       <c r="D423" t="s">
-        <v>35</v>
+        <v>6</v>
       </c>
     </row>
     <row r="424" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A424" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="B424" t="s">
-        <v>31</v>
+        <v>8</v>
       </c>
       <c r="C424" t="b">
         <v>0</v>
@@ -6955,49 +6964,49 @@
     </row>
     <row r="425" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A425" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="B425" t="s">
-        <v>97</v>
+        <v>32</v>
       </c>
       <c r="C425" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D425" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
     </row>
     <row r="426" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A426" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="B426" t="s">
-        <v>115</v>
+        <v>34</v>
       </c>
       <c r="C426" t="b">
         <v>0</v>
       </c>
       <c r="D426" t="s">
-        <v>6</v>
+        <v>35</v>
       </c>
     </row>
     <row r="427" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A427" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="B427" t="s">
-        <v>175</v>
+        <v>31</v>
       </c>
       <c r="C427" t="b">
         <v>0</v>
       </c>
       <c r="D427" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="428" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A428" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B428" t="s">
         <v>97</v>
@@ -7011,7 +7020,7 @@
     </row>
     <row r="429" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A429" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B429" t="s">
         <v>115</v>
@@ -7025,10 +7034,10 @@
     </row>
     <row r="430" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A430" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B430" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="C430" t="b">
         <v>0</v>
@@ -7039,13 +7048,13 @@
     </row>
     <row r="431" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A431" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="B431" t="s">
-        <v>177</v>
+        <v>97</v>
       </c>
       <c r="C431" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D431" t="s">
         <v>6</v>
@@ -7053,13 +7062,13 @@
     </row>
     <row r="432" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A432" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B432" t="s">
-        <v>179</v>
+        <v>115</v>
       </c>
       <c r="C432" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D432" t="s">
         <v>6</v>
@@ -7067,13 +7076,13 @@
     </row>
     <row r="433" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A433" t="s">
+        <v>179</v>
+      </c>
+      <c r="B433" t="s">
         <v>178</v>
       </c>
-      <c r="B433" t="s">
-        <v>10</v>
-      </c>
       <c r="C433" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D433" t="s">
         <v>6</v>
@@ -7081,10 +7090,10 @@
     </row>
     <row r="434" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A434" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B434" t="s">
-        <v>12</v>
+        <v>180</v>
       </c>
       <c r="C434" t="b">
         <v>0</v>
@@ -7095,58 +7104,58 @@
     </row>
     <row r="435" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A435" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="B435" t="s">
-        <v>32</v>
+        <v>182</v>
       </c>
       <c r="C435" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D435" t="s">
-        <v>33</v>
+        <v>6</v>
       </c>
     </row>
     <row r="436" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A436" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="B436" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C436" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D436" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="437" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A437" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="B437" t="s">
-        <v>180</v>
+        <v>12</v>
       </c>
       <c r="C437" t="b">
         <v>0</v>
       </c>
       <c r="D437" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="438" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A438" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="B438" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="C438" t="b">
         <v>0</v>
       </c>
       <c r="D438" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
     </row>
     <row r="439" spans="1:4" x14ac:dyDescent="0.25">
@@ -7154,13 +7163,13 @@
         <v>181</v>
       </c>
       <c r="B439" t="s">
-        <v>182</v>
+        <v>8</v>
       </c>
       <c r="C439" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D439" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="440" spans="1:4" x14ac:dyDescent="0.25">
@@ -7168,13 +7177,13 @@
         <v>181</v>
       </c>
       <c r="B440" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
       <c r="C440" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D440" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="441" spans="1:4" x14ac:dyDescent="0.25">
@@ -7182,10 +7191,10 @@
         <v>181</v>
       </c>
       <c r="B441" t="s">
-        <v>10</v>
+        <v>38</v>
       </c>
       <c r="C441" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D441" t="s">
         <v>6</v>
@@ -7193,13 +7202,13 @@
     </row>
     <row r="442" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A442" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="B442" t="s">
-        <v>12</v>
+        <v>185</v>
       </c>
       <c r="C442" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D442" t="s">
         <v>6</v>
@@ -7207,86 +7216,86 @@
     </row>
     <row r="443" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A443" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="B443" t="s">
-        <v>32</v>
+        <v>182</v>
       </c>
       <c r="C443" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D443" t="s">
-        <v>33</v>
+        <v>6</v>
       </c>
     </row>
     <row r="444" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A444" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="B444" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C444" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D444" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="445" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A445" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="B445" t="s">
-        <v>46</v>
+        <v>12</v>
       </c>
       <c r="C445" t="b">
         <v>0</v>
       </c>
       <c r="D445" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="446" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A446" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="B446" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="C446" t="b">
         <v>0</v>
       </c>
       <c r="D446" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
     </row>
     <row r="447" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A447" t="s">
-        <v>84</v>
+        <v>184</v>
       </c>
       <c r="B447" t="s">
-        <v>183</v>
+        <v>8</v>
       </c>
       <c r="C447" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D447" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="448" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A448" t="s">
-        <v>84</v>
+        <v>184</v>
       </c>
       <c r="B448" t="s">
-        <v>12</v>
+        <v>46</v>
       </c>
       <c r="C448" t="b">
         <v>0</v>
       </c>
       <c r="D448" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="449" spans="1:4" x14ac:dyDescent="0.25">
@@ -7294,38 +7303,38 @@
         <v>184</v>
       </c>
       <c r="B449" t="s">
-        <v>185</v>
+        <v>38</v>
       </c>
       <c r="C449" t="b">
         <v>0</v>
       </c>
       <c r="D449" t="s">
-        <v>186</v>
+        <v>6</v>
       </c>
     </row>
     <row r="450" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A450" t="s">
-        <v>184</v>
+        <v>84</v>
       </c>
       <c r="B450" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="C450" t="b">
         <v>1</v>
       </c>
       <c r="D450" t="s">
-        <v>188</v>
+        <v>6</v>
       </c>
     </row>
     <row r="451" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A451" t="s">
-        <v>189</v>
+        <v>84</v>
       </c>
       <c r="B451" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="C451" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D451" t="s">
         <v>6</v>
@@ -7333,38 +7342,38 @@
     </row>
     <row r="452" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A452" t="s">
+        <v>187</v>
+      </c>
+      <c r="B452" t="s">
+        <v>188</v>
+      </c>
+      <c r="C452" t="b">
+        <v>0</v>
+      </c>
+      <c r="D452" t="s">
         <v>189</v>
-      </c>
-      <c r="B452" t="s">
-        <v>190</v>
-      </c>
-      <c r="C452" t="b">
-        <v>1</v>
-      </c>
-      <c r="D452" t="s">
-        <v>6</v>
       </c>
     </row>
     <row r="453" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A453" t="s">
+        <v>187</v>
+      </c>
+      <c r="B453" t="s">
+        <v>190</v>
+      </c>
+      <c r="C453" t="b">
+        <v>1</v>
+      </c>
+      <c r="D453" t="s">
         <v>191</v>
-      </c>
-      <c r="B453" t="s">
-        <v>5</v>
-      </c>
-      <c r="C453" t="b">
-        <v>1</v>
-      </c>
-      <c r="D453" t="s">
-        <v>6</v>
       </c>
     </row>
     <row r="454" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A454" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="B454" t="s">
-        <v>190</v>
+        <v>5</v>
       </c>
       <c r="C454" t="b">
         <v>1</v>
@@ -7378,7 +7387,7 @@
         <v>192</v>
       </c>
       <c r="B455" t="s">
-        <v>97</v>
+        <v>193</v>
       </c>
       <c r="C455" t="b">
         <v>1</v>
@@ -7389,10 +7398,10 @@
     </row>
     <row r="456" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A456" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="B456" t="s">
-        <v>193</v>
+        <v>5</v>
       </c>
       <c r="C456" t="b">
         <v>1</v>
@@ -7406,7 +7415,7 @@
         <v>194</v>
       </c>
       <c r="B457" t="s">
-        <v>97</v>
+        <v>193</v>
       </c>
       <c r="C457" t="b">
         <v>1</v>
@@ -7417,10 +7426,10 @@
     </row>
     <row r="458" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A458" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="B458" t="s">
-        <v>195</v>
+        <v>97</v>
       </c>
       <c r="C458" t="b">
         <v>1</v>
@@ -7431,10 +7440,10 @@
     </row>
     <row r="459" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A459" t="s">
+        <v>195</v>
+      </c>
+      <c r="B459" t="s">
         <v>196</v>
-      </c>
-      <c r="B459" t="s">
-        <v>5</v>
       </c>
       <c r="C459" t="b">
         <v>1</v>
@@ -7448,7 +7457,7 @@
         <v>197</v>
       </c>
       <c r="B460" t="s">
-        <v>5</v>
+        <v>97</v>
       </c>
       <c r="C460" t="b">
         <v>1</v>
@@ -7459,10 +7468,10 @@
     </row>
     <row r="461" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A461" t="s">
+        <v>197</v>
+      </c>
+      <c r="B461" t="s">
         <v>198</v>
-      </c>
-      <c r="B461" t="s">
-        <v>199</v>
       </c>
       <c r="C461" t="b">
         <v>1</v>
@@ -7473,7 +7482,7 @@
     </row>
     <row r="462" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A462" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B462" t="s">
         <v>5</v>
@@ -7490,10 +7499,10 @@
         <v>200</v>
       </c>
       <c r="B463" t="s">
-        <v>201</v>
+        <v>5</v>
       </c>
       <c r="C463" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D463" t="s">
         <v>6</v>
@@ -7501,10 +7510,10 @@
     </row>
     <row r="464" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A464" t="s">
+        <v>201</v>
+      </c>
+      <c r="B464" t="s">
         <v>202</v>
-      </c>
-      <c r="B464" t="s">
-        <v>5</v>
       </c>
       <c r="C464" t="b">
         <v>1</v>
@@ -7515,13 +7524,13 @@
     </row>
     <row r="465" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A465" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="B465" t="s">
-        <v>201</v>
+        <v>5</v>
       </c>
       <c r="C465" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D465" t="s">
         <v>6</v>
@@ -7532,10 +7541,10 @@
         <v>203</v>
       </c>
       <c r="B466" t="s">
-        <v>5</v>
+        <v>204</v>
       </c>
       <c r="C466" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D466" t="s">
         <v>6</v>
@@ -7543,13 +7552,13 @@
     </row>
     <row r="467" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A467" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="B467" t="s">
-        <v>201</v>
+        <v>5</v>
       </c>
       <c r="C467" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D467" t="s">
         <v>6</v>
@@ -7557,13 +7566,13 @@
     </row>
     <row r="468" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A468" t="s">
+        <v>205</v>
+      </c>
+      <c r="B468" t="s">
         <v>204</v>
       </c>
-      <c r="B468" t="s">
-        <v>5</v>
-      </c>
       <c r="C468" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D468" t="s">
         <v>6</v>
@@ -7571,13 +7580,13 @@
     </row>
     <row r="469" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A469" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="B469" t="s">
-        <v>201</v>
+        <v>5</v>
       </c>
       <c r="C469" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D469" t="s">
         <v>6</v>
@@ -7585,13 +7594,13 @@
     </row>
     <row r="470" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A470" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B470" t="s">
-        <v>5</v>
+        <v>204</v>
       </c>
       <c r="C470" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D470" t="s">
         <v>6</v>
@@ -7599,13 +7608,13 @@
     </row>
     <row r="471" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A471" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="B471" t="s">
         <v>5</v>
       </c>
       <c r="C471" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D471" t="s">
         <v>6</v>
@@ -7613,10 +7622,10 @@
     </row>
     <row r="472" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A472" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="B472" t="s">
-        <v>182</v>
+        <v>204</v>
       </c>
       <c r="C472" t="b">
         <v>0</v>
@@ -7627,13 +7636,13 @@
     </row>
     <row r="473" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A473" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="B473" t="s">
-        <v>179</v>
+        <v>5</v>
       </c>
       <c r="C473" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D473" t="s">
         <v>6</v>
@@ -7641,13 +7650,13 @@
     </row>
     <row r="474" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A474" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="B474" t="s">
-        <v>207</v>
+        <v>5</v>
       </c>
       <c r="C474" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D474" t="s">
         <v>6</v>
@@ -7655,10 +7664,10 @@
     </row>
     <row r="475" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A475" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="B475" t="s">
-        <v>12</v>
+        <v>185</v>
       </c>
       <c r="C475" t="b">
         <v>0</v>
@@ -7669,13 +7678,13 @@
     </row>
     <row r="476" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A476" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="B476" t="s">
-        <v>5</v>
+        <v>182</v>
       </c>
       <c r="C476" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D476" t="s">
         <v>6</v>
@@ -7683,13 +7692,13 @@
     </row>
     <row r="477" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A477" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="B477" t="s">
-        <v>7</v>
+        <v>210</v>
       </c>
       <c r="C477" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D477" t="s">
         <v>6</v>
@@ -7697,24 +7706,24 @@
     </row>
     <row r="478" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A478" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="B478" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="C478" t="b">
         <v>0</v>
       </c>
       <c r="D478" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="479" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A479" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="B479" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="C479" t="b">
         <v>1</v>
@@ -7725,10 +7734,10 @@
     </row>
     <row r="480" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A480" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="B480" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="C480" t="b">
         <v>0</v>
@@ -7739,24 +7748,24 @@
     </row>
     <row r="481" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A481" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="B481" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="C481" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D481" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="482" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A482" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="B482" t="s">
-        <v>45</v>
+        <v>10</v>
       </c>
       <c r="C482" t="b">
         <v>1</v>
@@ -7767,24 +7776,24 @@
     </row>
     <row r="483" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A483" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="B483" t="s">
-        <v>46</v>
+        <v>11</v>
       </c>
       <c r="C483" t="b">
         <v>0</v>
       </c>
       <c r="D483" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="484" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A484" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="B484" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C484" t="b">
         <v>1</v>
@@ -7795,13 +7804,13 @@
     </row>
     <row r="485" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A485" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="B485" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="C485" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D485" t="s">
         <v>6</v>
@@ -7809,24 +7818,24 @@
     </row>
     <row r="486" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A486" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="B486" t="s">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="C486" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D486" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="487" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A487" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="B487" t="s">
-        <v>52</v>
+        <v>13</v>
       </c>
       <c r="C487" t="b">
         <v>1</v>
@@ -7837,57 +7846,99 @@
     </row>
     <row r="488" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A488" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="B488" t="s">
-        <v>19</v>
+        <v>37</v>
       </c>
       <c r="C488" t="b">
         <v>0</v>
       </c>
       <c r="D488" t="s">
-        <v>20</v>
+        <v>6</v>
       </c>
     </row>
     <row r="489" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A489" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="B489" t="s">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="C489" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D489" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="490" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A490" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="B490" t="s">
-        <v>32</v>
+        <v>52</v>
       </c>
       <c r="C490" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D490" t="s">
-        <v>33</v>
+        <v>6</v>
       </c>
     </row>
     <row r="491" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A491" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="B491" t="s">
+        <v>19</v>
+      </c>
+      <c r="C491" t="b">
+        <v>0</v>
+      </c>
+      <c r="D491" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="492" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A492" t="s">
+        <v>211</v>
+      </c>
+      <c r="B492" t="s">
+        <v>31</v>
+      </c>
+      <c r="C492" t="b">
+        <v>0</v>
+      </c>
+      <c r="D492" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="493" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A493" t="s">
+        <v>211</v>
+      </c>
+      <c r="B493" t="s">
+        <v>32</v>
+      </c>
+      <c r="C493" t="b">
+        <v>0</v>
+      </c>
+      <c r="D493" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="494" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A494" t="s">
+        <v>211</v>
+      </c>
+      <c r="B494" t="s">
         <v>34</v>
       </c>
-      <c r="C491" t="b">
-        <v>0</v>
-      </c>
-      <c r="D491" t="s">
+      <c r="C494" t="b">
+        <v>0</v>
+      </c>
+      <c r="D494" t="s">
         <v>35</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Deploying to gh-pages from @ open-resource-discovery/specification@7fea121301a03d3d01f188d6a5a9d1442f5e1d7e 🚀
</commit_message>
<xml_diff>
--- a/spec-v1/interfaces/Document.xlsx
+++ b/spec-v1/interfaces/Document.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1483" uniqueCount="212">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1486" uniqueCount="213">
   <si>
     <t>Entity Name</t>
   </si>
@@ -536,6 +536,9 @@
   </si>
   <si>
     <t>baseUrl</t>
+  </si>
+  <si>
+    <t>globalId</t>
   </si>
   <si>
     <t>System Type</t>
@@ -1023,7 +1026,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D494"/>
+  <dimension ref="A1:D495"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6799,13 +6802,13 @@
         <v>173</v>
       </c>
       <c r="B413" t="s">
-        <v>8</v>
+        <v>175</v>
       </c>
       <c r="C413" t="b">
         <v>0</v>
       </c>
       <c r="D413" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="414" spans="1:4" x14ac:dyDescent="0.25">
@@ -6813,13 +6816,13 @@
         <v>173</v>
       </c>
       <c r="B414" t="s">
-        <v>32</v>
+        <v>8</v>
       </c>
       <c r="C414" t="b">
         <v>0</v>
       </c>
       <c r="D414" t="s">
-        <v>33</v>
+        <v>9</v>
       </c>
     </row>
     <row r="415" spans="1:4" x14ac:dyDescent="0.25">
@@ -6827,13 +6830,13 @@
         <v>173</v>
       </c>
       <c r="B415" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C415" t="b">
         <v>0</v>
       </c>
       <c r="D415" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="416" spans="1:4" x14ac:dyDescent="0.25">
@@ -6841,83 +6844,83 @@
         <v>173</v>
       </c>
       <c r="B416" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="C416" t="b">
         <v>0</v>
       </c>
       <c r="D416" t="s">
-        <v>9</v>
+        <v>35</v>
       </c>
     </row>
     <row r="417" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A417" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="B417" t="s">
-        <v>161</v>
+        <v>31</v>
       </c>
       <c r="C417" t="b">
         <v>0</v>
       </c>
       <c r="D417" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="418" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A418" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B418" t="s">
-        <v>8</v>
+        <v>161</v>
       </c>
       <c r="C418" t="b">
         <v>0</v>
       </c>
       <c r="D418" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="419" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A419" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B419" t="s">
-        <v>32</v>
+        <v>8</v>
       </c>
       <c r="C419" t="b">
         <v>0</v>
       </c>
       <c r="D419" t="s">
-        <v>33</v>
+        <v>9</v>
       </c>
     </row>
     <row r="420" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A420" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B420" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C420" t="b">
         <v>0</v>
       </c>
       <c r="D420" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="421" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A421" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B421" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="C421" t="b">
         <v>0</v>
       </c>
       <c r="D421" t="s">
-        <v>9</v>
+        <v>35</v>
       </c>
     </row>
     <row r="422" spans="1:4" x14ac:dyDescent="0.25">
@@ -6925,21 +6928,21 @@
         <v>176</v>
       </c>
       <c r="B422" t="s">
-        <v>13</v>
+        <v>31</v>
       </c>
       <c r="C422" t="b">
         <v>0</v>
       </c>
       <c r="D422" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="423" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A423" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B423" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="C423" t="b">
         <v>0</v>
@@ -6950,58 +6953,58 @@
     </row>
     <row r="424" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A424" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B424" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C424" t="b">
         <v>0</v>
       </c>
       <c r="D424" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="425" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A425" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B425" t="s">
-        <v>32</v>
+        <v>8</v>
       </c>
       <c r="C425" t="b">
         <v>0</v>
       </c>
       <c r="D425" t="s">
-        <v>33</v>
+        <v>9</v>
       </c>
     </row>
     <row r="426" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A426" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B426" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C426" t="b">
         <v>0</v>
       </c>
       <c r="D426" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="427" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A427" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B427" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="C427" t="b">
         <v>0</v>
       </c>
       <c r="D427" t="s">
-        <v>9</v>
+        <v>35</v>
       </c>
     </row>
     <row r="428" spans="1:4" x14ac:dyDescent="0.25">
@@ -7009,24 +7012,24 @@
         <v>177</v>
       </c>
       <c r="B428" t="s">
-        <v>97</v>
+        <v>31</v>
       </c>
       <c r="C428" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D428" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="429" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A429" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="B429" t="s">
-        <v>115</v>
+        <v>97</v>
       </c>
       <c r="C429" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D429" t="s">
         <v>6</v>
@@ -7034,10 +7037,10 @@
     </row>
     <row r="430" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A430" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="B430" t="s">
-        <v>178</v>
+        <v>115</v>
       </c>
       <c r="C430" t="b">
         <v>0</v>
@@ -7048,13 +7051,13 @@
     </row>
     <row r="431" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A431" t="s">
+        <v>178</v>
+      </c>
+      <c r="B431" t="s">
         <v>179</v>
       </c>
-      <c r="B431" t="s">
-        <v>97</v>
-      </c>
       <c r="C431" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D431" t="s">
         <v>6</v>
@@ -7062,13 +7065,13 @@
     </row>
     <row r="432" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A432" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="B432" t="s">
-        <v>115</v>
+        <v>97</v>
       </c>
       <c r="C432" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D432" t="s">
         <v>6</v>
@@ -7076,10 +7079,10 @@
     </row>
     <row r="433" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A433" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="B433" t="s">
-        <v>178</v>
+        <v>115</v>
       </c>
       <c r="C433" t="b">
         <v>0</v>
@@ -7090,10 +7093,10 @@
     </row>
     <row r="434" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A434" t="s">
+        <v>180</v>
+      </c>
+      <c r="B434" t="s">
         <v>179</v>
-      </c>
-      <c r="B434" t="s">
-        <v>180</v>
       </c>
       <c r="C434" t="b">
         <v>0</v>
@@ -7104,13 +7107,13 @@
     </row>
     <row r="435" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A435" t="s">
+        <v>180</v>
+      </c>
+      <c r="B435" t="s">
         <v>181</v>
       </c>
-      <c r="B435" t="s">
-        <v>182</v>
-      </c>
       <c r="C435" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D435" t="s">
         <v>6</v>
@@ -7118,10 +7121,10 @@
     </row>
     <row r="436" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A436" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="B436" t="s">
-        <v>10</v>
+        <v>183</v>
       </c>
       <c r="C436" t="b">
         <v>1</v>
@@ -7132,13 +7135,13 @@
     </row>
     <row r="437" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A437" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="B437" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C437" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D437" t="s">
         <v>6</v>
@@ -7146,38 +7149,38 @@
     </row>
     <row r="438" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A438" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="B438" t="s">
-        <v>32</v>
+        <v>12</v>
       </c>
       <c r="C438" t="b">
         <v>0</v>
       </c>
       <c r="D438" t="s">
-        <v>33</v>
+        <v>6</v>
       </c>
     </row>
     <row r="439" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A439" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="B439" t="s">
-        <v>8</v>
+        <v>32</v>
       </c>
       <c r="C439" t="b">
         <v>0</v>
       </c>
       <c r="D439" t="s">
-        <v>9</v>
+        <v>33</v>
       </c>
     </row>
     <row r="440" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A440" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="B440" t="s">
-        <v>183</v>
+        <v>8</v>
       </c>
       <c r="C440" t="b">
         <v>0</v>
@@ -7188,27 +7191,27 @@
     </row>
     <row r="441" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A441" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="B441" t="s">
-        <v>38</v>
+        <v>184</v>
       </c>
       <c r="C441" t="b">
         <v>0</v>
       </c>
       <c r="D441" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="442" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A442" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="B442" t="s">
-        <v>185</v>
+        <v>38</v>
       </c>
       <c r="C442" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D442" t="s">
         <v>6</v>
@@ -7216,10 +7219,10 @@
     </row>
     <row r="443" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A443" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="B443" t="s">
-        <v>182</v>
+        <v>186</v>
       </c>
       <c r="C443" t="b">
         <v>1</v>
@@ -7230,10 +7233,10 @@
     </row>
     <row r="444" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A444" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="B444" t="s">
-        <v>10</v>
+        <v>183</v>
       </c>
       <c r="C444" t="b">
         <v>1</v>
@@ -7244,13 +7247,13 @@
     </row>
     <row r="445" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A445" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="B445" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C445" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D445" t="s">
         <v>6</v>
@@ -7258,38 +7261,38 @@
     </row>
     <row r="446" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A446" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="B446" t="s">
-        <v>32</v>
+        <v>12</v>
       </c>
       <c r="C446" t="b">
         <v>0</v>
       </c>
       <c r="D446" t="s">
-        <v>33</v>
+        <v>6</v>
       </c>
     </row>
     <row r="447" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A447" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="B447" t="s">
-        <v>8</v>
+        <v>32</v>
       </c>
       <c r="C447" t="b">
         <v>0</v>
       </c>
       <c r="D447" t="s">
-        <v>9</v>
+        <v>33</v>
       </c>
     </row>
     <row r="448" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A448" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="B448" t="s">
-        <v>46</v>
+        <v>8</v>
       </c>
       <c r="C448" t="b">
         <v>0</v>
@@ -7300,27 +7303,27 @@
     </row>
     <row r="449" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A449" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="B449" t="s">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="C449" t="b">
         <v>0</v>
       </c>
       <c r="D449" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="450" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A450" t="s">
-        <v>84</v>
+        <v>185</v>
       </c>
       <c r="B450" t="s">
-        <v>186</v>
+        <v>38</v>
       </c>
       <c r="C450" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D450" t="s">
         <v>6</v>
@@ -7331,10 +7334,10 @@
         <v>84</v>
       </c>
       <c r="B451" t="s">
-        <v>12</v>
+        <v>187</v>
       </c>
       <c r="C451" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D451" t="s">
         <v>6</v>
@@ -7342,52 +7345,52 @@
     </row>
     <row r="452" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A452" t="s">
-        <v>187</v>
+        <v>84</v>
       </c>
       <c r="B452" t="s">
-        <v>188</v>
+        <v>12</v>
       </c>
       <c r="C452" t="b">
         <v>0</v>
       </c>
       <c r="D452" t="s">
-        <v>189</v>
+        <v>6</v>
       </c>
     </row>
     <row r="453" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A453" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="B453" t="s">
+        <v>189</v>
+      </c>
+      <c r="C453" t="b">
+        <v>0</v>
+      </c>
+      <c r="D453" t="s">
         <v>190</v>
-      </c>
-      <c r="C453" t="b">
-        <v>1</v>
-      </c>
-      <c r="D453" t="s">
-        <v>191</v>
       </c>
     </row>
     <row r="454" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A454" t="s">
+        <v>188</v>
+      </c>
+      <c r="B454" t="s">
+        <v>191</v>
+      </c>
+      <c r="C454" t="b">
+        <v>1</v>
+      </c>
+      <c r="D454" t="s">
         <v>192</v>
-      </c>
-      <c r="B454" t="s">
-        <v>5</v>
-      </c>
-      <c r="C454" t="b">
-        <v>1</v>
-      </c>
-      <c r="D454" t="s">
-        <v>6</v>
       </c>
     </row>
     <row r="455" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A455" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="B455" t="s">
-        <v>193</v>
+        <v>5</v>
       </c>
       <c r="C455" t="b">
         <v>1</v>
@@ -7398,10 +7401,10 @@
     </row>
     <row r="456" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A456" t="s">
+        <v>193</v>
+      </c>
+      <c r="B456" t="s">
         <v>194</v>
-      </c>
-      <c r="B456" t="s">
-        <v>5</v>
       </c>
       <c r="C456" t="b">
         <v>1</v>
@@ -7412,10 +7415,10 @@
     </row>
     <row r="457" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A457" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="B457" t="s">
-        <v>193</v>
+        <v>5</v>
       </c>
       <c r="C457" t="b">
         <v>1</v>
@@ -7429,7 +7432,7 @@
         <v>195</v>
       </c>
       <c r="B458" t="s">
-        <v>97</v>
+        <v>194</v>
       </c>
       <c r="C458" t="b">
         <v>1</v>
@@ -7440,10 +7443,10 @@
     </row>
     <row r="459" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A459" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="B459" t="s">
-        <v>196</v>
+        <v>97</v>
       </c>
       <c r="C459" t="b">
         <v>1</v>
@@ -7454,10 +7457,10 @@
     </row>
     <row r="460" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A460" t="s">
+        <v>196</v>
+      </c>
+      <c r="B460" t="s">
         <v>197</v>
-      </c>
-      <c r="B460" t="s">
-        <v>97</v>
       </c>
       <c r="C460" t="b">
         <v>1</v>
@@ -7468,10 +7471,10 @@
     </row>
     <row r="461" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A461" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="B461" t="s">
-        <v>198</v>
+        <v>97</v>
       </c>
       <c r="C461" t="b">
         <v>1</v>
@@ -7482,10 +7485,10 @@
     </row>
     <row r="462" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A462" t="s">
+        <v>198</v>
+      </c>
+      <c r="B462" t="s">
         <v>199</v>
-      </c>
-      <c r="B462" t="s">
-        <v>5</v>
       </c>
       <c r="C462" t="b">
         <v>1</v>
@@ -7513,7 +7516,7 @@
         <v>201</v>
       </c>
       <c r="B464" t="s">
-        <v>202</v>
+        <v>5</v>
       </c>
       <c r="C464" t="b">
         <v>1</v>
@@ -7524,10 +7527,10 @@
     </row>
     <row r="465" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A465" t="s">
+        <v>202</v>
+      </c>
+      <c r="B465" t="s">
         <v>203</v>
-      </c>
-      <c r="B465" t="s">
-        <v>5</v>
       </c>
       <c r="C465" t="b">
         <v>1</v>
@@ -7538,13 +7541,13 @@
     </row>
     <row r="466" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A466" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="B466" t="s">
-        <v>204</v>
+        <v>5</v>
       </c>
       <c r="C466" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D466" t="s">
         <v>6</v>
@@ -7552,13 +7555,13 @@
     </row>
     <row r="467" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A467" t="s">
+        <v>204</v>
+      </c>
+      <c r="B467" t="s">
         <v>205</v>
       </c>
-      <c r="B467" t="s">
-        <v>5</v>
-      </c>
       <c r="C467" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D467" t="s">
         <v>6</v>
@@ -7566,13 +7569,13 @@
     </row>
     <row r="468" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A468" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B468" t="s">
-        <v>204</v>
+        <v>5</v>
       </c>
       <c r="C468" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D468" t="s">
         <v>6</v>
@@ -7583,10 +7586,10 @@
         <v>206</v>
       </c>
       <c r="B469" t="s">
-        <v>5</v>
+        <v>205</v>
       </c>
       <c r="C469" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D469" t="s">
         <v>6</v>
@@ -7594,13 +7597,13 @@
     </row>
     <row r="470" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A470" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="B470" t="s">
-        <v>204</v>
+        <v>5</v>
       </c>
       <c r="C470" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D470" t="s">
         <v>6</v>
@@ -7611,10 +7614,10 @@
         <v>207</v>
       </c>
       <c r="B471" t="s">
-        <v>5</v>
+        <v>205</v>
       </c>
       <c r="C471" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D471" t="s">
         <v>6</v>
@@ -7622,13 +7625,13 @@
     </row>
     <row r="472" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A472" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="B472" t="s">
-        <v>204</v>
+        <v>5</v>
       </c>
       <c r="C472" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D472" t="s">
         <v>6</v>
@@ -7639,10 +7642,10 @@
         <v>208</v>
       </c>
       <c r="B473" t="s">
-        <v>5</v>
+        <v>205</v>
       </c>
       <c r="C473" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D473" t="s">
         <v>6</v>
@@ -7656,7 +7659,7 @@
         <v>5</v>
       </c>
       <c r="C474" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D474" t="s">
         <v>6</v>
@@ -7664,10 +7667,10 @@
     </row>
     <row r="475" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A475" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="B475" t="s">
-        <v>185</v>
+        <v>5</v>
       </c>
       <c r="C475" t="b">
         <v>0</v>
@@ -7678,10 +7681,10 @@
     </row>
     <row r="476" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A476" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="B476" t="s">
-        <v>182</v>
+        <v>186</v>
       </c>
       <c r="C476" t="b">
         <v>0</v>
@@ -7692,13 +7695,13 @@
     </row>
     <row r="477" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A477" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="B477" t="s">
-        <v>210</v>
+        <v>183</v>
       </c>
       <c r="C477" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D477" t="s">
         <v>6</v>
@@ -7706,13 +7709,13 @@
     </row>
     <row r="478" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A478" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="B478" t="s">
-        <v>12</v>
+        <v>211</v>
       </c>
       <c r="C478" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D478" t="s">
         <v>6</v>
@@ -7720,13 +7723,13 @@
     </row>
     <row r="479" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A479" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="B479" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="C479" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D479" t="s">
         <v>6</v>
@@ -7734,13 +7737,13 @@
     </row>
     <row r="480" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A480" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="B480" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C480" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D480" t="s">
         <v>6</v>
@@ -7748,41 +7751,41 @@
     </row>
     <row r="481" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A481" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="B481" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C481" t="b">
         <v>0</v>
       </c>
       <c r="D481" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="482" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A482" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="B482" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C482" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D482" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="483" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A483" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="B483" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C483" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D483" t="s">
         <v>6</v>
@@ -7790,13 +7793,13 @@
     </row>
     <row r="484" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A484" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="B484" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C484" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D484" t="s">
         <v>6</v>
@@ -7804,10 +7807,10 @@
     </row>
     <row r="485" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A485" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="B485" t="s">
-        <v>45</v>
+        <v>12</v>
       </c>
       <c r="C485" t="b">
         <v>1</v>
@@ -7818,41 +7821,41 @@
     </row>
     <row r="486" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A486" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="B486" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C486" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D486" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="487" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A487" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="B487" t="s">
-        <v>13</v>
+        <v>46</v>
       </c>
       <c r="C487" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D487" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="488" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A488" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="B488" t="s">
-        <v>37</v>
+        <v>13</v>
       </c>
       <c r="C488" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D488" t="s">
         <v>6</v>
@@ -7860,13 +7863,13 @@
     </row>
     <row r="489" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A489" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="B489" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C489" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D489" t="s">
         <v>6</v>
@@ -7874,10 +7877,10 @@
     </row>
     <row r="490" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A490" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="B490" t="s">
-        <v>52</v>
+        <v>38</v>
       </c>
       <c r="C490" t="b">
         <v>1</v>
@@ -7888,57 +7891,71 @@
     </row>
     <row r="491" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A491" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="B491" t="s">
-        <v>19</v>
+        <v>52</v>
       </c>
       <c r="C491" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D491" t="s">
-        <v>20</v>
+        <v>6</v>
       </c>
     </row>
     <row r="492" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A492" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="B492" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="C492" t="b">
         <v>0</v>
       </c>
       <c r="D492" t="s">
-        <v>9</v>
+        <v>20</v>
       </c>
     </row>
     <row r="493" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A493" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="B493" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C493" t="b">
         <v>0</v>
       </c>
       <c r="D493" t="s">
-        <v>33</v>
+        <v>9</v>
       </c>
     </row>
     <row r="494" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A494" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="B494" t="s">
+        <v>32</v>
+      </c>
+      <c r="C494" t="b">
+        <v>0</v>
+      </c>
+      <c r="D494" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="495" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A495" t="s">
+        <v>212</v>
+      </c>
+      <c r="B495" t="s">
         <v>34</v>
       </c>
-      <c r="C494" t="b">
-        <v>0</v>
-      </c>
-      <c r="D494" t="s">
+      <c r="C495" t="b">
+        <v>0</v>
+      </c>
+      <c r="D495" t="s">
         <v>35</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Deploying to gh-pages from @ open-resource-discovery/specification@9f8728913addadae31d7c870bba73af271cc6f14 🚀
</commit_message>
<xml_diff>
--- a/spec-v1/interfaces/Document.xlsx
+++ b/spec-v1/interfaces/Document.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1486" uniqueCount="213">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1495" uniqueCount="216">
   <si>
     <t>Entity Name</t>
   </si>
@@ -331,6 +331,12 @@
     <t>entityTypes</t>
   </si>
   <si>
+    <t>relatedDataProducts</t>
+  </si>
+  <si>
+    <t>array&lt;RelatedDataProduct&gt;</t>
+  </si>
+  <si>
     <t>inputPorts</t>
   </si>
   <si>
@@ -635,6 +641,9 @@
   </si>
   <si>
     <t>Related Event Resource</t>
+  </si>
+  <si>
+    <t>Related Data Product</t>
   </si>
   <si>
     <t>Related Capability</t>
@@ -1026,7 +1035,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D495"/>
+  <dimension ref="A1:D498"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -3823,7 +3832,7 @@
         <v>108</v>
       </c>
       <c r="C200" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D200" t="s">
         <v>109</v>
@@ -3834,13 +3843,13 @@
         <v>102</v>
       </c>
       <c r="B201" t="s">
-        <v>74</v>
+        <v>110</v>
       </c>
       <c r="C201" t="b">
         <v>1</v>
       </c>
       <c r="D201" t="s">
-        <v>6</v>
+        <v>111</v>
       </c>
     </row>
     <row r="202" spans="1:4" x14ac:dyDescent="0.25">
@@ -3848,13 +3857,13 @@
         <v>102</v>
       </c>
       <c r="B202" t="s">
-        <v>110</v>
+        <v>74</v>
       </c>
       <c r="C202" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D202" t="s">
-        <v>111</v>
+        <v>6</v>
       </c>
     </row>
     <row r="203" spans="1:4" x14ac:dyDescent="0.25">
@@ -3862,13 +3871,13 @@
         <v>102</v>
       </c>
       <c r="B203" t="s">
-        <v>19</v>
+        <v>112</v>
       </c>
       <c r="C203" t="b">
         <v>0</v>
       </c>
       <c r="D203" t="s">
-        <v>20</v>
+        <v>113</v>
       </c>
     </row>
     <row r="204" spans="1:4" x14ac:dyDescent="0.25">
@@ -3876,13 +3885,13 @@
         <v>102</v>
       </c>
       <c r="B204" t="s">
-        <v>29</v>
+        <v>19</v>
       </c>
       <c r="C204" t="b">
         <v>0</v>
       </c>
       <c r="D204" t="s">
-        <v>9</v>
+        <v>20</v>
       </c>
     </row>
     <row r="205" spans="1:4" x14ac:dyDescent="0.25">
@@ -3890,7 +3899,7 @@
         <v>102</v>
       </c>
       <c r="B205" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C205" t="b">
         <v>0</v>
@@ -3904,7 +3913,7 @@
         <v>102</v>
       </c>
       <c r="B206" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C206" t="b">
         <v>0</v>
@@ -3918,7 +3927,7 @@
         <v>102</v>
       </c>
       <c r="B207" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="C207" t="b">
         <v>0</v>
@@ -3932,13 +3941,13 @@
         <v>102</v>
       </c>
       <c r="B208" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C208" t="b">
         <v>0</v>
       </c>
       <c r="D208" t="s">
-        <v>33</v>
+        <v>9</v>
       </c>
     </row>
     <row r="209" spans="1:4" x14ac:dyDescent="0.25">
@@ -3946,13 +3955,13 @@
         <v>102</v>
       </c>
       <c r="B209" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C209" t="b">
         <v>0</v>
       </c>
       <c r="D209" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="210" spans="1:4" x14ac:dyDescent="0.25">
@@ -3960,13 +3969,13 @@
         <v>102</v>
       </c>
       <c r="B210" t="s">
-        <v>14</v>
+        <v>34</v>
       </c>
       <c r="C210" t="b">
         <v>0</v>
       </c>
       <c r="D210" t="s">
-        <v>6</v>
+        <v>35</v>
       </c>
     </row>
     <row r="211" spans="1:4" x14ac:dyDescent="0.25">
@@ -3974,7 +3983,7 @@
         <v>102</v>
       </c>
       <c r="B211" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C211" t="b">
         <v>0</v>
@@ -3988,13 +3997,13 @@
         <v>102</v>
       </c>
       <c r="B212" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C212" t="b">
         <v>0</v>
       </c>
       <c r="D212" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="213" spans="1:4" x14ac:dyDescent="0.25">
@@ -4002,32 +4011,32 @@
         <v>102</v>
       </c>
       <c r="B213" t="s">
-        <v>85</v>
+        <v>16</v>
       </c>
       <c r="C213" t="b">
         <v>0</v>
       </c>
       <c r="D213" t="s">
-        <v>51</v>
+        <v>9</v>
       </c>
     </row>
     <row r="214" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A214" t="s">
-        <v>112</v>
+        <v>102</v>
       </c>
       <c r="B214" t="s">
-        <v>5</v>
+        <v>85</v>
       </c>
       <c r="C214" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D214" t="s">
-        <v>6</v>
+        <v>51</v>
       </c>
     </row>
     <row r="215" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A215" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B215" t="s">
         <v>5</v>
@@ -4041,10 +4050,10 @@
     </row>
     <row r="216" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A216" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="B216" t="s">
-        <v>97</v>
+        <v>5</v>
       </c>
       <c r="C216" t="b">
         <v>1</v>
@@ -4055,13 +4064,13 @@
     </row>
     <row r="217" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A217" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="B217" t="s">
-        <v>115</v>
+        <v>97</v>
       </c>
       <c r="C217" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D217" t="s">
         <v>6</v>
@@ -4069,13 +4078,13 @@
     </row>
     <row r="218" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A218" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="B218" t="s">
-        <v>98</v>
+        <v>117</v>
       </c>
       <c r="C218" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D218" t="s">
         <v>6</v>
@@ -4083,10 +4092,10 @@
     </row>
     <row r="219" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A219" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="B219" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C219" t="b">
         <v>1</v>
@@ -4097,13 +4106,13 @@
     </row>
     <row r="220" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A220" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="B220" t="s">
-        <v>38</v>
+        <v>99</v>
       </c>
       <c r="C220" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D220" t="s">
         <v>6</v>
@@ -4111,41 +4120,41 @@
     </row>
     <row r="221" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A221" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="B221" t="s">
-        <v>100</v>
+        <v>38</v>
       </c>
       <c r="C221" t="b">
         <v>0</v>
       </c>
       <c r="D221" t="s">
-        <v>101</v>
+        <v>6</v>
       </c>
     </row>
     <row r="222" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A222" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="B222" t="s">
-        <v>116</v>
+        <v>100</v>
       </c>
       <c r="C222" t="b">
         <v>0</v>
       </c>
       <c r="D222" t="s">
-        <v>6</v>
+        <v>101</v>
       </c>
     </row>
     <row r="223" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A223" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B223" t="s">
-        <v>97</v>
+        <v>118</v>
       </c>
       <c r="C223" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D223" t="s">
         <v>6</v>
@@ -4153,13 +4162,13 @@
     </row>
     <row r="224" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A224" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B224" t="s">
-        <v>115</v>
+        <v>97</v>
       </c>
       <c r="C224" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D224" t="s">
         <v>6</v>
@@ -4167,13 +4176,13 @@
     </row>
     <row r="225" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A225" t="s">
+        <v>119</v>
+      </c>
+      <c r="B225" t="s">
         <v>117</v>
       </c>
-      <c r="B225" t="s">
-        <v>98</v>
-      </c>
       <c r="C225" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D225" t="s">
         <v>6</v>
@@ -4181,10 +4190,10 @@
     </row>
     <row r="226" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A226" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B226" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C226" t="b">
         <v>1</v>
@@ -4195,38 +4204,38 @@
     </row>
     <row r="227" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A227" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B227" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C227" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D227" t="s">
-        <v>101</v>
+        <v>6</v>
       </c>
     </row>
     <row r="228" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A228" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B228" t="s">
-        <v>38</v>
+        <v>100</v>
       </c>
       <c r="C228" t="b">
         <v>0</v>
       </c>
       <c r="D228" t="s">
-        <v>6</v>
+        <v>101</v>
       </c>
     </row>
     <row r="229" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A229" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B229" t="s">
-        <v>116</v>
+        <v>38</v>
       </c>
       <c r="C229" t="b">
         <v>0</v>
@@ -4237,13 +4246,13 @@
     </row>
     <row r="230" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A230" t="s">
+        <v>119</v>
+      </c>
+      <c r="B230" t="s">
         <v>118</v>
       </c>
-      <c r="B230" t="s">
-        <v>5</v>
-      </c>
       <c r="C230" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D230" t="s">
         <v>6</v>
@@ -4251,13 +4260,13 @@
     </row>
     <row r="231" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A231" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B231" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C231" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D231" t="s">
         <v>6</v>
@@ -4265,41 +4274,41 @@
     </row>
     <row r="232" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A232" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B232" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C232" t="b">
         <v>0</v>
       </c>
       <c r="D232" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="233" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A233" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B233" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C233" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D233" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="234" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A234" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B234" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C234" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D234" t="s">
         <v>6</v>
@@ -4307,10 +4316,10 @@
     </row>
     <row r="235" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A235" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B235" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C235" t="b">
         <v>0</v>
@@ -4321,10 +4330,10 @@
     </row>
     <row r="236" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A236" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B236" t="s">
-        <v>44</v>
+        <v>12</v>
       </c>
       <c r="C236" t="b">
         <v>0</v>
@@ -4335,13 +4344,13 @@
     </row>
     <row r="237" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A237" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B237" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C237" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D237" t="s">
         <v>6</v>
@@ -4349,41 +4358,41 @@
     </row>
     <row r="238" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A238" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B238" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C238" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D238" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="239" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A239" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B239" t="s">
-        <v>13</v>
+        <v>46</v>
       </c>
       <c r="C239" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D239" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="240" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A240" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B240" t="s">
-        <v>37</v>
+        <v>13</v>
       </c>
       <c r="C240" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D240" t="s">
         <v>6</v>
@@ -4391,13 +4400,13 @@
     </row>
     <row r="241" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A241" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B241" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C241" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D241" t="s">
         <v>6</v>
@@ -4405,10 +4414,10 @@
     </row>
     <row r="242" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A242" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B242" t="s">
-        <v>52</v>
+        <v>38</v>
       </c>
       <c r="C242" t="b">
         <v>1</v>
@@ -4419,66 +4428,66 @@
     </row>
     <row r="243" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A243" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B243" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C243" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D243" t="s">
-        <v>51</v>
+        <v>6</v>
       </c>
     </row>
     <row r="244" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A244" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B244" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C244" t="b">
         <v>0</v>
       </c>
       <c r="D244" t="s">
-        <v>6</v>
+        <v>51</v>
       </c>
     </row>
     <row r="245" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A245" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B245" t="s">
-        <v>26</v>
+        <v>54</v>
       </c>
       <c r="C245" t="b">
         <v>0</v>
       </c>
       <c r="D245" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="246" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A246" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B246" t="s">
-        <v>74</v>
+        <v>26</v>
       </c>
       <c r="C246" t="b">
         <v>0</v>
       </c>
       <c r="D246" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="247" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A247" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B247" t="s">
-        <v>59</v>
+        <v>74</v>
       </c>
       <c r="C247" t="b">
         <v>0</v>
@@ -4489,10 +4498,10 @@
     </row>
     <row r="248" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A248" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B248" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C248" t="b">
         <v>0</v>
@@ -4503,52 +4512,52 @@
     </row>
     <row r="249" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A249" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B249" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C249" t="b">
         <v>0</v>
       </c>
       <c r="D249" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="250" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A250" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B250" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C250" t="b">
         <v>0</v>
       </c>
       <c r="D250" t="s">
-        <v>63</v>
+        <v>9</v>
       </c>
     </row>
     <row r="251" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A251" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B251" t="s">
-        <v>16</v>
+        <v>62</v>
       </c>
       <c r="C251" t="b">
         <v>0</v>
       </c>
       <c r="D251" t="s">
-        <v>9</v>
+        <v>63</v>
       </c>
     </row>
     <row r="252" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A252" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B252" t="s">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="C252" t="b">
         <v>0</v>
@@ -4559,10 +4568,10 @@
     </row>
     <row r="253" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A253" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B253" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C253" t="b">
         <v>0</v>
@@ -4573,10 +4582,10 @@
     </row>
     <row r="254" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A254" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B254" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C254" t="b">
         <v>0</v>
@@ -4587,10 +4596,10 @@
     </row>
     <row r="255" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A255" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B255" t="s">
-        <v>92</v>
+        <v>29</v>
       </c>
       <c r="C255" t="b">
         <v>0</v>
@@ -4601,21 +4610,21 @@
     </row>
     <row r="256" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A256" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B256" t="s">
-        <v>119</v>
+        <v>92</v>
       </c>
       <c r="C256" t="b">
         <v>0</v>
       </c>
       <c r="D256" t="s">
-        <v>120</v>
+        <v>9</v>
       </c>
     </row>
     <row r="257" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A257" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B257" t="s">
         <v>121</v>
@@ -4624,88 +4633,88 @@
         <v>0</v>
       </c>
       <c r="D257" t="s">
-        <v>9</v>
+        <v>122</v>
       </c>
     </row>
     <row r="258" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A258" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B258" t="s">
-        <v>19</v>
+        <v>123</v>
       </c>
       <c r="C258" t="b">
         <v>0</v>
       </c>
       <c r="D258" t="s">
-        <v>20</v>
+        <v>9</v>
       </c>
     </row>
     <row r="259" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A259" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B259" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="C259" t="b">
         <v>0</v>
       </c>
       <c r="D259" t="s">
-        <v>9</v>
+        <v>20</v>
       </c>
     </row>
     <row r="260" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A260" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B260" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C260" t="b">
         <v>0</v>
       </c>
       <c r="D260" t="s">
-        <v>33</v>
+        <v>9</v>
       </c>
     </row>
     <row r="261" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A261" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B261" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C261" t="b">
         <v>0</v>
       </c>
       <c r="D261" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="262" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A262" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="B262" t="s">
-        <v>5</v>
+        <v>34</v>
       </c>
       <c r="C262" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D262" t="s">
-        <v>6</v>
+        <v>35</v>
       </c>
     </row>
     <row r="263" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A263" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B263" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="C263" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D263" t="s">
         <v>6</v>
@@ -4713,10 +4722,10 @@
     </row>
     <row r="264" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A264" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B264" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C264" t="b">
         <v>0</v>
@@ -4727,13 +4736,13 @@
     </row>
     <row r="265" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A265" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B265" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C265" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D265" t="s">
         <v>6</v>
@@ -4741,13 +4750,13 @@
     </row>
     <row r="266" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A266" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B266" t="s">
-        <v>37</v>
+        <v>13</v>
       </c>
       <c r="C266" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D266" t="s">
         <v>6</v>
@@ -4755,13 +4764,13 @@
     </row>
     <row r="267" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A267" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B267" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C267" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D267" t="s">
         <v>6</v>
@@ -4769,10 +4778,10 @@
     </row>
     <row r="268" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A268" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B268" t="s">
-        <v>52</v>
+        <v>38</v>
       </c>
       <c r="C268" t="b">
         <v>1</v>
@@ -4783,72 +4792,72 @@
     </row>
     <row r="269" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A269" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B269" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="C269" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D269" t="s">
-        <v>56</v>
+        <v>6</v>
       </c>
     </row>
     <row r="270" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A270" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B270" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="C270" t="b">
         <v>0</v>
       </c>
       <c r="D270" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="271" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A271" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B271" t="s">
-        <v>94</v>
+        <v>57</v>
       </c>
       <c r="C271" t="b">
         <v>0</v>
       </c>
       <c r="D271" t="s">
-        <v>123</v>
+        <v>58</v>
       </c>
     </row>
     <row r="272" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A272" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B272" t="s">
-        <v>31</v>
+        <v>94</v>
       </c>
       <c r="C272" t="b">
         <v>0</v>
       </c>
       <c r="D272" t="s">
-        <v>9</v>
+        <v>125</v>
       </c>
     </row>
     <row r="273" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A273" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B273" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C273" t="b">
         <v>0</v>
       </c>
       <c r="D273" t="s">
-        <v>33</v>
+        <v>9</v>
       </c>
     </row>
     <row r="274" spans="1:4" x14ac:dyDescent="0.25">
@@ -4856,21 +4865,21 @@
         <v>124</v>
       </c>
       <c r="B274" t="s">
-        <v>97</v>
+        <v>32</v>
       </c>
       <c r="C274" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D274" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
     </row>
     <row r="275" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A275" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B275" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C275" t="b">
         <v>1</v>
@@ -4881,10 +4890,10 @@
     </row>
     <row r="276" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A276" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B276" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C276" t="b">
         <v>1</v>
@@ -4895,38 +4904,38 @@
     </row>
     <row r="277" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A277" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B277" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C277" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D277" t="s">
-        <v>101</v>
+        <v>6</v>
       </c>
     </row>
     <row r="278" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A278" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B278" t="s">
-        <v>38</v>
+        <v>100</v>
       </c>
       <c r="C278" t="b">
         <v>0</v>
       </c>
       <c r="D278" t="s">
-        <v>6</v>
+        <v>101</v>
       </c>
     </row>
     <row r="279" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A279" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B279" t="s">
-        <v>116</v>
+        <v>38</v>
       </c>
       <c r="C279" t="b">
         <v>0</v>
@@ -4937,13 +4946,13 @@
     </row>
     <row r="280" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A280" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B280" t="s">
-        <v>5</v>
+        <v>118</v>
       </c>
       <c r="C280" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D280" t="s">
         <v>6</v>
@@ -4951,38 +4960,38 @@
     </row>
     <row r="281" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A281" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B281" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="C281" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D281" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="282" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A282" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B282" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C282" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D282" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="283" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A283" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B283" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C283" t="b">
         <v>1</v>
@@ -4993,13 +5002,13 @@
     </row>
     <row r="284" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A284" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B284" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C284" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D284" t="s">
         <v>6</v>
@@ -5007,13 +5016,13 @@
     </row>
     <row r="285" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A285" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B285" t="s">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="C285" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D285" t="s">
         <v>6</v>
@@ -5021,13 +5030,13 @@
     </row>
     <row r="286" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A286" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B286" t="s">
-        <v>126</v>
+        <v>25</v>
       </c>
       <c r="C286" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D286" t="s">
         <v>6</v>
@@ -5035,44 +5044,44 @@
     </row>
     <row r="287" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A287" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B287" t="s">
-        <v>31</v>
+        <v>128</v>
       </c>
       <c r="C287" t="b">
         <v>0</v>
       </c>
       <c r="D287" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="288" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A288" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B288" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C288" t="b">
         <v>0</v>
       </c>
       <c r="D288" t="s">
-        <v>33</v>
+        <v>9</v>
       </c>
     </row>
     <row r="289" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A289" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B289" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C289" t="b">
         <v>0</v>
       </c>
       <c r="D289" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="290" spans="1:4" x14ac:dyDescent="0.25">
@@ -5080,24 +5089,24 @@
         <v>127</v>
       </c>
       <c r="B290" t="s">
-        <v>5</v>
+        <v>34</v>
       </c>
       <c r="C290" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D290" t="s">
-        <v>6</v>
+        <v>35</v>
       </c>
     </row>
     <row r="291" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A291" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B291" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C291" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D291" t="s">
         <v>6</v>
@@ -5105,41 +5114,41 @@
     </row>
     <row r="292" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A292" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B292" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C292" t="b">
         <v>0</v>
       </c>
       <c r="D292" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="293" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A293" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B293" t="s">
-        <v>97</v>
+        <v>8</v>
       </c>
       <c r="C293" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D293" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="294" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A294" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B294" t="s">
-        <v>115</v>
+        <v>97</v>
       </c>
       <c r="C294" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D294" t="s">
         <v>6</v>
@@ -5147,13 +5156,13 @@
     </row>
     <row r="295" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A295" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B295" t="s">
-        <v>10</v>
+        <v>117</v>
       </c>
       <c r="C295" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D295" t="s">
         <v>6</v>
@@ -5161,13 +5170,13 @@
     </row>
     <row r="296" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A296" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B296" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C296" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D296" t="s">
         <v>6</v>
@@ -5175,10 +5184,10 @@
     </row>
     <row r="297" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A297" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B297" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C297" t="b">
         <v>0</v>
@@ -5189,10 +5198,10 @@
     </row>
     <row r="298" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A298" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B298" t="s">
-        <v>44</v>
+        <v>12</v>
       </c>
       <c r="C298" t="b">
         <v>0</v>
@@ -5203,13 +5212,13 @@
     </row>
     <row r="299" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A299" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B299" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C299" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D299" t="s">
         <v>6</v>
@@ -5217,24 +5226,24 @@
     </row>
     <row r="300" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A300" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B300" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C300" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D300" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="301" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A301" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B301" t="s">
-        <v>26</v>
+        <v>46</v>
       </c>
       <c r="C301" t="b">
         <v>0</v>
@@ -5245,27 +5254,27 @@
     </row>
     <row r="302" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A302" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B302" t="s">
-        <v>13</v>
+        <v>26</v>
       </c>
       <c r="C302" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D302" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="303" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A303" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B303" t="s">
-        <v>37</v>
+        <v>13</v>
       </c>
       <c r="C303" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D303" t="s">
         <v>6</v>
@@ -5273,13 +5282,13 @@
     </row>
     <row r="304" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A304" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B304" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C304" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D304" t="s">
         <v>6</v>
@@ -5287,10 +5296,10 @@
     </row>
     <row r="305" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A305" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B305" t="s">
-        <v>52</v>
+        <v>38</v>
       </c>
       <c r="C305" t="b">
         <v>1</v>
@@ -5301,38 +5310,38 @@
     </row>
     <row r="306" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A306" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B306" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C306" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D306" t="s">
-        <v>51</v>
+        <v>6</v>
       </c>
     </row>
     <row r="307" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A307" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B307" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C307" t="b">
         <v>0</v>
       </c>
       <c r="D307" t="s">
-        <v>6</v>
+        <v>51</v>
       </c>
     </row>
     <row r="308" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A308" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B308" t="s">
-        <v>74</v>
+        <v>54</v>
       </c>
       <c r="C308" t="b">
         <v>0</v>
@@ -5343,10 +5352,10 @@
     </row>
     <row r="309" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A309" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B309" t="s">
-        <v>59</v>
+        <v>74</v>
       </c>
       <c r="C309" t="b">
         <v>0</v>
@@ -5357,10 +5366,10 @@
     </row>
     <row r="310" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A310" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B310" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C310" t="b">
         <v>0</v>
@@ -5371,164 +5380,164 @@
     </row>
     <row r="311" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A311" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B311" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C311" t="b">
         <v>0</v>
       </c>
       <c r="D311" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="312" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A312" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B312" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C312" t="b">
         <v>0</v>
       </c>
       <c r="D312" t="s">
-        <v>63</v>
+        <v>9</v>
       </c>
     </row>
     <row r="313" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A313" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B313" t="s">
-        <v>92</v>
+        <v>62</v>
       </c>
       <c r="C313" t="b">
         <v>0</v>
       </c>
       <c r="D313" t="s">
-        <v>9</v>
+        <v>63</v>
       </c>
     </row>
     <row r="314" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A314" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B314" t="s">
-        <v>55</v>
+        <v>92</v>
       </c>
       <c r="C314" t="b">
         <v>0</v>
       </c>
       <c r="D314" t="s">
-        <v>56</v>
+        <v>9</v>
       </c>
     </row>
     <row r="315" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A315" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B315" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="C315" t="b">
         <v>0</v>
       </c>
       <c r="D315" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="316" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A316" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B316" t="s">
-        <v>128</v>
+        <v>57</v>
       </c>
       <c r="C316" t="b">
         <v>0</v>
       </c>
       <c r="D316" t="s">
-        <v>129</v>
+        <v>58</v>
       </c>
     </row>
     <row r="317" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A317" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B317" t="s">
-        <v>121</v>
+        <v>130</v>
       </c>
       <c r="C317" t="b">
         <v>0</v>
       </c>
       <c r="D317" t="s">
-        <v>9</v>
+        <v>131</v>
       </c>
     </row>
     <row r="318" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A318" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B318" t="s">
-        <v>94</v>
+        <v>123</v>
       </c>
       <c r="C318" t="b">
         <v>0</v>
       </c>
       <c r="D318" t="s">
-        <v>130</v>
+        <v>9</v>
       </c>
     </row>
     <row r="319" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A319" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B319" t="s">
-        <v>19</v>
+        <v>94</v>
       </c>
       <c r="C319" t="b">
         <v>0</v>
       </c>
       <c r="D319" t="s">
-        <v>20</v>
+        <v>132</v>
       </c>
     </row>
     <row r="320" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A320" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B320" t="s">
-        <v>83</v>
+        <v>19</v>
       </c>
       <c r="C320" t="b">
         <v>0</v>
       </c>
       <c r="D320" t="s">
-        <v>84</v>
+        <v>20</v>
       </c>
     </row>
     <row r="321" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A321" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B321" t="s">
-        <v>27</v>
+        <v>83</v>
       </c>
       <c r="C321" t="b">
         <v>0</v>
       </c>
       <c r="D321" t="s">
-        <v>9</v>
+        <v>84</v>
       </c>
     </row>
     <row r="322" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A322" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B322" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C322" t="b">
         <v>0</v>
@@ -5539,10 +5548,10 @@
     </row>
     <row r="323" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A323" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B323" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C323" t="b">
         <v>0</v>
@@ -5553,10 +5562,10 @@
     </row>
     <row r="324" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A324" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B324" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C324" t="b">
         <v>0</v>
@@ -5567,83 +5576,83 @@
     </row>
     <row r="325" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A325" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B325" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C325" t="b">
         <v>0</v>
       </c>
       <c r="D325" t="s">
-        <v>33</v>
+        <v>9</v>
       </c>
     </row>
     <row r="326" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A326" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B326" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C326" t="b">
         <v>0</v>
       </c>
       <c r="D326" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="327" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A327" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B327" t="s">
-        <v>16</v>
+        <v>34</v>
       </c>
       <c r="C327" t="b">
         <v>0</v>
       </c>
       <c r="D327" t="s">
-        <v>9</v>
+        <v>35</v>
       </c>
     </row>
     <row r="328" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A328" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B328" t="s">
-        <v>85</v>
+        <v>16</v>
       </c>
       <c r="C328" t="b">
         <v>0</v>
       </c>
       <c r="D328" t="s">
-        <v>51</v>
+        <v>9</v>
       </c>
     </row>
     <row r="329" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A329" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="B329" t="s">
-        <v>97</v>
+        <v>85</v>
       </c>
       <c r="C329" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D329" t="s">
-        <v>6</v>
+        <v>51</v>
       </c>
     </row>
     <row r="330" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A330" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B330" t="s">
-        <v>115</v>
+        <v>97</v>
       </c>
       <c r="C330" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D330" t="s">
         <v>6</v>
@@ -5651,13 +5660,13 @@
     </row>
     <row r="331" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A331" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B331" t="s">
-        <v>98</v>
+        <v>117</v>
       </c>
       <c r="C331" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D331" t="s">
         <v>6</v>
@@ -5665,10 +5674,10 @@
     </row>
     <row r="332" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A332" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B332" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C332" t="b">
         <v>1</v>
@@ -5679,38 +5688,38 @@
     </row>
     <row r="333" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A333" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B333" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C333" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D333" t="s">
-        <v>101</v>
+        <v>6</v>
       </c>
     </row>
     <row r="334" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A334" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B334" t="s">
-        <v>38</v>
+        <v>100</v>
       </c>
       <c r="C334" t="b">
         <v>0</v>
       </c>
       <c r="D334" t="s">
-        <v>6</v>
+        <v>101</v>
       </c>
     </row>
     <row r="335" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A335" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B335" t="s">
-        <v>116</v>
+        <v>38</v>
       </c>
       <c r="C335" t="b">
         <v>0</v>
@@ -5721,13 +5730,13 @@
     </row>
     <row r="336" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A336" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B336" t="s">
-        <v>5</v>
+        <v>118</v>
       </c>
       <c r="C336" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D336" t="s">
         <v>6</v>
@@ -5735,13 +5744,13 @@
     </row>
     <row r="337" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A337" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B337" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C337" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D337" t="s">
         <v>6</v>
@@ -5749,41 +5758,41 @@
     </row>
     <row r="338" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A338" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B338" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C338" t="b">
         <v>0</v>
       </c>
       <c r="D338" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="339" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A339" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B339" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C339" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D339" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="340" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A340" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B340" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C340" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D340" t="s">
         <v>6</v>
@@ -5791,10 +5800,10 @@
     </row>
     <row r="341" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A341" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B341" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C341" t="b">
         <v>0</v>
@@ -5805,13 +5814,13 @@
     </row>
     <row r="342" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A342" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B342" t="s">
-        <v>45</v>
+        <v>12</v>
       </c>
       <c r="C342" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D342" t="s">
         <v>6</v>
@@ -5819,41 +5828,41 @@
     </row>
     <row r="343" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A343" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B343" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C343" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D343" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="344" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A344" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B344" t="s">
-        <v>13</v>
+        <v>46</v>
       </c>
       <c r="C344" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D344" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="345" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A345" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B345" t="s">
-        <v>37</v>
+        <v>13</v>
       </c>
       <c r="C345" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D345" t="s">
         <v>6</v>
@@ -5861,13 +5870,13 @@
     </row>
     <row r="346" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A346" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B346" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C346" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D346" t="s">
         <v>6</v>
@@ -5875,10 +5884,10 @@
     </row>
     <row r="347" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A347" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B347" t="s">
-        <v>52</v>
+        <v>38</v>
       </c>
       <c r="C347" t="b">
         <v>1</v>
@@ -5889,13 +5898,13 @@
     </row>
     <row r="348" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A348" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B348" t="s">
-        <v>60</v>
+        <v>52</v>
       </c>
       <c r="C348" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D348" t="s">
         <v>6</v>
@@ -5903,49 +5912,49 @@
     </row>
     <row r="349" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A349" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B349" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C349" t="b">
         <v>0</v>
       </c>
       <c r="D349" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="350" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A350" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B350" t="s">
-        <v>133</v>
+        <v>61</v>
       </c>
       <c r="C350" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D350" t="s">
-        <v>51</v>
+        <v>9</v>
       </c>
     </row>
     <row r="351" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A351" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B351" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C351" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D351" t="s">
-        <v>135</v>
+        <v>51</v>
       </c>
     </row>
     <row r="352" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A352" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B352" t="s">
         <v>136</v>
@@ -5954,85 +5963,85 @@
         <v>0</v>
       </c>
       <c r="D352" t="s">
-        <v>9</v>
+        <v>137</v>
       </c>
     </row>
     <row r="353" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A353" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B353" t="s">
-        <v>19</v>
+        <v>138</v>
       </c>
       <c r="C353" t="b">
         <v>0</v>
       </c>
       <c r="D353" t="s">
-        <v>20</v>
+        <v>9</v>
       </c>
     </row>
     <row r="354" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A354" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B354" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="C354" t="b">
         <v>0</v>
       </c>
       <c r="D354" t="s">
-        <v>9</v>
+        <v>20</v>
       </c>
     </row>
     <row r="355" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A355" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B355" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C355" t="b">
         <v>0</v>
       </c>
       <c r="D355" t="s">
-        <v>33</v>
+        <v>9</v>
       </c>
     </row>
     <row r="356" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A356" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B356" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C356" t="b">
         <v>0</v>
       </c>
       <c r="D356" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="357" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A357" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="B357" t="s">
-        <v>10</v>
+        <v>34</v>
       </c>
       <c r="C357" t="b">
         <v>0</v>
       </c>
       <c r="D357" t="s">
-        <v>6</v>
+        <v>35</v>
       </c>
     </row>
     <row r="358" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A358" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B358" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C358" t="b">
         <v>0</v>
@@ -6043,27 +6052,27 @@
     </row>
     <row r="359" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A359" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B359" t="s">
-        <v>133</v>
+        <v>12</v>
       </c>
       <c r="C359" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D359" t="s">
-        <v>51</v>
+        <v>6</v>
       </c>
     </row>
     <row r="360" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A360" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B360" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="C360" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D360" t="s">
         <v>51</v>
@@ -6071,21 +6080,21 @@
     </row>
     <row r="361" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A361" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B361" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C361" t="b">
         <v>0</v>
       </c>
       <c r="D361" t="s">
-        <v>140</v>
+        <v>51</v>
       </c>
     </row>
     <row r="362" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A362" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B362" t="s">
         <v>141</v>
@@ -6099,7 +6108,7 @@
     </row>
     <row r="363" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A363" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B363" t="s">
         <v>143</v>
@@ -6113,7 +6122,7 @@
     </row>
     <row r="364" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A364" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B364" t="s">
         <v>145</v>
@@ -6127,41 +6136,41 @@
     </row>
     <row r="365" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A365" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B365" t="s">
-        <v>32</v>
+        <v>147</v>
       </c>
       <c r="C365" t="b">
         <v>0</v>
       </c>
       <c r="D365" t="s">
-        <v>33</v>
+        <v>148</v>
       </c>
     </row>
     <row r="366" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A366" t="s">
-        <v>147</v>
+        <v>139</v>
       </c>
       <c r="B366" t="s">
-        <v>5</v>
+        <v>32</v>
       </c>
       <c r="C366" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D366" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
     </row>
     <row r="367" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A367" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="B367" t="s">
-        <v>148</v>
+        <v>5</v>
       </c>
       <c r="C367" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D367" t="s">
         <v>6</v>
@@ -6169,55 +6178,55 @@
     </row>
     <row r="368" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A368" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="B368" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="C368" t="b">
         <v>0</v>
       </c>
       <c r="D368" t="s">
-        <v>150</v>
+        <v>6</v>
       </c>
     </row>
     <row r="369" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A369" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="B369" t="s">
-        <v>32</v>
+        <v>151</v>
       </c>
       <c r="C369" t="b">
         <v>0</v>
       </c>
       <c r="D369" t="s">
-        <v>33</v>
+        <v>152</v>
       </c>
     </row>
     <row r="370" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A370" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="B370" t="s">
-        <v>5</v>
+        <v>32</v>
       </c>
       <c r="C370" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D370" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
     </row>
     <row r="371" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A371" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="B371" t="s">
-        <v>148</v>
+        <v>5</v>
       </c>
       <c r="C371" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D371" t="s">
         <v>6</v>
@@ -6225,58 +6234,58 @@
     </row>
     <row r="372" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A372" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="B372" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="C372" t="b">
         <v>0</v>
       </c>
       <c r="D372" t="s">
-        <v>152</v>
+        <v>6</v>
       </c>
     </row>
     <row r="373" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A373" t="s">
+        <v>153</v>
+      </c>
+      <c r="B373" t="s">
         <v>151</v>
       </c>
-      <c r="B373" t="s">
-        <v>153</v>
-      </c>
       <c r="C373" t="b">
         <v>0</v>
       </c>
       <c r="D373" t="s">
-        <v>9</v>
+        <v>154</v>
       </c>
     </row>
     <row r="374" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A374" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="B374" t="s">
-        <v>32</v>
+        <v>155</v>
       </c>
       <c r="C374" t="b">
         <v>0</v>
       </c>
       <c r="D374" t="s">
-        <v>33</v>
+        <v>9</v>
       </c>
     </row>
     <row r="375" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A375" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B375" t="s">
-        <v>155</v>
+        <v>32</v>
       </c>
       <c r="C375" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D375" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
     </row>
     <row r="376" spans="1:4" x14ac:dyDescent="0.25">
@@ -6298,7 +6307,7 @@
         <v>158</v>
       </c>
       <c r="B377" t="s">
-        <v>5</v>
+        <v>159</v>
       </c>
       <c r="C377" t="b">
         <v>1</v>
@@ -6309,13 +6318,13 @@
     </row>
     <row r="378" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A378" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="B378" t="s">
-        <v>148</v>
+        <v>5</v>
       </c>
       <c r="C378" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D378" t="s">
         <v>6</v>
@@ -6323,30 +6332,30 @@
     </row>
     <row r="379" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A379" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="B379" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="C379" t="b">
         <v>0</v>
       </c>
       <c r="D379" t="s">
-        <v>159</v>
+        <v>6</v>
       </c>
     </row>
     <row r="380" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A380" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="B380" t="s">
-        <v>32</v>
+        <v>151</v>
       </c>
       <c r="C380" t="b">
         <v>0</v>
       </c>
       <c r="D380" t="s">
-        <v>33</v>
+        <v>161</v>
       </c>
     </row>
     <row r="381" spans="1:4" x14ac:dyDescent="0.25">
@@ -6354,24 +6363,24 @@
         <v>160</v>
       </c>
       <c r="B381" t="s">
-        <v>161</v>
+        <v>32</v>
       </c>
       <c r="C381" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D381" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
     </row>
     <row r="382" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A382" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="B382" t="s">
-        <v>54</v>
+        <v>163</v>
       </c>
       <c r="C382" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D382" t="s">
         <v>6</v>
@@ -6382,10 +6391,10 @@
         <v>162</v>
       </c>
       <c r="B383" t="s">
-        <v>163</v>
+        <v>54</v>
       </c>
       <c r="C383" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D383" t="s">
         <v>6</v>
@@ -6396,7 +6405,7 @@
         <v>164</v>
       </c>
       <c r="B384" t="s">
-        <v>5</v>
+        <v>165</v>
       </c>
       <c r="C384" t="b">
         <v>1</v>
@@ -6407,10 +6416,10 @@
     </row>
     <row r="385" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A385" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B385" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="C385" t="b">
         <v>1</v>
@@ -6421,24 +6430,24 @@
     </row>
     <row r="386" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A386" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B386" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
       <c r="C386" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D386" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="387" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A387" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B387" t="s">
-        <v>31</v>
+        <v>167</v>
       </c>
       <c r="C387" t="b">
         <v>0</v>
@@ -6449,30 +6458,30 @@
     </row>
     <row r="388" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A388" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B388" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C388" t="b">
         <v>0</v>
       </c>
       <c r="D388" t="s">
-        <v>33</v>
+        <v>9</v>
       </c>
     </row>
     <row r="389" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A389" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B389" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C389" t="b">
         <v>0</v>
       </c>
       <c r="D389" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="390" spans="1:4" x14ac:dyDescent="0.25">
@@ -6480,21 +6489,21 @@
         <v>166</v>
       </c>
       <c r="B390" t="s">
-        <v>13</v>
+        <v>34</v>
       </c>
       <c r="C390" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D390" t="s">
-        <v>6</v>
+        <v>35</v>
       </c>
     </row>
     <row r="391" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A391" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B391" t="s">
-        <v>52</v>
+        <v>13</v>
       </c>
       <c r="C391" t="b">
         <v>1</v>
@@ -6505,10 +6514,10 @@
     </row>
     <row r="392" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A392" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B392" t="s">
-        <v>167</v>
+        <v>52</v>
       </c>
       <c r="C392" t="b">
         <v>1</v>
@@ -6519,13 +6528,13 @@
     </row>
     <row r="393" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A393" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B393" t="s">
-        <v>12</v>
+        <v>169</v>
       </c>
       <c r="C393" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D393" t="s">
         <v>6</v>
@@ -6533,10 +6542,10 @@
     </row>
     <row r="394" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A394" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B394" t="s">
-        <v>99</v>
+        <v>12</v>
       </c>
       <c r="C394" t="b">
         <v>0</v>
@@ -6550,10 +6559,10 @@
         <v>168</v>
       </c>
       <c r="B395" t="s">
-        <v>10</v>
+        <v>99</v>
       </c>
       <c r="C395" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D395" t="s">
         <v>6</v>
@@ -6561,10 +6570,10 @@
     </row>
     <row r="396" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A396" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="B396" t="s">
-        <v>99</v>
+        <v>10</v>
       </c>
       <c r="C396" t="b">
         <v>1</v>
@@ -6575,13 +6584,13 @@
     </row>
     <row r="397" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A397" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="B397" t="s">
-        <v>12</v>
+        <v>99</v>
       </c>
       <c r="C397" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D397" t="s">
         <v>6</v>
@@ -6589,13 +6598,13 @@
     </row>
     <row r="398" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A398" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="B398" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C398" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D398" t="s">
         <v>6</v>
@@ -6603,10 +6612,10 @@
     </row>
     <row r="399" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A399" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="B399" t="s">
-        <v>99</v>
+        <v>10</v>
       </c>
       <c r="C399" t="b">
         <v>1</v>
@@ -6617,13 +6626,13 @@
     </row>
     <row r="400" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A400" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="B400" t="s">
-        <v>12</v>
+        <v>99</v>
       </c>
       <c r="C400" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D400" t="s">
         <v>6</v>
@@ -6631,13 +6640,13 @@
     </row>
     <row r="401" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A401" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="B401" t="s">
-        <v>98</v>
+        <v>12</v>
       </c>
       <c r="C401" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D401" t="s">
         <v>6</v>
@@ -6645,10 +6654,10 @@
     </row>
     <row r="402" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A402" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="B402" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C402" t="b">
         <v>1</v>
@@ -6659,13 +6668,13 @@
     </row>
     <row r="403" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A403" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="B403" t="s">
-        <v>115</v>
+        <v>97</v>
       </c>
       <c r="C403" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D403" t="s">
         <v>6</v>
@@ -6673,13 +6682,13 @@
     </row>
     <row r="404" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A404" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="B404" t="s">
-        <v>99</v>
+        <v>117</v>
       </c>
       <c r="C404" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D404" t="s">
         <v>6</v>
@@ -6687,10 +6696,10 @@
     </row>
     <row r="405" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A405" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B405" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="C405" t="b">
         <v>1</v>
@@ -6701,13 +6710,13 @@
     </row>
     <row r="406" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A406" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="B406" t="s">
-        <v>115</v>
+        <v>97</v>
       </c>
       <c r="C406" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D406" t="s">
         <v>6</v>
@@ -6715,13 +6724,13 @@
     </row>
     <row r="407" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A407" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="B407" t="s">
-        <v>99</v>
+        <v>117</v>
       </c>
       <c r="C407" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D407" t="s">
         <v>6</v>
@@ -6729,10 +6738,10 @@
     </row>
     <row r="408" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A408" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="B408" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="C408" t="b">
         <v>1</v>
@@ -6743,13 +6752,13 @@
     </row>
     <row r="409" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A409" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="B409" t="s">
-        <v>115</v>
+        <v>97</v>
       </c>
       <c r="C409" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D409" t="s">
         <v>6</v>
@@ -6757,13 +6766,13 @@
     </row>
     <row r="410" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A410" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="B410" t="s">
-        <v>99</v>
+        <v>117</v>
       </c>
       <c r="C410" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D410" t="s">
         <v>6</v>
@@ -6771,13 +6780,13 @@
     </row>
     <row r="411" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A411" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="B411" t="s">
-        <v>174</v>
+        <v>99</v>
       </c>
       <c r="C411" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D411" t="s">
         <v>6</v>
@@ -6785,10 +6794,10 @@
     </row>
     <row r="412" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A412" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="B412" t="s">
-        <v>7</v>
+        <v>176</v>
       </c>
       <c r="C412" t="b">
         <v>0</v>
@@ -6799,10 +6808,10 @@
     </row>
     <row r="413" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A413" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="B413" t="s">
-        <v>175</v>
+        <v>7</v>
       </c>
       <c r="C413" t="b">
         <v>0</v>
@@ -6813,150 +6822,150 @@
     </row>
     <row r="414" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A414" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="B414" t="s">
-        <v>8</v>
+        <v>177</v>
       </c>
       <c r="C414" t="b">
         <v>0</v>
       </c>
       <c r="D414" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="415" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A415" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="B415" t="s">
-        <v>32</v>
+        <v>8</v>
       </c>
       <c r="C415" t="b">
         <v>0</v>
       </c>
       <c r="D415" t="s">
-        <v>33</v>
+        <v>9</v>
       </c>
     </row>
     <row r="416" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A416" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="B416" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C416" t="b">
         <v>0</v>
       </c>
       <c r="D416" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="417" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A417" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="B417" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="C417" t="b">
         <v>0</v>
       </c>
       <c r="D417" t="s">
-        <v>9</v>
+        <v>35</v>
       </c>
     </row>
     <row r="418" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A418" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="B418" t="s">
-        <v>161</v>
+        <v>31</v>
       </c>
       <c r="C418" t="b">
         <v>0</v>
       </c>
       <c r="D418" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="419" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A419" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="B419" t="s">
-        <v>8</v>
+        <v>163</v>
       </c>
       <c r="C419" t="b">
         <v>0</v>
       </c>
       <c r="D419" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="420" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A420" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="B420" t="s">
-        <v>32</v>
+        <v>8</v>
       </c>
       <c r="C420" t="b">
         <v>0</v>
       </c>
       <c r="D420" t="s">
-        <v>33</v>
+        <v>9</v>
       </c>
     </row>
     <row r="421" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A421" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="B421" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C421" t="b">
         <v>0</v>
       </c>
       <c r="D421" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="422" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A422" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="B422" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="C422" t="b">
         <v>0</v>
       </c>
       <c r="D422" t="s">
-        <v>9</v>
+        <v>35</v>
       </c>
     </row>
     <row r="423" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A423" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="B423" t="s">
-        <v>13</v>
+        <v>31</v>
       </c>
       <c r="C423" t="b">
         <v>0</v>
       </c>
       <c r="D423" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="424" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A424" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="B424" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="C424" t="b">
         <v>0</v>
@@ -6967,83 +6976,83 @@
     </row>
     <row r="425" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A425" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="B425" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C425" t="b">
         <v>0</v>
       </c>
       <c r="D425" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="426" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A426" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="B426" t="s">
-        <v>32</v>
+        <v>8</v>
       </c>
       <c r="C426" t="b">
         <v>0</v>
       </c>
       <c r="D426" t="s">
-        <v>33</v>
+        <v>9</v>
       </c>
     </row>
     <row r="427" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A427" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="B427" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C427" t="b">
         <v>0</v>
       </c>
       <c r="D427" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="428" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A428" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="B428" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="C428" t="b">
         <v>0</v>
       </c>
       <c r="D428" t="s">
-        <v>9</v>
+        <v>35</v>
       </c>
     </row>
     <row r="429" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A429" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B429" t="s">
-        <v>97</v>
+        <v>31</v>
       </c>
       <c r="C429" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D429" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="430" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A430" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="B430" t="s">
-        <v>115</v>
+        <v>97</v>
       </c>
       <c r="C430" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D430" t="s">
         <v>6</v>
@@ -7051,10 +7060,10 @@
     </row>
     <row r="431" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A431" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="B431" t="s">
-        <v>179</v>
+        <v>117</v>
       </c>
       <c r="C431" t="b">
         <v>0</v>
@@ -7068,10 +7077,10 @@
         <v>180</v>
       </c>
       <c r="B432" t="s">
-        <v>97</v>
+        <v>181</v>
       </c>
       <c r="C432" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D432" t="s">
         <v>6</v>
@@ -7079,13 +7088,13 @@
     </row>
     <row r="433" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A433" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="B433" t="s">
-        <v>115</v>
+        <v>97</v>
       </c>
       <c r="C433" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D433" t="s">
         <v>6</v>
@@ -7093,10 +7102,10 @@
     </row>
     <row r="434" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A434" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="B434" t="s">
-        <v>179</v>
+        <v>117</v>
       </c>
       <c r="C434" t="b">
         <v>0</v>
@@ -7107,7 +7116,7 @@
     </row>
     <row r="435" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A435" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="B435" t="s">
         <v>181</v>
@@ -7127,7 +7136,7 @@
         <v>183</v>
       </c>
       <c r="C436" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D436" t="s">
         <v>6</v>
@@ -7135,10 +7144,10 @@
     </row>
     <row r="437" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A437" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="B437" t="s">
-        <v>10</v>
+        <v>185</v>
       </c>
       <c r="C437" t="b">
         <v>1</v>
@@ -7149,13 +7158,13 @@
     </row>
     <row r="438" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A438" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="B438" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C438" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D438" t="s">
         <v>6</v>
@@ -7163,38 +7172,38 @@
     </row>
     <row r="439" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A439" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="B439" t="s">
-        <v>32</v>
+        <v>12</v>
       </c>
       <c r="C439" t="b">
         <v>0</v>
       </c>
       <c r="D439" t="s">
-        <v>33</v>
+        <v>6</v>
       </c>
     </row>
     <row r="440" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A440" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="B440" t="s">
-        <v>8</v>
+        <v>32</v>
       </c>
       <c r="C440" t="b">
         <v>0</v>
       </c>
       <c r="D440" t="s">
-        <v>9</v>
+        <v>33</v>
       </c>
     </row>
     <row r="441" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A441" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="B441" t="s">
-        <v>184</v>
+        <v>8</v>
       </c>
       <c r="C441" t="b">
         <v>0</v>
@@ -7205,27 +7214,27 @@
     </row>
     <row r="442" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A442" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="B442" t="s">
-        <v>38</v>
+        <v>186</v>
       </c>
       <c r="C442" t="b">
         <v>0</v>
       </c>
       <c r="D442" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="443" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A443" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B443" t="s">
-        <v>186</v>
+        <v>38</v>
       </c>
       <c r="C443" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D443" t="s">
         <v>6</v>
@@ -7233,10 +7242,10 @@
     </row>
     <row r="444" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A444" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="B444" t="s">
-        <v>183</v>
+        <v>188</v>
       </c>
       <c r="C444" t="b">
         <v>1</v>
@@ -7247,10 +7256,10 @@
     </row>
     <row r="445" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A445" t="s">
+        <v>187</v>
+      </c>
+      <c r="B445" t="s">
         <v>185</v>
-      </c>
-      <c r="B445" t="s">
-        <v>10</v>
       </c>
       <c r="C445" t="b">
         <v>1</v>
@@ -7261,13 +7270,13 @@
     </row>
     <row r="446" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A446" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="B446" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C446" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D446" t="s">
         <v>6</v>
@@ -7275,38 +7284,38 @@
     </row>
     <row r="447" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A447" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="B447" t="s">
-        <v>32</v>
+        <v>12</v>
       </c>
       <c r="C447" t="b">
         <v>0</v>
       </c>
       <c r="D447" t="s">
-        <v>33</v>
+        <v>6</v>
       </c>
     </row>
     <row r="448" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A448" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="B448" t="s">
-        <v>8</v>
+        <v>32</v>
       </c>
       <c r="C448" t="b">
         <v>0</v>
       </c>
       <c r="D448" t="s">
-        <v>9</v>
+        <v>33</v>
       </c>
     </row>
     <row r="449" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A449" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="B449" t="s">
-        <v>46</v>
+        <v>8</v>
       </c>
       <c r="C449" t="b">
         <v>0</v>
@@ -7317,27 +7326,27 @@
     </row>
     <row r="450" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A450" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="B450" t="s">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="C450" t="b">
         <v>0</v>
       </c>
       <c r="D450" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="451" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A451" t="s">
-        <v>84</v>
+        <v>187</v>
       </c>
       <c r="B451" t="s">
-        <v>187</v>
+        <v>38</v>
       </c>
       <c r="C451" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D451" t="s">
         <v>6</v>
@@ -7348,10 +7357,10 @@
         <v>84</v>
       </c>
       <c r="B452" t="s">
-        <v>12</v>
+        <v>189</v>
       </c>
       <c r="C452" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D452" t="s">
         <v>6</v>
@@ -7359,27 +7368,27 @@
     </row>
     <row r="453" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A453" t="s">
-        <v>188</v>
+        <v>84</v>
       </c>
       <c r="B453" t="s">
-        <v>189</v>
+        <v>12</v>
       </c>
       <c r="C453" t="b">
         <v>0</v>
       </c>
       <c r="D453" t="s">
-        <v>190</v>
+        <v>6</v>
       </c>
     </row>
     <row r="454" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A454" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B454" t="s">
         <v>191</v>
       </c>
       <c r="C454" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D454" t="s">
         <v>192</v>
@@ -7387,24 +7396,24 @@
     </row>
     <row r="455" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A455" t="s">
+        <v>190</v>
+      </c>
+      <c r="B455" t="s">
         <v>193</v>
       </c>
-      <c r="B455" t="s">
-        <v>5</v>
-      </c>
       <c r="C455" t="b">
         <v>1</v>
       </c>
       <c r="D455" t="s">
-        <v>6</v>
+        <v>194</v>
       </c>
     </row>
     <row r="456" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A456" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="B456" t="s">
-        <v>194</v>
+        <v>5</v>
       </c>
       <c r="C456" t="b">
         <v>1</v>
@@ -7418,7 +7427,7 @@
         <v>195</v>
       </c>
       <c r="B457" t="s">
-        <v>5</v>
+        <v>196</v>
       </c>
       <c r="C457" t="b">
         <v>1</v>
@@ -7429,10 +7438,10 @@
     </row>
     <row r="458" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A458" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="B458" t="s">
-        <v>194</v>
+        <v>5</v>
       </c>
       <c r="C458" t="b">
         <v>1</v>
@@ -7443,10 +7452,10 @@
     </row>
     <row r="459" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A459" t="s">
+        <v>197</v>
+      </c>
+      <c r="B459" t="s">
         <v>196</v>
-      </c>
-      <c r="B459" t="s">
-        <v>97</v>
       </c>
       <c r="C459" t="b">
         <v>1</v>
@@ -7457,10 +7466,10 @@
     </row>
     <row r="460" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A460" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="B460" t="s">
-        <v>197</v>
+        <v>97</v>
       </c>
       <c r="C460" t="b">
         <v>1</v>
@@ -7474,7 +7483,7 @@
         <v>198</v>
       </c>
       <c r="B461" t="s">
-        <v>97</v>
+        <v>199</v>
       </c>
       <c r="C461" t="b">
         <v>1</v>
@@ -7485,10 +7494,10 @@
     </row>
     <row r="462" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A462" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="B462" t="s">
-        <v>199</v>
+        <v>97</v>
       </c>
       <c r="C462" t="b">
         <v>1</v>
@@ -7502,7 +7511,7 @@
         <v>200</v>
       </c>
       <c r="B463" t="s">
-        <v>5</v>
+        <v>201</v>
       </c>
       <c r="C463" t="b">
         <v>1</v>
@@ -7513,7 +7522,7 @@
     </row>
     <row r="464" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A464" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B464" t="s">
         <v>5</v>
@@ -7527,10 +7536,10 @@
     </row>
     <row r="465" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A465" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="B465" t="s">
-        <v>203</v>
+        <v>5</v>
       </c>
       <c r="C465" t="b">
         <v>1</v>
@@ -7544,7 +7553,7 @@
         <v>204</v>
       </c>
       <c r="B466" t="s">
-        <v>5</v>
+        <v>205</v>
       </c>
       <c r="C466" t="b">
         <v>1</v>
@@ -7555,13 +7564,13 @@
     </row>
     <row r="467" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A467" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="B467" t="s">
-        <v>205</v>
+        <v>5</v>
       </c>
       <c r="C467" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D467" t="s">
         <v>6</v>
@@ -7572,10 +7581,10 @@
         <v>206</v>
       </c>
       <c r="B468" t="s">
-        <v>5</v>
+        <v>207</v>
       </c>
       <c r="C468" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D468" t="s">
         <v>6</v>
@@ -7583,13 +7592,13 @@
     </row>
     <row r="469" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A469" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="B469" t="s">
-        <v>205</v>
+        <v>5</v>
       </c>
       <c r="C469" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D469" t="s">
         <v>6</v>
@@ -7597,13 +7606,13 @@
     </row>
     <row r="470" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A470" t="s">
+        <v>208</v>
+      </c>
+      <c r="B470" t="s">
         <v>207</v>
       </c>
-      <c r="B470" t="s">
-        <v>5</v>
-      </c>
       <c r="C470" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D470" t="s">
         <v>6</v>
@@ -7611,13 +7620,13 @@
     </row>
     <row r="471" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A471" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="B471" t="s">
-        <v>205</v>
+        <v>5</v>
       </c>
       <c r="C471" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D471" t="s">
         <v>6</v>
@@ -7625,13 +7634,13 @@
     </row>
     <row r="472" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A472" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="B472" t="s">
-        <v>5</v>
+        <v>207</v>
       </c>
       <c r="C472" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D472" t="s">
         <v>6</v>
@@ -7639,13 +7648,13 @@
     </row>
     <row r="473" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A473" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="B473" t="s">
-        <v>205</v>
+        <v>5</v>
       </c>
       <c r="C473" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D473" t="s">
         <v>6</v>
@@ -7653,13 +7662,13 @@
     </row>
     <row r="474" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A474" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="B474" t="s">
-        <v>5</v>
+        <v>207</v>
       </c>
       <c r="C474" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D474" t="s">
         <v>6</v>
@@ -7667,13 +7676,13 @@
     </row>
     <row r="475" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A475" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="B475" t="s">
         <v>5</v>
       </c>
       <c r="C475" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D475" t="s">
         <v>6</v>
@@ -7681,10 +7690,10 @@
     </row>
     <row r="476" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A476" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="B476" t="s">
-        <v>186</v>
+        <v>207</v>
       </c>
       <c r="C476" t="b">
         <v>0</v>
@@ -7695,13 +7704,13 @@
     </row>
     <row r="477" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A477" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="B477" t="s">
-        <v>183</v>
+        <v>5</v>
       </c>
       <c r="C477" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D477" t="s">
         <v>6</v>
@@ -7709,13 +7718,13 @@
     </row>
     <row r="478" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A478" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="B478" t="s">
-        <v>211</v>
+        <v>5</v>
       </c>
       <c r="C478" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D478" t="s">
         <v>6</v>
@@ -7723,10 +7732,10 @@
     </row>
     <row r="479" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A479" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="B479" t="s">
-        <v>12</v>
+        <v>188</v>
       </c>
       <c r="C479" t="b">
         <v>0</v>
@@ -7737,13 +7746,13 @@
     </row>
     <row r="480" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A480" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="B480" t="s">
-        <v>5</v>
+        <v>185</v>
       </c>
       <c r="C480" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D480" t="s">
         <v>6</v>
@@ -7751,13 +7760,13 @@
     </row>
     <row r="481" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A481" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="B481" t="s">
-        <v>7</v>
+        <v>214</v>
       </c>
       <c r="C481" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D481" t="s">
         <v>6</v>
@@ -7765,24 +7774,24 @@
     </row>
     <row r="482" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A482" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="B482" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="C482" t="b">
         <v>0</v>
       </c>
       <c r="D482" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="483" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A483" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="B483" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="C483" t="b">
         <v>1</v>
@@ -7793,10 +7802,10 @@
     </row>
     <row r="484" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A484" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="B484" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="C484" t="b">
         <v>0</v>
@@ -7807,24 +7816,24 @@
     </row>
     <row r="485" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A485" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="B485" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="C485" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D485" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="486" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A486" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="B486" t="s">
-        <v>45</v>
+        <v>10</v>
       </c>
       <c r="C486" t="b">
         <v>1</v>
@@ -7835,24 +7844,24 @@
     </row>
     <row r="487" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A487" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="B487" t="s">
-        <v>46</v>
+        <v>11</v>
       </c>
       <c r="C487" t="b">
         <v>0</v>
       </c>
       <c r="D487" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="488" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A488" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="B488" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C488" t="b">
         <v>1</v>
@@ -7863,13 +7872,13 @@
     </row>
     <row r="489" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A489" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="B489" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="C489" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D489" t="s">
         <v>6</v>
@@ -7877,24 +7886,24 @@
     </row>
     <row r="490" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A490" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="B490" t="s">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="C490" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D490" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="491" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A491" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="B491" t="s">
-        <v>52</v>
+        <v>13</v>
       </c>
       <c r="C491" t="b">
         <v>1</v>
@@ -7905,57 +7914,99 @@
     </row>
     <row r="492" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A492" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="B492" t="s">
-        <v>19</v>
+        <v>37</v>
       </c>
       <c r="C492" t="b">
         <v>0</v>
       </c>
       <c r="D492" t="s">
-        <v>20</v>
+        <v>6</v>
       </c>
     </row>
     <row r="493" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A493" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="B493" t="s">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="C493" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D493" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="494" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A494" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="B494" t="s">
-        <v>32</v>
+        <v>52</v>
       </c>
       <c r="C494" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D494" t="s">
-        <v>33</v>
+        <v>6</v>
       </c>
     </row>
     <row r="495" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A495" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="B495" t="s">
+        <v>19</v>
+      </c>
+      <c r="C495" t="b">
+        <v>0</v>
+      </c>
+      <c r="D495" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="496" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A496" t="s">
+        <v>215</v>
+      </c>
+      <c r="B496" t="s">
+        <v>31</v>
+      </c>
+      <c r="C496" t="b">
+        <v>0</v>
+      </c>
+      <c r="D496" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="497" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A497" t="s">
+        <v>215</v>
+      </c>
+      <c r="B497" t="s">
+        <v>32</v>
+      </c>
+      <c r="C497" t="b">
+        <v>0</v>
+      </c>
+      <c r="D497" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="498" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A498" t="s">
+        <v>215</v>
+      </c>
+      <c r="B498" t="s">
         <v>34</v>
       </c>
-      <c r="C495" t="b">
-        <v>0</v>
-      </c>
-      <c r="D495" t="s">
+      <c r="C498" t="b">
+        <v>0</v>
+      </c>
+      <c r="D498" t="s">
         <v>35</v>
       </c>
     </row>

</xml_diff>